<commit_message>
Added commitment summary and debt tracking
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pratham OS\Development\Finance-AI\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{423AB30A-553D-4AFF-BAD0-9FA9A7F81C6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A43078E-2AAE-4E2D-B628-8E97D8DF2C44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="6" xr2:uid="{D6DE1A26-0963-4585-A363-547897EAF3B2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{D6DE1A26-0963-4585-A363-547897EAF3B2}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Dashboard" sheetId="4" r:id="rId3"/>
     <sheet name="Monthly Review" sheetId="5" r:id="rId4"/>
     <sheet name="Skill Tracker" sheetId="9" r:id="rId5"/>
-    <sheet name="Finance Commitments" sheetId="10" r:id="rId6"/>
+    <sheet name="Financial Commitments" sheetId="10" r:id="rId6"/>
     <sheet name="Income" sheetId="11" r:id="rId7"/>
     <sheet name="Income engine" sheetId="6" r:id="rId8"/>
     <sheet name="Carrer Tracker" sheetId="7" r:id="rId9"/>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="223">
   <si>
     <t>August Financial Plan</t>
   </si>
@@ -194,12 +194,6 @@
     <t>Current Balance</t>
   </si>
   <si>
-    <t>train tickets</t>
-  </si>
-  <si>
-    <t>chicken</t>
-  </si>
-  <si>
     <t>INCOME</t>
   </si>
   <si>
@@ -735,6 +729,9 @@
   </si>
   <si>
     <t>Gift</t>
+  </si>
+  <si>
+    <t>Showerma with cousins</t>
   </si>
 </sst>
 </file>
@@ -952,9 +949,6 @@
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -963,15 +957,15 @@
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="13">
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -991,47 +985,6 @@
           <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="10" formatCode="&quot;₹&quot;\ #,##0;[Red]&quot;₹&quot;\ \-#,##0"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="20" formatCode="dd/mmm/yy"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <border outline="0">
@@ -1064,6 +1017,50 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="10" formatCode="&quot;₹&quot;\ #,##0;[Red]&quot;₹&quot;\ \-#,##0"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="20" formatCode="dd/mmm/yy"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1078,7 +1075,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{42D67FA3-A40A-4607-BCB9-468A9ECB0007}" name="Table1" displayName="Table1" ref="A1:J1048576" totalsRowShown="0" headerRowDxfId="12" tableBorderDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{42D67FA3-A40A-4607-BCB9-468A9ECB0007}" name="Table1" displayName="Table1" ref="A1:J1048576" totalsRowShown="0" headerRowDxfId="3" tableBorderDxfId="2">
   <autoFilter ref="A1:J1048576" xr:uid="{42D67FA3-A40A-4607-BCB9-468A9ECB0007}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{1D37F906-33D7-46E6-8270-56D5EEA80EC7}" name="Date"/>
@@ -1115,7 +1112,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{7C5D4057-F5F1-485E-AE6E-34A855BB81C8}" name="IncomeTable" displayName="IncomeTable" ref="A1:G4" totalsRowShown="0" headerRowDxfId="3" dataDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{7C5D4057-F5F1-485E-AE6E-34A855BB81C8}" name="IncomeTable" displayName="IncomeTable" ref="A1:G4" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
   <autoFilter ref="A1:G4" xr:uid="{7C5D4057-F5F1-485E-AE6E-34A855BB81C8}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{85417279-B333-4129-826F-4B13A464B0A1}" name="Date" dataDxfId="10"/>
@@ -1123,8 +1120,8 @@
     <tableColumn id="3" xr3:uid="{A9F1D760-964B-4BC4-876E-FE2B218C85B6}" name="Category" dataDxfId="8"/>
     <tableColumn id="4" xr3:uid="{31C0BCAE-AC93-4345-9B1C-546CE0735A6B}" name="Amount" dataDxfId="7"/>
     <tableColumn id="5" xr3:uid="{C6E99480-C881-404B-8F25-E2549BD2CCCD}" name="Status" dataDxfId="6"/>
-    <tableColumn id="7" xr3:uid="{29AC2CCC-8D50-4D4F-9049-D5CBB08CDAB6}" name="Recurring" dataDxfId="0"/>
-    <tableColumn id="6" xr3:uid="{4D5A0A55-4298-4332-9A93-683CDAE35676}" name="Notes" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{29AC2CCC-8D50-4D4F-9049-D5CBB08CDAB6}" name="Recurring" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{4D5A0A55-4298-4332-9A93-683CDAE35676}" name="Notes" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1470,12 +1467,12 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -1659,10 +1656,10 @@
     <mergeCell ref="A1:D1"/>
   </mergeCells>
   <conditionalFormatting sqref="B17:B20">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1678,69 +1675,69 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>155</v>
-      </c>
       <c r="E1" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
   </sheetData>
@@ -1761,25 +1758,25 @@
         <v>35</v>
       </c>
       <c r="E1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="K1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="M1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="O1" t="s">
+        <v>184</v>
+      </c>
+      <c r="Q1" t="s">
         <v>186</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.3">
@@ -1790,25 +1787,25 @@
         <v>36</v>
       </c>
       <c r="E2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="G2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="I2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="K2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="M2" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="O2" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="Q2" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.3">
@@ -1816,22 +1813,22 @@
         <v>7</v>
       </c>
       <c r="E3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="G3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="K3" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="M3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="O3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="Q3" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.3">
@@ -1839,22 +1836,22 @@
         <v>6</v>
       </c>
       <c r="E4" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G4" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="I4" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="K4" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="O4" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="Q4" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.3">
@@ -1862,16 +1859,16 @@
         <v>29</v>
       </c>
       <c r="I5" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="K5" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="O5" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="Q5" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.3">
@@ -1879,10 +1876,10 @@
         <v>30</v>
       </c>
       <c r="K6" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="Q6" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.3">
@@ -1890,13 +1887,13 @@
         <v>31</v>
       </c>
       <c r="C7" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="K7" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="Q7" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.3">
@@ -1904,10 +1901,10 @@
         <v>32</v>
       </c>
       <c r="C8" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="K8" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.3">
@@ -1915,53 +1912,53 @@
         <v>33</v>
       </c>
       <c r="C9" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="K9" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C10" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="K10" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C11" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C12" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C13" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C14" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.3">
@@ -1969,7 +1966,7 @@
         <v>34</v>
       </c>
       <c r="C15" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.3">
@@ -1979,17 +1976,17 @@
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
   </sheetData>
@@ -2017,13 +2014,13 @@
         <v>27</v>
       </c>
       <c r="B1" s="21" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C1" s="22" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D1" s="21" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E1" s="21" t="s">
         <v>24</v>
@@ -2038,68 +2035,60 @@
         <v>26</v>
       </c>
       <c r="I1" s="21" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="J1" s="21" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="12">
-        <v>46198</v>
+        <v>46201</v>
       </c>
       <c r="B2" s="13" t="str">
         <f>TEXT(Transactions!$A2,"mmmm")</f>
         <v>June</v>
       </c>
-      <c r="C2" s="14"/>
-      <c r="D2" s="13"/>
+      <c r="C2" s="14">
+        <v>2026</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>67</v>
+      </c>
       <c r="E2" s="13" t="s">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="F2" s="13" t="s">
-        <v>43</v>
+        <v>222</v>
       </c>
       <c r="G2" s="13">
-        <v>250</v>
+        <v>260</v>
       </c>
       <c r="H2" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="I2" s="13"/>
-      <c r="J2" s="13"/>
+        <v>36</v>
+      </c>
+      <c r="I2" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="J2" s="13" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="15">
-        <v>46198</v>
-      </c>
-      <c r="B3" s="16" t="str">
-        <f>TEXT(Transactions!$A3,"mmmm")</f>
-        <v>June</v>
-      </c>
+      <c r="A3" s="15"/>
+      <c r="B3" s="16"/>
       <c r="C3" s="17"/>
       <c r="D3" s="16"/>
-      <c r="E3" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="F3" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="G3" s="16">
-        <v>240</v>
-      </c>
-      <c r="H3" s="16" t="s">
-        <v>36</v>
-      </c>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="16"/>
+      <c r="H3" s="16"/>
       <c r="I3" s="16"/>
       <c r="J3" s="16"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="18"/>
-      <c r="B4" s="13" t="str">
-        <f>TEXT(Transactions!$A4,"mmmm")</f>
-        <v>January</v>
-      </c>
+      <c r="A4" s="12"/>
+      <c r="B4" s="13"/>
       <c r="C4" s="14"/>
       <c r="D4" s="13"/>
       <c r="E4" s="13"/>
@@ -3592,12 +3581,12 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B5" s="5">
         <v>22000</v>
@@ -3605,7 +3594,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B6" s="5">
         <v>0</v>
@@ -3613,7 +3602,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B7" s="6">
         <f>B5+B6</f>
@@ -3628,7 +3617,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B10" s="7"/>
     </row>
@@ -3641,7 +3630,7 @@
       </c>
       <c r="B12" s="6">
         <f>SUM(Transactions!$G$2:$G$100)</f>
-        <v>490</v>
+        <v>260</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
@@ -3659,7 +3648,7 @@
       </c>
       <c r="B14" s="6">
         <f>SUMIF(Transactions!$H$2:$H$100,"Want",Transactions!$G$2:$G$100)</f>
-        <v>240</v>
+        <v>260</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
@@ -3668,7 +3657,7 @@
       </c>
       <c r="B15" s="6">
         <f>SUMIF(Transactions!$E$2:$E$100,"Food",Transactions!$G$2:$G$100)</f>
-        <v>240</v>
+        <v>260</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
@@ -3677,7 +3666,7 @@
       </c>
       <c r="B16" s="6">
         <f>SUMIF(Transactions!$E$2:$E$100,"Travel",Transactions!$G$2:$G$100)</f>
-        <v>250</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
@@ -3688,7 +3677,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B19" s="7"/>
     </row>
@@ -3701,21 +3690,21 @@
       </c>
       <c r="B21" s="6">
         <f>B7-B12</f>
-        <v>21510</v>
+        <v>21740</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B22" s="1">
         <f>B21/B7%</f>
-        <v>97.772727272727266</v>
+        <v>98.818181818181813</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B23" s="1" t="str">
         <f>IF(B21&gt;=5000,"🟢 Excellent",IF(B21&gt;=0,"🟡 Stable","🔴 Risk"))</f>
@@ -3724,7 +3713,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B24" s="1" t="str">
         <f>IF(B21&gt;=0,"✅ On Track","⚠️ Overspending")</f>
@@ -3733,7 +3722,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B27" s="25">
         <f>SUM(FinancialCommitments[Remaining])</f>
@@ -3742,7 +3731,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B29" s="26">
         <f>1-(SUM(FinancialCommitments[Remaining])/SUM(FinancialCommitments[Amount]))</f>
@@ -3751,11 +3740,11 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B31" s="7">
         <f>B21-B27</f>
-        <v>10510</v>
+        <v>10740</v>
       </c>
     </row>
   </sheetData>
@@ -3770,7 +3759,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B1" s="8">
         <v>46174</v>
@@ -3778,7 +3767,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -3793,47 +3782,47 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -3848,64 +3837,64 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>164</v>
+      </c>
+      <c r="B1" t="s">
+        <v>165</v>
+      </c>
+      <c r="C1" t="s">
         <v>166</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>167</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>168</v>
-      </c>
-      <c r="D1" t="s">
-        <v>169</v>
-      </c>
-      <c r="E1" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
   </sheetData>
@@ -3925,31 +3914,31 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B1" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D1" t="s">
         <v>2</v>
       </c>
       <c r="E1" t="s">
+        <v>194</v>
+      </c>
+      <c r="F1" t="s">
+        <v>195</v>
+      </c>
+      <c r="G1" t="s">
         <v>196</v>
       </c>
-      <c r="F1" t="s">
-        <v>197</v>
-      </c>
-      <c r="G1" t="s">
-        <v>198</v>
-      </c>
       <c r="H1" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="I1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
@@ -3957,10 +3946,10 @@
         <v>46204</v>
       </c>
       <c r="B2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C2" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="D2" s="25">
         <v>10000</v>
@@ -3972,13 +3961,13 @@
         <v>10000</v>
       </c>
       <c r="G2" t="s">
+        <v>199</v>
+      </c>
+      <c r="H2" t="s">
+        <v>200</v>
+      </c>
+      <c r="I2" t="s">
         <v>201</v>
-      </c>
-      <c r="H2" t="s">
-        <v>202</v>
-      </c>
-      <c r="I2" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
@@ -3986,10 +3975,10 @@
         <v>46206</v>
       </c>
       <c r="B3" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C3" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="D3" s="25">
         <v>2000</v>
@@ -4004,10 +3993,10 @@
         <v>46249</v>
       </c>
       <c r="H3" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="I3" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
   </sheetData>
@@ -4037,7 +4026,7 @@
         <v>27</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>24</v>
@@ -4046,82 +4035,82 @@
         <v>2</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="30">
+      <c r="A2" s="29">
         <v>46204</v>
       </c>
-      <c r="B2" s="28" t="s">
-        <v>129</v>
-      </c>
-      <c r="C2" s="28" t="s">
+      <c r="B2" s="27" t="s">
+        <v>127</v>
+      </c>
+      <c r="C2" s="27" t="s">
+        <v>209</v>
+      </c>
+      <c r="D2" s="28">
+        <v>22000</v>
+      </c>
+      <c r="E2" s="27" t="s">
+        <v>210</v>
+      </c>
+      <c r="F2" s="27" t="s">
+        <v>75</v>
+      </c>
+      <c r="G2" s="27" t="s">
         <v>211</v>
       </c>
-      <c r="D2" s="29">
-        <v>22000</v>
-      </c>
-      <c r="E2" s="28" t="s">
+    </row>
+    <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="29">
+        <v>46218</v>
+      </c>
+      <c r="B3" s="27" t="s">
+        <v>96</v>
+      </c>
+      <c r="C3" s="27" t="s">
         <v>212</v>
       </c>
-      <c r="F2" s="28" t="s">
-        <v>77</v>
-      </c>
-      <c r="G2" s="28" t="s">
+      <c r="D3" s="28">
+        <v>5000</v>
+      </c>
+      <c r="E3" s="27" t="s">
+        <v>141</v>
+      </c>
+      <c r="F3" s="27" t="s">
+        <v>76</v>
+      </c>
+      <c r="G3" s="27" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="30">
-        <v>46218</v>
-      </c>
-      <c r="B3" s="28" t="s">
-        <v>98</v>
-      </c>
-      <c r="C3" s="28" t="s">
+    <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="29">
+        <v>46223</v>
+      </c>
+      <c r="B4" s="27" t="s">
         <v>214</v>
       </c>
-      <c r="D3" s="29">
-        <v>5000</v>
-      </c>
-      <c r="E3" s="28" t="s">
-        <v>143</v>
-      </c>
-      <c r="F3" s="28" t="s">
-        <v>78</v>
-      </c>
-      <c r="G3" s="28" t="s">
+      <c r="C4" s="27" t="s">
         <v>215</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="30">
-        <v>46223</v>
-      </c>
-      <c r="B4" s="28" t="s">
-        <v>216</v>
-      </c>
-      <c r="C4" s="28" t="s">
-        <v>217</v>
-      </c>
-      <c r="D4" s="29">
+      <c r="D4" s="28">
         <v>2000</v>
       </c>
-      <c r="E4" s="28" t="s">
-        <v>212</v>
-      </c>
-      <c r="F4" s="28" t="s">
-        <v>78</v>
-      </c>
-      <c r="G4" s="28" t="s">
-        <v>204</v>
+      <c r="E4" s="27" t="s">
+        <v>210</v>
+      </c>
+      <c r="F4" s="27" t="s">
+        <v>76</v>
+      </c>
+      <c r="G4" s="27" t="s">
+        <v>202</v>
       </c>
     </row>
   </sheetData>
@@ -4150,21 +4139,21 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
@@ -4173,40 +4162,40 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B5" s="1">
         <v>24</v>
       </c>
       <c r="J5" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="J7" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
@@ -4217,12 +4206,12 @@
         <v>8600</v>
       </c>
       <c r="J9" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B10" s="23">
         <v>0</v>
@@ -4230,35 +4219,35 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="J11" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="J13" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="D15" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="E15" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="D15" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>97</v>
-      </c>
       <c r="J15" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
@@ -4266,16 +4255,16 @@
         <v>13</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D16" s="1">
         <v>22000</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
@@ -4283,19 +4272,19 @@
         <v>14</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D17" s="1">
         <v>23000</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="J17" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
@@ -4303,93 +4292,93 @@
         <v>15</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D18" s="1">
         <v>28000</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C19" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="D19" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="D19" s="1" t="s">
-        <v>108</v>
-      </c>
       <c r="E19" s="1" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="J19" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="J21" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="J23" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="J25" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="J27" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="J29" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="J31" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="33" spans="10:10" x14ac:dyDescent="0.3">
       <c r="J33" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="35" spans="10:10" x14ac:dyDescent="0.3">
       <c r="J35" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -4410,37 +4399,37 @@
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C1" t="s">
         <v>127</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>128</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>129</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>130</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
+        <v>178</v>
+      </c>
+      <c r="H1" t="s">
         <v>131</v>
       </c>
-      <c r="F1" t="s">
-        <v>132</v>
-      </c>
-      <c r="G1" t="s">
-        <v>180</v>
-      </c>
-      <c r="H1" t="s">
-        <v>133</v>
-      </c>
       <c r="I1" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="J1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="Q1" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.3">
@@ -4448,16 +4437,16 @@
         <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C2">
         <v>22000</v>
       </c>
       <c r="F2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="Q2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.3">
@@ -4465,16 +4454,16 @@
         <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C3">
         <v>23000</v>
       </c>
       <c r="F3" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="Q3" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.3">
@@ -4482,33 +4471,33 @@
         <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C4">
         <v>28000</v>
       </c>
       <c r="F4" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="Q4" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B5" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C5">
         <v>20000</v>
       </c>
       <c r="F5" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="Q5" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implement net position engine
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pratham OS\Development\Finance-AI\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A43078E-2AAE-4E2D-B628-8E97D8DF2C44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57220A0F-D1A6-469D-A718-42CE8834C301}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{D6DE1A26-0963-4585-A363-547897EAF3B2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="5" xr2:uid="{D6DE1A26-0963-4585-A363-547897EAF3B2}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan" sheetId="1" r:id="rId1"/>
@@ -30,6 +30,7 @@
     <definedName name="Categoreis">Lists!#REF!</definedName>
     <definedName name="Categories">Lists!$A$1:$A$15</definedName>
     <definedName name="Choice">Lists!$I$1:$I$2</definedName>
+    <definedName name="CommitmentStatus">Lists!$I$7:$I$8</definedName>
     <definedName name="IncomeCategory">Lists!$C$7:$C$16</definedName>
     <definedName name="IncomeStatus">Lists!$I$4:$I$5</definedName>
     <definedName name="InterviewResult">Lists!$M$1:$M$3</definedName>
@@ -63,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="225">
   <si>
     <t>August Financial Plan</t>
   </si>
@@ -732,15 +733,22 @@
   </si>
   <si>
     <t>Showerma with cousins</t>
+  </si>
+  <si>
+    <t>Paid</t>
+  </si>
+  <si>
+    <t>Raj</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="6" formatCode="&quot;₹&quot;\ #,##0;[Red]&quot;₹&quot;\ \-#,##0"/>
     <numFmt numFmtId="44" formatCode="_ &quot;₹&quot;\ * #,##0.00_ ;_ &quot;₹&quot;\ * \-#,##0.00_ ;_ &quot;₹&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -920,7 +928,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -960,12 +968,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="13">
+  <dxfs count="16">
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -983,37 +1001,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="2" tint="-9.9978637043366805E-2"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1061,6 +1048,37 @@
         <scheme val="minor"/>
       </font>
     </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="2" tint="-9.9978637043366805E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1075,7 +1093,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{42D67FA3-A40A-4607-BCB9-468A9ECB0007}" name="Table1" displayName="Table1" ref="A1:J1048576" totalsRowShown="0" headerRowDxfId="3" tableBorderDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{42D67FA3-A40A-4607-BCB9-468A9ECB0007}" name="Table1" displayName="Table1" ref="A1:J1048576" totalsRowShown="0" headerRowDxfId="15" tableBorderDxfId="14">
   <autoFilter ref="A1:J1048576" xr:uid="{42D67FA3-A40A-4607-BCB9-468A9ECB0007}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{1D37F906-33D7-46E6-8270-56D5EEA80EC7}" name="Date"/>
@@ -1100,9 +1118,9 @@
     <tableColumn id="1" xr3:uid="{C10697DD-F282-4D7F-A12A-9BFC6193DC4E}" name="Date "/>
     <tableColumn id="2" xr3:uid="{D6130D6E-B2EE-4D09-94CD-7E8053CD1C7B}" name="From"/>
     <tableColumn id="3" xr3:uid="{8ECD20EB-BEF0-47D5-8DA5-28D491EC7B0A}" name="Type"/>
-    <tableColumn id="4" xr3:uid="{87D047F3-8B64-4D30-ACC0-42FFF26FEC3E}" name="Amount"/>
-    <tableColumn id="5" xr3:uid="{C982624C-E448-4958-A5CE-7D794FC142FA}" name="Repaid"/>
-    <tableColumn id="6" xr3:uid="{665D5056-3744-4E56-95C7-F0943FD35707}" name="Remaining"/>
+    <tableColumn id="4" xr3:uid="{87D047F3-8B64-4D30-ACC0-42FFF26FEC3E}" name="Amount" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{C982624C-E448-4958-A5CE-7D794FC142FA}" name="Repaid" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{665D5056-3744-4E56-95C7-F0943FD35707}" name="Remaining" dataDxfId="0"/>
     <tableColumn id="7" xr3:uid="{FFDA91C5-2668-4023-9FEE-465A59D85270}" name="Due Date"/>
     <tableColumn id="8" xr3:uid="{748EB09B-78B0-49AB-AC7E-88A7F4C42C89}" name="Status"/>
     <tableColumn id="9" xr3:uid="{9F5FA8E8-540D-4C48-B339-C097673FD287}" name="Notes"/>
@@ -1112,16 +1130,16 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{7C5D4057-F5F1-485E-AE6E-34A855BB81C8}" name="IncomeTable" displayName="IncomeTable" ref="A1:G4" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{7C5D4057-F5F1-485E-AE6E-34A855BB81C8}" name="IncomeTable" displayName="IncomeTable" ref="A1:G4" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
   <autoFilter ref="A1:G4" xr:uid="{7C5D4057-F5F1-485E-AE6E-34A855BB81C8}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{85417279-B333-4129-826F-4B13A464B0A1}" name="Date" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{72151722-7F6E-43AF-AADF-05A0452D151E}" name="Source" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{A9F1D760-964B-4BC4-876E-FE2B218C85B6}" name="Category" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{31C0BCAE-AC93-4345-9B1C-546CE0735A6B}" name="Amount" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{C6E99480-C881-404B-8F25-E2549BD2CCCD}" name="Status" dataDxfId="6"/>
-    <tableColumn id="7" xr3:uid="{29AC2CCC-8D50-4D4F-9049-D5CBB08CDAB6}" name="Recurring" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{4D5A0A55-4298-4332-9A93-683CDAE35676}" name="Notes" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{85417279-B333-4129-826F-4B13A464B0A1}" name="Date" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{72151722-7F6E-43AF-AADF-05A0452D151E}" name="Source" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{A9F1D760-964B-4BC4-876E-FE2B218C85B6}" name="Category" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{31C0BCAE-AC93-4345-9B1C-546CE0735A6B}" name="Amount" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{C6E99480-C881-404B-8F25-E2549BD2CCCD}" name="Status" dataDxfId="7"/>
+    <tableColumn id="7" xr3:uid="{29AC2CCC-8D50-4D4F-9049-D5CBB08CDAB6}" name="Recurring" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{4D5A0A55-4298-4332-9A93-683CDAE35676}" name="Notes" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1656,10 +1674,10 @@
     <mergeCell ref="A1:D1"/>
   </mergeCells>
   <conditionalFormatting sqref="B17:B20">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="4" priority="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="3" priority="2" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1889,6 +1907,9 @@
       <c r="C7" t="s">
         <v>209</v>
       </c>
+      <c r="I7" t="s">
+        <v>200</v>
+      </c>
       <c r="K7" t="s">
         <v>138</v>
       </c>
@@ -1902,6 +1923,9 @@
       </c>
       <c r="C8" t="s">
         <v>96</v>
+      </c>
+      <c r="I8" t="s">
+        <v>223</v>
       </c>
       <c r="K8" t="s">
         <v>137</v>
@@ -3735,7 +3759,7 @@
       </c>
       <c r="B29" s="26">
         <f>1-(SUM(FinancialCommitments[Remaining])/SUM(FinancialCommitments[Amount]))</f>
-        <v>8.333333333333337E-2</v>
+        <v>0.15384615384615385</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
@@ -3904,11 +3928,12 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED4B5016-8080-45D9-A027-E465FB36B2D6}">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="4" width="9.33203125" customWidth="1"/>
-    <col min="6" max="6" width="11.6640625" customWidth="1"/>
+    <col min="4" max="4" width="13" style="31" customWidth="1"/>
+    <col min="5" max="5" width="9.44140625" style="31" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.6640625" style="31" customWidth="1"/>
     <col min="7" max="7" width="10.33203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3922,13 +3947,13 @@
       <c r="C1" t="s">
         <v>66</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="31" t="s">
         <v>194</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="31" t="s">
         <v>195</v>
       </c>
       <c r="G1" t="s">
@@ -3951,13 +3976,13 @@
       <c r="C2" t="s">
         <v>198</v>
       </c>
-      <c r="D2" s="25">
+      <c r="D2" s="31">
         <v>10000</v>
       </c>
-      <c r="E2" s="25">
+      <c r="E2" s="31">
         <v>0</v>
       </c>
-      <c r="F2" s="25">
+      <c r="F2" s="31">
         <v>10000</v>
       </c>
       <c r="G2" t="s">
@@ -3980,13 +4005,13 @@
       <c r="C3" t="s">
         <v>203</v>
       </c>
-      <c r="D3" s="25">
+      <c r="D3" s="31">
         <v>2000</v>
       </c>
-      <c r="E3" s="25">
+      <c r="E3" s="31">
         <v>1000</v>
       </c>
-      <c r="F3" s="25">
+      <c r="F3" s="31">
         <v>1000</v>
       </c>
       <c r="G3" s="24">
@@ -3999,10 +4024,42 @@
         <v>204</v>
       </c>
     </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" s="24">
+        <v>46208</v>
+      </c>
+      <c r="B4" t="s">
+        <v>224</v>
+      </c>
+      <c r="C4" t="s">
+        <v>203</v>
+      </c>
+      <c r="D4" s="31">
+        <v>1000</v>
+      </c>
+      <c r="E4" s="31">
+        <v>1000</v>
+      </c>
+      <c r="F4" s="31">
+        <v>0</v>
+      </c>
+      <c r="G4" s="24">
+        <v>46209</v>
+      </c>
+      <c r="H4" t="s">
+        <v>223</v>
+      </c>
+      <c r="I4" t="s">
+        <v>201</v>
+      </c>
+    </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1:C1048576" xr:uid="{C13FD2A8-23CC-45C1-BECC-766CFBB6D4A6}">
       <formula1>LoanType</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H1:H1048576" xr:uid="{4DC35CFB-9EF8-4609-96E8-FC7DC36AECDA}">
+      <formula1>CommitmentStatus</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add expense category analytics
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pratham OS\Development\Finance-AI\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57220A0F-D1A6-469D-A718-42CE8834C301}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0983308-D2AC-4F9A-A500-FE05507656B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="5" xr2:uid="{D6DE1A26-0963-4585-A363-547897EAF3B2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{D6DE1A26-0963-4585-A363-547897EAF3B2}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan" sheetId="1" r:id="rId1"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="229">
   <si>
     <t>August Financial Plan</t>
   </si>
@@ -739,6 +739,18 @@
   </si>
   <si>
     <t>Raj</t>
+  </si>
+  <si>
+    <t>June</t>
+  </si>
+  <si>
+    <t>rapido</t>
+  </si>
+  <si>
+    <t>june</t>
+  </si>
+  <si>
+    <t>breakfast</t>
   </si>
 </sst>
 </file>
@@ -928,7 +940,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -965,22 +977,20 @@
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="16">
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
-    </dxf>
+  <dxfs count="17">
     <dxf>
       <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
     </dxf>
@@ -1079,6 +1089,15 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1093,7 +1112,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{42D67FA3-A40A-4607-BCB9-468A9ECB0007}" name="Table1" displayName="Table1" ref="A1:J1048576" totalsRowShown="0" headerRowDxfId="15" tableBorderDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{42D67FA3-A40A-4607-BCB9-468A9ECB0007}" name="Table1" displayName="Table1" ref="A1:J1048576" totalsRowShown="0" headerRowDxfId="13" tableBorderDxfId="12">
   <autoFilter ref="A1:J1048576" xr:uid="{42D67FA3-A40A-4607-BCB9-468A9ECB0007}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{1D37F906-33D7-46E6-8270-56D5EEA80EC7}" name="Date"/>
@@ -1102,7 +1121,7 @@
     <tableColumn id="4" xr3:uid="{E805A8A8-660D-4099-912A-BE1B697553ED}" name="Type"/>
     <tableColumn id="5" xr3:uid="{ABF1E4D7-7922-479D-94F4-994DCBA1062D}" name="Category"/>
     <tableColumn id="6" xr3:uid="{E21EA904-BC60-4EB5-B4BD-249E5A12FC76}" name="Description "/>
-    <tableColumn id="7" xr3:uid="{EFA172CE-B81A-4A83-BB09-0C52BED62422}" name="Amount"/>
+    <tableColumn id="7" xr3:uid="{EFA172CE-B81A-4A83-BB09-0C52BED62422}" name="Amount" dataDxfId="0"/>
     <tableColumn id="8" xr3:uid="{E811D3EB-DAD5-46D9-B70D-01072B332F5C}" name="Need/Want"/>
     <tableColumn id="9" xr3:uid="{1E8766C9-2C6F-4CE3-9C7E-C6C8545D3945}" name="Payment Mode"/>
     <tableColumn id="10" xr3:uid="{BA26CD78-BAFB-4644-808D-0A18546F6CAF}" name="Recurring"/>
@@ -1118,9 +1137,9 @@
     <tableColumn id="1" xr3:uid="{C10697DD-F282-4D7F-A12A-9BFC6193DC4E}" name="Date "/>
     <tableColumn id="2" xr3:uid="{D6130D6E-B2EE-4D09-94CD-7E8053CD1C7B}" name="From"/>
     <tableColumn id="3" xr3:uid="{8ECD20EB-BEF0-47D5-8DA5-28D491EC7B0A}" name="Type"/>
-    <tableColumn id="4" xr3:uid="{87D047F3-8B64-4D30-ACC0-42FFF26FEC3E}" name="Amount" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{C982624C-E448-4958-A5CE-7D794FC142FA}" name="Repaid" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{665D5056-3744-4E56-95C7-F0943FD35707}" name="Remaining" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{87D047F3-8B64-4D30-ACC0-42FFF26FEC3E}" name="Amount" dataDxfId="16"/>
+    <tableColumn id="5" xr3:uid="{C982624C-E448-4958-A5CE-7D794FC142FA}" name="Repaid" dataDxfId="15"/>
+    <tableColumn id="6" xr3:uid="{665D5056-3744-4E56-95C7-F0943FD35707}" name="Remaining" dataDxfId="14"/>
     <tableColumn id="7" xr3:uid="{FFDA91C5-2668-4023-9FEE-465A59D85270}" name="Due Date"/>
     <tableColumn id="8" xr3:uid="{748EB09B-78B0-49AB-AC7E-88A7F4C42C89}" name="Status"/>
     <tableColumn id="9" xr3:uid="{9F5FA8E8-540D-4C48-B339-C097673FD287}" name="Notes"/>
@@ -1130,16 +1149,16 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{7C5D4057-F5F1-485E-AE6E-34A855BB81C8}" name="IncomeTable" displayName="IncomeTable" ref="A1:G4" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{7C5D4057-F5F1-485E-AE6E-34A855BB81C8}" name="IncomeTable" displayName="IncomeTable" ref="A1:G4" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
   <autoFilter ref="A1:G4" xr:uid="{7C5D4057-F5F1-485E-AE6E-34A855BB81C8}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{85417279-B333-4129-826F-4B13A464B0A1}" name="Date" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{72151722-7F6E-43AF-AADF-05A0452D151E}" name="Source" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{A9F1D760-964B-4BC4-876E-FE2B218C85B6}" name="Category" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{31C0BCAE-AC93-4345-9B1C-546CE0735A6B}" name="Amount" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{C6E99480-C881-404B-8F25-E2549BD2CCCD}" name="Status" dataDxfId="7"/>
-    <tableColumn id="7" xr3:uid="{29AC2CCC-8D50-4D4F-9049-D5CBB08CDAB6}" name="Recurring" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{4D5A0A55-4298-4332-9A93-683CDAE35676}" name="Notes" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{85417279-B333-4129-826F-4B13A464B0A1}" name="Date" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{72151722-7F6E-43AF-AADF-05A0452D151E}" name="Source" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{A9F1D760-964B-4BC4-876E-FE2B218C85B6}" name="Category" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{31C0BCAE-AC93-4345-9B1C-546CE0735A6B}" name="Amount" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{C6E99480-C881-404B-8F25-E2549BD2CCCD}" name="Status" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{29AC2CCC-8D50-4D4F-9049-D5CBB08CDAB6}" name="Recurring" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{4D5A0A55-4298-4332-9A93-683CDAE35676}" name="Notes" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1485,12 +1504,12 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -1674,10 +1693,10 @@
     <mergeCell ref="A1:D1"/>
   </mergeCells>
   <conditionalFormatting sqref="B17:B20">
-    <cfRule type="cellIs" dxfId="4" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2027,7 +2046,7 @@
     <col min="4" max="4" width="9.5546875" customWidth="1"/>
     <col min="5" max="5" width="10.21875" customWidth="1"/>
     <col min="6" max="6" width="12.88671875" customWidth="1"/>
-    <col min="7" max="7" width="9.33203125" customWidth="1"/>
+    <col min="7" max="7" width="9.33203125" style="30" customWidth="1"/>
     <col min="8" max="8" width="12.33203125" customWidth="1"/>
     <col min="9" max="9" width="15.109375" customWidth="1"/>
     <col min="10" max="10" width="10.77734375" customWidth="1"/>
@@ -2052,7 +2071,7 @@
       <c r="F1" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="G1" s="21" t="s">
+      <c r="G1" s="32" t="s">
         <v>2</v>
       </c>
       <c r="H1" s="21" t="s">
@@ -2085,7 +2104,7 @@
       <c r="F2" s="13" t="s">
         <v>222</v>
       </c>
-      <c r="G2" s="13">
+      <c r="G2" s="33">
         <v>260</v>
       </c>
       <c r="H2" s="13" t="s">
@@ -2099,43 +2118,101 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="15"/>
-      <c r="B3" s="16"/>
-      <c r="C3" s="17"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
-      <c r="I3" s="16"/>
-      <c r="J3" s="16"/>
+      <c r="A3" s="15">
+        <v>46204</v>
+      </c>
+      <c r="B3" s="16" t="s">
+        <v>225</v>
+      </c>
+      <c r="C3" s="17">
+        <v>2026</v>
+      </c>
+      <c r="D3" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="E3" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="16" t="s">
+        <v>226</v>
+      </c>
+      <c r="G3" s="34">
+        <v>40</v>
+      </c>
+      <c r="H3" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="I3" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="J3" s="16" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="12"/>
-      <c r="B4" s="13"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="13"/>
-      <c r="H4" s="13"/>
-      <c r="I4" s="13"/>
-      <c r="J4" s="13"/>
+      <c r="A4" s="12">
+        <v>46205</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>227</v>
+      </c>
+      <c r="C4" s="14">
+        <v>2026</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="13" t="s">
+        <v>226</v>
+      </c>
+      <c r="G4" s="33">
+        <v>200</v>
+      </c>
+      <c r="H4" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="I4" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="J4" s="13" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="19"/>
+      <c r="A5" s="15">
+        <v>46205</v>
+      </c>
       <c r="B5" s="16" t="str">
         <f>TEXT(Transactions!$A5,"mmmm")</f>
-        <v>January</v>
-      </c>
-      <c r="C5" s="17"/>
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="16"/>
-      <c r="G5" s="16"/>
-      <c r="H5" s="16"/>
-      <c r="I5" s="16"/>
-      <c r="J5" s="16"/>
+        <v>July</v>
+      </c>
+      <c r="C5" s="17">
+        <v>2026</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="E5" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="F5" s="16" t="s">
+        <v>228</v>
+      </c>
+      <c r="G5" s="34">
+        <v>60</v>
+      </c>
+      <c r="H5" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="I5" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="J5" s="16" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="18"/>
@@ -2147,7 +2224,7 @@
       <c r="D6" s="13"/>
       <c r="E6" s="13"/>
       <c r="F6" s="13"/>
-      <c r="G6" s="13"/>
+      <c r="G6" s="33"/>
       <c r="H6" s="13"/>
       <c r="I6" s="13"/>
       <c r="J6" s="13"/>
@@ -2162,7 +2239,7 @@
       <c r="D7" s="16"/>
       <c r="E7" s="16"/>
       <c r="F7" s="16"/>
-      <c r="G7" s="16"/>
+      <c r="G7" s="34"/>
       <c r="H7" s="16"/>
       <c r="I7" s="16"/>
       <c r="J7" s="16"/>
@@ -2177,7 +2254,7 @@
       <c r="D8" s="13"/>
       <c r="E8" s="13"/>
       <c r="F8" s="13"/>
-      <c r="G8" s="13"/>
+      <c r="G8" s="33"/>
       <c r="H8" s="13"/>
       <c r="I8" s="13"/>
       <c r="J8" s="13"/>
@@ -2192,7 +2269,7 @@
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
       <c r="F9" s="16"/>
-      <c r="G9" s="16"/>
+      <c r="G9" s="34"/>
       <c r="H9" s="16"/>
       <c r="I9" s="16"/>
       <c r="J9" s="16"/>
@@ -2207,7 +2284,7 @@
       <c r="D10" s="13"/>
       <c r="E10" s="13"/>
       <c r="F10" s="13"/>
-      <c r="G10" s="13"/>
+      <c r="G10" s="33"/>
       <c r="H10" s="13"/>
       <c r="I10" s="13"/>
       <c r="J10" s="13"/>
@@ -2222,7 +2299,7 @@
       <c r="D11" s="16"/>
       <c r="E11" s="16"/>
       <c r="F11" s="16"/>
-      <c r="G11" s="16"/>
+      <c r="G11" s="34"/>
       <c r="H11" s="16"/>
       <c r="I11" s="16"/>
       <c r="J11" s="16"/>
@@ -2237,7 +2314,7 @@
       <c r="D12" s="13"/>
       <c r="E12" s="13"/>
       <c r="F12" s="13"/>
-      <c r="G12" s="13"/>
+      <c r="G12" s="33"/>
       <c r="H12" s="13"/>
       <c r="I12" s="13"/>
       <c r="J12" s="13"/>
@@ -2252,7 +2329,7 @@
       <c r="D13" s="16"/>
       <c r="E13" s="16"/>
       <c r="F13" s="16"/>
-      <c r="G13" s="16"/>
+      <c r="G13" s="34"/>
       <c r="H13" s="16"/>
       <c r="I13" s="16"/>
       <c r="J13" s="16"/>
@@ -2267,7 +2344,7 @@
       <c r="D14" s="13"/>
       <c r="E14" s="13"/>
       <c r="F14" s="13"/>
-      <c r="G14" s="13"/>
+      <c r="G14" s="33"/>
       <c r="H14" s="13"/>
       <c r="I14" s="13"/>
       <c r="J14" s="13"/>
@@ -2282,7 +2359,7 @@
       <c r="D15" s="16"/>
       <c r="E15" s="16"/>
       <c r="F15" s="16"/>
-      <c r="G15" s="16"/>
+      <c r="G15" s="34"/>
       <c r="H15" s="16"/>
       <c r="I15" s="16"/>
       <c r="J15" s="16"/>
@@ -2297,7 +2374,7 @@
       <c r="D16" s="13"/>
       <c r="E16" s="13"/>
       <c r="F16" s="13"/>
-      <c r="G16" s="13"/>
+      <c r="G16" s="33"/>
       <c r="H16" s="13"/>
       <c r="I16" s="13"/>
       <c r="J16" s="13"/>
@@ -2312,7 +2389,7 @@
       <c r="D17" s="16"/>
       <c r="E17" s="16"/>
       <c r="F17" s="16"/>
-      <c r="G17" s="16"/>
+      <c r="G17" s="34"/>
       <c r="H17" s="16"/>
       <c r="I17" s="16"/>
       <c r="J17" s="16"/>
@@ -2327,7 +2404,7 @@
       <c r="D18" s="13"/>
       <c r="E18" s="13"/>
       <c r="F18" s="13"/>
-      <c r="G18" s="13"/>
+      <c r="G18" s="33"/>
       <c r="H18" s="13"/>
       <c r="I18" s="13"/>
       <c r="J18" s="13"/>
@@ -2342,7 +2419,7 @@
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
       <c r="F19" s="16"/>
-      <c r="G19" s="16"/>
+      <c r="G19" s="34"/>
       <c r="H19" s="16"/>
       <c r="I19" s="16"/>
       <c r="J19" s="16"/>
@@ -2357,7 +2434,7 @@
       <c r="D20" s="13"/>
       <c r="E20" s="13"/>
       <c r="F20" s="13"/>
-      <c r="G20" s="13"/>
+      <c r="G20" s="33"/>
       <c r="H20" s="13"/>
       <c r="I20" s="13"/>
       <c r="J20" s="13"/>
@@ -2372,7 +2449,7 @@
       <c r="D21" s="16"/>
       <c r="E21" s="16"/>
       <c r="F21" s="16"/>
-      <c r="G21" s="16"/>
+      <c r="G21" s="34"/>
       <c r="H21" s="16"/>
       <c r="I21" s="16"/>
       <c r="J21" s="16"/>
@@ -2387,7 +2464,7 @@
       <c r="D22" s="13"/>
       <c r="E22" s="13"/>
       <c r="F22" s="13"/>
-      <c r="G22" s="13"/>
+      <c r="G22" s="33"/>
       <c r="H22" s="13"/>
       <c r="I22" s="13"/>
       <c r="J22" s="13"/>
@@ -2402,7 +2479,7 @@
       <c r="D23" s="16"/>
       <c r="E23" s="16"/>
       <c r="F23" s="16"/>
-      <c r="G23" s="16"/>
+      <c r="G23" s="34"/>
       <c r="H23" s="16"/>
       <c r="I23" s="16"/>
       <c r="J23" s="16"/>
@@ -2417,7 +2494,7 @@
       <c r="D24" s="13"/>
       <c r="E24" s="13"/>
       <c r="F24" s="13"/>
-      <c r="G24" s="13"/>
+      <c r="G24" s="33"/>
       <c r="H24" s="13"/>
       <c r="I24" s="13"/>
       <c r="J24" s="13"/>
@@ -2432,7 +2509,7 @@
       <c r="D25" s="16"/>
       <c r="E25" s="16"/>
       <c r="F25" s="16"/>
-      <c r="G25" s="16"/>
+      <c r="G25" s="34"/>
       <c r="H25" s="16"/>
       <c r="I25" s="16"/>
       <c r="J25" s="16"/>
@@ -2447,7 +2524,7 @@
       <c r="D26" s="13"/>
       <c r="E26" s="13"/>
       <c r="F26" s="13"/>
-      <c r="G26" s="13"/>
+      <c r="G26" s="33"/>
       <c r="H26" s="13"/>
       <c r="I26" s="13"/>
       <c r="J26" s="13"/>
@@ -2462,7 +2539,7 @@
       <c r="D27" s="16"/>
       <c r="E27" s="16"/>
       <c r="F27" s="16"/>
-      <c r="G27" s="16"/>
+      <c r="G27" s="34"/>
       <c r="H27" s="16"/>
       <c r="I27" s="16"/>
       <c r="J27" s="16"/>
@@ -2477,7 +2554,7 @@
       <c r="D28" s="13"/>
       <c r="E28" s="13"/>
       <c r="F28" s="13"/>
-      <c r="G28" s="13"/>
+      <c r="G28" s="33"/>
       <c r="H28" s="13"/>
       <c r="I28" s="13"/>
       <c r="J28" s="13"/>
@@ -2492,7 +2569,7 @@
       <c r="D29" s="16"/>
       <c r="E29" s="16"/>
       <c r="F29" s="16"/>
-      <c r="G29" s="16"/>
+      <c r="G29" s="34"/>
       <c r="H29" s="16"/>
       <c r="I29" s="16"/>
       <c r="J29" s="16"/>
@@ -2507,7 +2584,7 @@
       <c r="D30" s="13"/>
       <c r="E30" s="13"/>
       <c r="F30" s="13"/>
-      <c r="G30" s="13"/>
+      <c r="G30" s="33"/>
       <c r="H30" s="13"/>
       <c r="I30" s="13"/>
       <c r="J30" s="13"/>
@@ -2522,7 +2599,7 @@
       <c r="D31" s="16"/>
       <c r="E31" s="16"/>
       <c r="F31" s="16"/>
-      <c r="G31" s="16"/>
+      <c r="G31" s="34"/>
       <c r="H31" s="16"/>
       <c r="I31" s="16"/>
       <c r="J31" s="16"/>
@@ -2537,7 +2614,7 @@
       <c r="D32" s="13"/>
       <c r="E32" s="13"/>
       <c r="F32" s="13"/>
-      <c r="G32" s="13"/>
+      <c r="G32" s="33"/>
       <c r="H32" s="13"/>
       <c r="I32" s="13"/>
       <c r="J32" s="13"/>
@@ -2552,7 +2629,7 @@
       <c r="D33" s="16"/>
       <c r="E33" s="16"/>
       <c r="F33" s="16"/>
-      <c r="G33" s="16"/>
+      <c r="G33" s="34"/>
       <c r="H33" s="16"/>
       <c r="I33" s="16"/>
       <c r="J33" s="16"/>
@@ -2567,7 +2644,7 @@
       <c r="D34" s="13"/>
       <c r="E34" s="13"/>
       <c r="F34" s="13"/>
-      <c r="G34" s="13"/>
+      <c r="G34" s="33"/>
       <c r="H34" s="13"/>
       <c r="I34" s="13"/>
       <c r="J34" s="13"/>
@@ -2582,7 +2659,7 @@
       <c r="D35" s="16"/>
       <c r="E35" s="16"/>
       <c r="F35" s="16"/>
-      <c r="G35" s="16"/>
+      <c r="G35" s="34"/>
       <c r="H35" s="16"/>
       <c r="I35" s="16"/>
       <c r="J35" s="16"/>
@@ -2597,7 +2674,7 @@
       <c r="D36" s="13"/>
       <c r="E36" s="13"/>
       <c r="F36" s="13"/>
-      <c r="G36" s="13"/>
+      <c r="G36" s="33"/>
       <c r="H36" s="13"/>
       <c r="I36" s="13"/>
       <c r="J36" s="13"/>
@@ -2612,7 +2689,7 @@
       <c r="D37" s="16"/>
       <c r="E37" s="16"/>
       <c r="F37" s="16"/>
-      <c r="G37" s="16"/>
+      <c r="G37" s="34"/>
       <c r="H37" s="16"/>
       <c r="I37" s="16"/>
       <c r="J37" s="16"/>
@@ -2627,7 +2704,7 @@
       <c r="D38" s="13"/>
       <c r="E38" s="13"/>
       <c r="F38" s="13"/>
-      <c r="G38" s="13"/>
+      <c r="G38" s="33"/>
       <c r="H38" s="13"/>
       <c r="I38" s="13"/>
       <c r="J38" s="13"/>
@@ -2642,7 +2719,7 @@
       <c r="D39" s="16"/>
       <c r="E39" s="16"/>
       <c r="F39" s="16"/>
-      <c r="G39" s="16"/>
+      <c r="G39" s="34"/>
       <c r="H39" s="16"/>
       <c r="I39" s="16"/>
       <c r="J39" s="16"/>
@@ -2657,7 +2734,7 @@
       <c r="D40" s="13"/>
       <c r="E40" s="13"/>
       <c r="F40" s="13"/>
-      <c r="G40" s="13"/>
+      <c r="G40" s="33"/>
       <c r="H40" s="13"/>
       <c r="I40" s="13"/>
       <c r="J40" s="13"/>
@@ -2672,7 +2749,7 @@
       <c r="D41" s="16"/>
       <c r="E41" s="16"/>
       <c r="F41" s="16"/>
-      <c r="G41" s="16"/>
+      <c r="G41" s="34"/>
       <c r="H41" s="16"/>
       <c r="I41" s="16"/>
       <c r="J41" s="16"/>
@@ -2687,7 +2764,7 @@
       <c r="D42" s="13"/>
       <c r="E42" s="13"/>
       <c r="F42" s="13"/>
-      <c r="G42" s="13"/>
+      <c r="G42" s="33"/>
       <c r="H42" s="13"/>
       <c r="I42" s="13"/>
       <c r="J42" s="13"/>
@@ -2702,7 +2779,7 @@
       <c r="D43" s="16"/>
       <c r="E43" s="16"/>
       <c r="F43" s="16"/>
-      <c r="G43" s="16"/>
+      <c r="G43" s="34"/>
       <c r="H43" s="16"/>
       <c r="I43" s="16"/>
       <c r="J43" s="16"/>
@@ -2717,7 +2794,7 @@
       <c r="D44" s="13"/>
       <c r="E44" s="13"/>
       <c r="F44" s="13"/>
-      <c r="G44" s="13"/>
+      <c r="G44" s="33"/>
       <c r="H44" s="13"/>
       <c r="I44" s="13"/>
       <c r="J44" s="13"/>
@@ -2732,7 +2809,7 @@
       <c r="D45" s="16"/>
       <c r="E45" s="16"/>
       <c r="F45" s="16"/>
-      <c r="G45" s="16"/>
+      <c r="G45" s="34"/>
       <c r="H45" s="16"/>
       <c r="I45" s="16"/>
       <c r="J45" s="16"/>
@@ -2747,7 +2824,7 @@
       <c r="D46" s="13"/>
       <c r="E46" s="13"/>
       <c r="F46" s="13"/>
-      <c r="G46" s="13"/>
+      <c r="G46" s="33"/>
       <c r="H46" s="13"/>
       <c r="I46" s="13"/>
       <c r="J46" s="13"/>
@@ -2762,7 +2839,7 @@
       <c r="D47" s="16"/>
       <c r="E47" s="16"/>
       <c r="F47" s="16"/>
-      <c r="G47" s="16"/>
+      <c r="G47" s="34"/>
       <c r="H47" s="16"/>
       <c r="I47" s="16"/>
       <c r="J47" s="16"/>
@@ -2777,7 +2854,7 @@
       <c r="D48" s="13"/>
       <c r="E48" s="13"/>
       <c r="F48" s="13"/>
-      <c r="G48" s="13"/>
+      <c r="G48" s="33"/>
       <c r="H48" s="13"/>
       <c r="I48" s="13"/>
       <c r="J48" s="13"/>
@@ -2792,7 +2869,7 @@
       <c r="D49" s="16"/>
       <c r="E49" s="16"/>
       <c r="F49" s="16"/>
-      <c r="G49" s="16"/>
+      <c r="G49" s="34"/>
       <c r="H49" s="16"/>
       <c r="I49" s="16"/>
       <c r="J49" s="16"/>
@@ -2807,7 +2884,7 @@
       <c r="D50" s="13"/>
       <c r="E50" s="13"/>
       <c r="F50" s="13"/>
-      <c r="G50" s="13"/>
+      <c r="G50" s="33"/>
       <c r="H50" s="13"/>
       <c r="I50" s="13"/>
       <c r="J50" s="13"/>
@@ -2822,7 +2899,7 @@
       <c r="D51" s="16"/>
       <c r="E51" s="16"/>
       <c r="F51" s="16"/>
-      <c r="G51" s="16"/>
+      <c r="G51" s="34"/>
       <c r="H51" s="16"/>
       <c r="I51" s="16"/>
       <c r="J51" s="16"/>
@@ -2837,7 +2914,7 @@
       <c r="D52" s="13"/>
       <c r="E52" s="13"/>
       <c r="F52" s="13"/>
-      <c r="G52" s="13"/>
+      <c r="G52" s="33"/>
       <c r="H52" s="13"/>
       <c r="I52" s="13"/>
       <c r="J52" s="13"/>
@@ -2852,7 +2929,7 @@
       <c r="D53" s="16"/>
       <c r="E53" s="16"/>
       <c r="F53" s="16"/>
-      <c r="G53" s="16"/>
+      <c r="G53" s="34"/>
       <c r="H53" s="16"/>
       <c r="I53" s="16"/>
       <c r="J53" s="16"/>
@@ -2867,7 +2944,7 @@
       <c r="D54" s="13"/>
       <c r="E54" s="13"/>
       <c r="F54" s="13"/>
-      <c r="G54" s="13"/>
+      <c r="G54" s="33"/>
       <c r="H54" s="13"/>
       <c r="I54" s="13"/>
       <c r="J54" s="13"/>
@@ -2882,7 +2959,7 @@
       <c r="D55" s="16"/>
       <c r="E55" s="16"/>
       <c r="F55" s="16"/>
-      <c r="G55" s="16"/>
+      <c r="G55" s="34"/>
       <c r="H55" s="16"/>
       <c r="I55" s="16"/>
       <c r="J55" s="16"/>
@@ -2897,7 +2974,7 @@
       <c r="D56" s="13"/>
       <c r="E56" s="13"/>
       <c r="F56" s="13"/>
-      <c r="G56" s="13"/>
+      <c r="G56" s="33"/>
       <c r="H56" s="13"/>
       <c r="I56" s="13"/>
       <c r="J56" s="13"/>
@@ -2912,7 +2989,7 @@
       <c r="D57" s="16"/>
       <c r="E57" s="16"/>
       <c r="F57" s="16"/>
-      <c r="G57" s="16"/>
+      <c r="G57" s="34"/>
       <c r="H57" s="16"/>
       <c r="I57" s="16"/>
       <c r="J57" s="16"/>
@@ -2927,7 +3004,7 @@
       <c r="D58" s="13"/>
       <c r="E58" s="13"/>
       <c r="F58" s="13"/>
-      <c r="G58" s="13"/>
+      <c r="G58" s="33"/>
       <c r="H58" s="13"/>
       <c r="I58" s="13"/>
       <c r="J58" s="13"/>
@@ -2942,7 +3019,7 @@
       <c r="D59" s="16"/>
       <c r="E59" s="16"/>
       <c r="F59" s="16"/>
-      <c r="G59" s="16"/>
+      <c r="G59" s="34"/>
       <c r="H59" s="16"/>
       <c r="I59" s="16"/>
       <c r="J59" s="16"/>
@@ -2957,7 +3034,7 @@
       <c r="D60" s="13"/>
       <c r="E60" s="13"/>
       <c r="F60" s="13"/>
-      <c r="G60" s="13"/>
+      <c r="G60" s="33"/>
       <c r="H60" s="13"/>
       <c r="I60" s="13"/>
       <c r="J60" s="13"/>
@@ -2972,7 +3049,7 @@
       <c r="D61" s="16"/>
       <c r="E61" s="16"/>
       <c r="F61" s="16"/>
-      <c r="G61" s="16"/>
+      <c r="G61" s="34"/>
       <c r="H61" s="16"/>
       <c r="I61" s="16"/>
       <c r="J61" s="16"/>
@@ -2987,7 +3064,7 @@
       <c r="D62" s="13"/>
       <c r="E62" s="13"/>
       <c r="F62" s="13"/>
-      <c r="G62" s="13"/>
+      <c r="G62" s="33"/>
       <c r="H62" s="13"/>
       <c r="I62" s="13"/>
       <c r="J62" s="13"/>
@@ -3002,7 +3079,7 @@
       <c r="D63" s="16"/>
       <c r="E63" s="16"/>
       <c r="F63" s="16"/>
-      <c r="G63" s="16"/>
+      <c r="G63" s="34"/>
       <c r="H63" s="16"/>
       <c r="I63" s="16"/>
       <c r="J63" s="16"/>
@@ -3017,7 +3094,7 @@
       <c r="D64" s="13"/>
       <c r="E64" s="13"/>
       <c r="F64" s="13"/>
-      <c r="G64" s="13"/>
+      <c r="G64" s="33"/>
       <c r="H64" s="13"/>
       <c r="I64" s="13"/>
       <c r="J64" s="13"/>
@@ -3032,7 +3109,7 @@
       <c r="D65" s="16"/>
       <c r="E65" s="16"/>
       <c r="F65" s="16"/>
-      <c r="G65" s="16"/>
+      <c r="G65" s="34"/>
       <c r="H65" s="16"/>
       <c r="I65" s="16"/>
       <c r="J65" s="16"/>
@@ -3047,7 +3124,7 @@
       <c r="D66" s="13"/>
       <c r="E66" s="13"/>
       <c r="F66" s="13"/>
-      <c r="G66" s="13"/>
+      <c r="G66" s="33"/>
       <c r="H66" s="13"/>
       <c r="I66" s="13"/>
       <c r="J66" s="13"/>
@@ -3062,7 +3139,7 @@
       <c r="D67" s="16"/>
       <c r="E67" s="16"/>
       <c r="F67" s="16"/>
-      <c r="G67" s="16"/>
+      <c r="G67" s="34"/>
       <c r="H67" s="16"/>
       <c r="I67" s="16"/>
       <c r="J67" s="16"/>
@@ -3077,7 +3154,7 @@
       <c r="D68" s="13"/>
       <c r="E68" s="13"/>
       <c r="F68" s="13"/>
-      <c r="G68" s="13"/>
+      <c r="G68" s="33"/>
       <c r="H68" s="13"/>
       <c r="I68" s="13"/>
       <c r="J68" s="13"/>
@@ -3092,7 +3169,7 @@
       <c r="D69" s="16"/>
       <c r="E69" s="16"/>
       <c r="F69" s="16"/>
-      <c r="G69" s="16"/>
+      <c r="G69" s="34"/>
       <c r="H69" s="16"/>
       <c r="I69" s="16"/>
       <c r="J69" s="16"/>
@@ -3107,7 +3184,7 @@
       <c r="D70" s="13"/>
       <c r="E70" s="13"/>
       <c r="F70" s="13"/>
-      <c r="G70" s="13"/>
+      <c r="G70" s="33"/>
       <c r="H70" s="13"/>
       <c r="I70" s="13"/>
       <c r="J70" s="13"/>
@@ -3122,7 +3199,7 @@
       <c r="D71" s="16"/>
       <c r="E71" s="16"/>
       <c r="F71" s="16"/>
-      <c r="G71" s="16"/>
+      <c r="G71" s="34"/>
       <c r="H71" s="16"/>
       <c r="I71" s="16"/>
       <c r="J71" s="16"/>
@@ -3137,7 +3214,7 @@
       <c r="D72" s="13"/>
       <c r="E72" s="13"/>
       <c r="F72" s="13"/>
-      <c r="G72" s="13"/>
+      <c r="G72" s="33"/>
       <c r="H72" s="13"/>
       <c r="I72" s="13"/>
       <c r="J72" s="13"/>
@@ -3152,7 +3229,7 @@
       <c r="D73" s="16"/>
       <c r="E73" s="16"/>
       <c r="F73" s="16"/>
-      <c r="G73" s="16"/>
+      <c r="G73" s="34"/>
       <c r="H73" s="16"/>
       <c r="I73" s="16"/>
       <c r="J73" s="16"/>
@@ -3167,7 +3244,7 @@
       <c r="D74" s="13"/>
       <c r="E74" s="13"/>
       <c r="F74" s="13"/>
-      <c r="G74" s="13"/>
+      <c r="G74" s="33"/>
       <c r="H74" s="13"/>
       <c r="I74" s="13"/>
       <c r="J74" s="13"/>
@@ -3182,7 +3259,7 @@
       <c r="D75" s="16"/>
       <c r="E75" s="16"/>
       <c r="F75" s="16"/>
-      <c r="G75" s="16"/>
+      <c r="G75" s="34"/>
       <c r="H75" s="16"/>
       <c r="I75" s="16"/>
       <c r="J75" s="16"/>
@@ -3197,7 +3274,7 @@
       <c r="D76" s="13"/>
       <c r="E76" s="13"/>
       <c r="F76" s="13"/>
-      <c r="G76" s="13"/>
+      <c r="G76" s="33"/>
       <c r="H76" s="13"/>
       <c r="I76" s="13"/>
       <c r="J76" s="13"/>
@@ -3212,7 +3289,7 @@
       <c r="D77" s="16"/>
       <c r="E77" s="16"/>
       <c r="F77" s="16"/>
-      <c r="G77" s="16"/>
+      <c r="G77" s="34"/>
       <c r="H77" s="16"/>
       <c r="I77" s="16"/>
       <c r="J77" s="16"/>
@@ -3227,7 +3304,7 @@
       <c r="D78" s="13"/>
       <c r="E78" s="13"/>
       <c r="F78" s="13"/>
-      <c r="G78" s="13"/>
+      <c r="G78" s="33"/>
       <c r="H78" s="13"/>
       <c r="I78" s="13"/>
       <c r="J78" s="13"/>
@@ -3242,7 +3319,7 @@
       <c r="D79" s="16"/>
       <c r="E79" s="16"/>
       <c r="F79" s="16"/>
-      <c r="G79" s="16"/>
+      <c r="G79" s="34"/>
       <c r="H79" s="16"/>
       <c r="I79" s="16"/>
       <c r="J79" s="16"/>
@@ -3257,7 +3334,7 @@
       <c r="D80" s="13"/>
       <c r="E80" s="13"/>
       <c r="F80" s="13"/>
-      <c r="G80" s="13"/>
+      <c r="G80" s="33"/>
       <c r="H80" s="13"/>
       <c r="I80" s="13"/>
       <c r="J80" s="13"/>
@@ -3272,7 +3349,7 @@
       <c r="D81" s="16"/>
       <c r="E81" s="16"/>
       <c r="F81" s="16"/>
-      <c r="G81" s="16"/>
+      <c r="G81" s="34"/>
       <c r="H81" s="16"/>
       <c r="I81" s="16"/>
       <c r="J81" s="16"/>
@@ -3287,7 +3364,7 @@
       <c r="D82" s="13"/>
       <c r="E82" s="13"/>
       <c r="F82" s="13"/>
-      <c r="G82" s="13"/>
+      <c r="G82" s="33"/>
       <c r="H82" s="13"/>
       <c r="I82" s="13"/>
       <c r="J82" s="13"/>
@@ -3302,7 +3379,7 @@
       <c r="D83" s="16"/>
       <c r="E83" s="16"/>
       <c r="F83" s="16"/>
-      <c r="G83" s="16"/>
+      <c r="G83" s="34"/>
       <c r="H83" s="16"/>
       <c r="I83" s="16"/>
       <c r="J83" s="16"/>
@@ -3317,7 +3394,7 @@
       <c r="D84" s="13"/>
       <c r="E84" s="13"/>
       <c r="F84" s="13"/>
-      <c r="G84" s="13"/>
+      <c r="G84" s="33"/>
       <c r="H84" s="13"/>
       <c r="I84" s="13"/>
       <c r="J84" s="13"/>
@@ -3332,7 +3409,7 @@
       <c r="D85" s="16"/>
       <c r="E85" s="16"/>
       <c r="F85" s="16"/>
-      <c r="G85" s="16"/>
+      <c r="G85" s="34"/>
       <c r="H85" s="16"/>
       <c r="I85" s="16"/>
       <c r="J85" s="16"/>
@@ -3347,7 +3424,7 @@
       <c r="D86" s="13"/>
       <c r="E86" s="13"/>
       <c r="F86" s="13"/>
-      <c r="G86" s="13"/>
+      <c r="G86" s="33"/>
       <c r="H86" s="13"/>
       <c r="I86" s="13"/>
       <c r="J86" s="13"/>
@@ -3362,7 +3439,7 @@
       <c r="D87" s="16"/>
       <c r="E87" s="16"/>
       <c r="F87" s="16"/>
-      <c r="G87" s="16"/>
+      <c r="G87" s="34"/>
       <c r="H87" s="16"/>
       <c r="I87" s="16"/>
       <c r="J87" s="16"/>
@@ -3377,7 +3454,7 @@
       <c r="D88" s="13"/>
       <c r="E88" s="13"/>
       <c r="F88" s="13"/>
-      <c r="G88" s="13"/>
+      <c r="G88" s="33"/>
       <c r="H88" s="13"/>
       <c r="I88" s="13"/>
       <c r="J88" s="13"/>
@@ -3392,7 +3469,7 @@
       <c r="D89" s="16"/>
       <c r="E89" s="16"/>
       <c r="F89" s="16"/>
-      <c r="G89" s="16"/>
+      <c r="G89" s="34"/>
       <c r="H89" s="16"/>
       <c r="I89" s="16"/>
       <c r="J89" s="16"/>
@@ -3407,7 +3484,7 @@
       <c r="D90" s="13"/>
       <c r="E90" s="13"/>
       <c r="F90" s="13"/>
-      <c r="G90" s="13"/>
+      <c r="G90" s="33"/>
       <c r="H90" s="13"/>
       <c r="I90" s="13"/>
       <c r="J90" s="13"/>
@@ -3422,7 +3499,7 @@
       <c r="D91" s="16"/>
       <c r="E91" s="16"/>
       <c r="F91" s="16"/>
-      <c r="G91" s="16"/>
+      <c r="G91" s="34"/>
       <c r="H91" s="16"/>
       <c r="I91" s="16"/>
       <c r="J91" s="16"/>
@@ -3437,7 +3514,7 @@
       <c r="D92" s="13"/>
       <c r="E92" s="13"/>
       <c r="F92" s="13"/>
-      <c r="G92" s="13"/>
+      <c r="G92" s="33"/>
       <c r="H92" s="13"/>
       <c r="I92" s="13"/>
       <c r="J92" s="13"/>
@@ -3452,7 +3529,7 @@
       <c r="D93" s="16"/>
       <c r="E93" s="16"/>
       <c r="F93" s="16"/>
-      <c r="G93" s="16"/>
+      <c r="G93" s="34"/>
       <c r="H93" s="16"/>
       <c r="I93" s="16"/>
       <c r="J93" s="16"/>
@@ -3467,7 +3544,7 @@
       <c r="D94" s="13"/>
       <c r="E94" s="13"/>
       <c r="F94" s="13"/>
-      <c r="G94" s="13"/>
+      <c r="G94" s="33"/>
       <c r="H94" s="13"/>
       <c r="I94" s="13"/>
       <c r="J94" s="13"/>
@@ -3482,7 +3559,7 @@
       <c r="D95" s="16"/>
       <c r="E95" s="16"/>
       <c r="F95" s="16"/>
-      <c r="G95" s="16"/>
+      <c r="G95" s="34"/>
       <c r="H95" s="16"/>
       <c r="I95" s="16"/>
       <c r="J95" s="16"/>
@@ -3497,7 +3574,7 @@
       <c r="D96" s="13"/>
       <c r="E96" s="13"/>
       <c r="F96" s="13"/>
-      <c r="G96" s="13"/>
+      <c r="G96" s="33"/>
       <c r="H96" s="13"/>
       <c r="I96" s="13"/>
       <c r="J96" s="13"/>
@@ -3512,7 +3589,7 @@
       <c r="D97" s="16"/>
       <c r="E97" s="16"/>
       <c r="F97" s="16"/>
-      <c r="G97" s="16"/>
+      <c r="G97" s="34"/>
       <c r="H97" s="16"/>
       <c r="I97" s="16"/>
       <c r="J97" s="16"/>
@@ -3527,7 +3604,7 @@
       <c r="D98" s="13"/>
       <c r="E98" s="13"/>
       <c r="F98" s="13"/>
-      <c r="G98" s="13"/>
+      <c r="G98" s="33"/>
       <c r="H98" s="13"/>
       <c r="I98" s="13"/>
       <c r="J98" s="13"/>
@@ -3542,7 +3619,7 @@
       <c r="D99" s="16"/>
       <c r="E99" s="16"/>
       <c r="F99" s="16"/>
-      <c r="G99" s="16"/>
+      <c r="G99" s="34"/>
       <c r="H99" s="16"/>
       <c r="I99" s="16"/>
       <c r="J99" s="16"/>
@@ -3557,7 +3634,7 @@
       <c r="D100" s="9"/>
       <c r="E100" s="9"/>
       <c r="F100" s="9"/>
-      <c r="G100" s="9"/>
+      <c r="G100" s="35"/>
       <c r="H100" s="9"/>
       <c r="I100" s="9"/>
       <c r="J100" s="9"/>
@@ -3654,7 +3731,7 @@
       </c>
       <c r="B12" s="6">
         <f>SUM(Transactions!$G$2:$G$100)</f>
-        <v>260</v>
+        <v>560</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
@@ -3681,7 +3758,7 @@
       </c>
       <c r="B15" s="6">
         <f>SUMIF(Transactions!$E$2:$E$100,"Food",Transactions!$G$2:$G$100)</f>
-        <v>260</v>
+        <v>320</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
@@ -3690,7 +3767,7 @@
       </c>
       <c r="B16" s="6">
         <f>SUMIF(Transactions!$E$2:$E$100,"Travel",Transactions!$G$2:$G$100)</f>
-        <v>0</v>
+        <v>240</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
@@ -3714,7 +3791,7 @@
       </c>
       <c r="B21" s="6">
         <f>B7-B12</f>
-        <v>21740</v>
+        <v>21440</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
@@ -3723,7 +3800,7 @@
       </c>
       <c r="B22" s="1">
         <f>B21/B7%</f>
-        <v>98.818181818181813</v>
+        <v>97.454545454545453</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
@@ -3768,7 +3845,7 @@
       </c>
       <c r="B31" s="7">
         <f>B21-B27</f>
-        <v>10740</v>
+        <v>10440</v>
       </c>
     </row>
   </sheetData>
@@ -3931,9 +4008,9 @@
   <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="4" width="13" style="31" customWidth="1"/>
-    <col min="5" max="5" width="9.44140625" style="31" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.6640625" style="31" customWidth="1"/>
+    <col min="4" max="4" width="13" style="30" customWidth="1"/>
+    <col min="5" max="5" width="9.44140625" style="30" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.6640625" style="30" customWidth="1"/>
     <col min="7" max="7" width="10.33203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3947,13 +4024,13 @@
       <c r="C1" t="s">
         <v>66</v>
       </c>
-      <c r="D1" s="31" t="s">
+      <c r="D1" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="31" t="s">
+      <c r="E1" s="30" t="s">
         <v>194</v>
       </c>
-      <c r="F1" s="31" t="s">
+      <c r="F1" s="30" t="s">
         <v>195</v>
       </c>
       <c r="G1" t="s">
@@ -3976,13 +4053,13 @@
       <c r="C2" t="s">
         <v>198</v>
       </c>
-      <c r="D2" s="31">
+      <c r="D2" s="30">
         <v>10000</v>
       </c>
-      <c r="E2" s="31">
+      <c r="E2" s="30">
         <v>0</v>
       </c>
-      <c r="F2" s="31">
+      <c r="F2" s="30">
         <v>10000</v>
       </c>
       <c r="G2" t="s">
@@ -4005,13 +4082,13 @@
       <c r="C3" t="s">
         <v>203</v>
       </c>
-      <c r="D3" s="31">
+      <c r="D3" s="30">
         <v>2000</v>
       </c>
-      <c r="E3" s="31">
+      <c r="E3" s="30">
         <v>1000</v>
       </c>
-      <c r="F3" s="31">
+      <c r="F3" s="30">
         <v>1000</v>
       </c>
       <c r="G3" s="24">
@@ -4034,13 +4111,13 @@
       <c r="C4" t="s">
         <v>203</v>
       </c>
-      <c r="D4" s="31">
+      <c r="D4" s="30">
         <v>1000</v>
       </c>
-      <c r="E4" s="31">
+      <c r="E4" s="30">
         <v>1000</v>
       </c>
-      <c r="F4" s="31">
+      <c r="F4" s="30">
         <v>0</v>
       </c>
       <c r="G4" s="24">

</xml_diff>

<commit_message>
v0.8.0 add budget analysis engine and budget insights engine
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -8,22 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pratham OS\Development\Finance-AI\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{068C975F-2FEC-41B3-9C79-82359F59E53F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0E21683-B879-4BDB-8E6F-21B29DB494F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{D6DE1A26-0963-4585-A363-547897EAF3B2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="2" xr2:uid="{D6DE1A26-0963-4585-A363-547897EAF3B2}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan" sheetId="1" r:id="rId1"/>
     <sheet name="Transactions" sheetId="2" r:id="rId2"/>
-    <sheet name="Dashboard" sheetId="4" r:id="rId3"/>
-    <sheet name="Monthly Review" sheetId="5" r:id="rId4"/>
-    <sheet name="Skill Tracker" sheetId="9" r:id="rId5"/>
-    <sheet name="Financial Commitments" sheetId="10" r:id="rId6"/>
-    <sheet name="Income" sheetId="11" r:id="rId7"/>
-    <sheet name="Income engine" sheetId="6" r:id="rId8"/>
-    <sheet name="Carrer Tracker" sheetId="7" r:id="rId9"/>
-    <sheet name="Interview Prep" sheetId="8" r:id="rId10"/>
-    <sheet name="Lists" sheetId="3" r:id="rId11"/>
+    <sheet name="Budget Sheet" sheetId="13" r:id="rId3"/>
+    <sheet name="Financial Commitments" sheetId="10" r:id="rId4"/>
+    <sheet name="Dashboard" sheetId="4" r:id="rId5"/>
+    <sheet name="Monthly Review" sheetId="5" r:id="rId6"/>
+    <sheet name="Skill Tracker" sheetId="9" r:id="rId7"/>
+    <sheet name="Income" sheetId="11" r:id="rId8"/>
+    <sheet name="Income engine" sheetId="6" r:id="rId9"/>
+    <sheet name="Carrer Tracker" sheetId="7" r:id="rId10"/>
+    <sheet name="Interview Prep" sheetId="8" r:id="rId11"/>
+    <sheet name="Lists" sheetId="3" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="AppliedStatus">Lists!$K$1:$K$10</definedName>
@@ -64,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="228">
   <si>
     <t>August Financial Plan</t>
   </si>
@@ -300,6 +301,9 @@
     <t>Recurring</t>
   </si>
   <si>
+    <t>Year</t>
+  </si>
+  <si>
     <t>Current Situation</t>
   </si>
   <si>
@@ -742,6 +746,9 @@
   </si>
   <si>
     <t>breakfast</t>
+  </si>
+  <si>
+    <t>Monthly_Budget</t>
   </si>
 </sst>
 </file>
@@ -753,7 +760,7 @@
     <numFmt numFmtId="44" formatCode="_ &quot;₹&quot;\ * #,##0.00_ ;_ &quot;₹&quot;\ * \-#,##0.00_ ;_ &quot;₹&quot;\ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -780,6 +787,12 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -898,7 +911,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -938,12 +951,16 @@
     <xf numFmtId="14" fontId="2" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="19">
+  <dxfs count="20">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
     </dxf>
@@ -1071,14 +1088,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{42D67FA3-A40A-4607-BCB9-468A9ECB0007}" name="Table1" displayName="Table1" ref="A1:H1048576" totalsRowShown="0" headerRowDxfId="18" tableBorderDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{42D67FA3-A40A-4607-BCB9-468A9ECB0007}" name="Table1" displayName="Table1" ref="A1:H1048576" totalsRowShown="0" headerRowDxfId="19" tableBorderDxfId="18">
   <autoFilter ref="A1:H1048576" xr:uid="{42D67FA3-A40A-4607-BCB9-468A9ECB0007}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{1D37F906-33D7-46E6-8270-56D5EEA80EC7}" name="Date" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{1D37F906-33D7-46E6-8270-56D5EEA80EC7}" name="Date" dataDxfId="1"/>
     <tableColumn id="4" xr3:uid="{E805A8A8-660D-4099-912A-BE1B697553ED}" name="Type"/>
     <tableColumn id="5" xr3:uid="{ABF1E4D7-7922-479D-94F4-994DCBA1062D}" name="Category"/>
     <tableColumn id="6" xr3:uid="{E21EA904-BC60-4EB5-B4BD-249E5A12FC76}" name="Description "/>
-    <tableColumn id="7" xr3:uid="{EFA172CE-B81A-4A83-BB09-0C52BED62422}" name="Amount" dataDxfId="16"/>
+    <tableColumn id="7" xr3:uid="{EFA172CE-B81A-4A83-BB09-0C52BED62422}" name="Amount" dataDxfId="17"/>
     <tableColumn id="8" xr3:uid="{E811D3EB-DAD5-46D9-B70D-01072B332F5C}" name="Need/Want"/>
     <tableColumn id="9" xr3:uid="{1E8766C9-2C6F-4CE3-9C7E-C6C8545D3945}" name="Payment Mode"/>
     <tableColumn id="10" xr3:uid="{BA26CD78-BAFB-4644-808D-0A18546F6CAF}" name="Recurring"/>
@@ -1088,15 +1105,27 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{204CD917-42D7-44E9-889E-B87F7E170616}" name="Table5" displayName="Table5" ref="A1:C100" totalsRowShown="0">
+  <autoFilter ref="A1:C100" xr:uid="{204CD917-42D7-44E9-889E-B87F7E170616}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{CCD99EA9-9CA0-4F69-8282-1EE2E5FE7967}" name="Month" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{5C307EC1-8BAE-4B8C-AF42-D468202B7A5E}" name="Year"/>
+    <tableColumn id="3" xr3:uid="{2B3569FD-9348-4E00-BFEA-53DF4F58E82C}" name="Monthly_Budget"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{1AFBBFA5-5EA2-4DA5-91C7-5EE90985F084}" name="FinancialCommitments" displayName="FinancialCommitments" ref="A1:I50" totalsRowShown="0">
   <autoFilter ref="A1:I50" xr:uid="{1AFBBFA5-5EA2-4DA5-91C7-5EE90985F084}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{C10697DD-F282-4D7F-A12A-9BFC6193DC4E}" name="Date " dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{C10697DD-F282-4D7F-A12A-9BFC6193DC4E}" name="Date " dataDxfId="2"/>
     <tableColumn id="2" xr3:uid="{D6130D6E-B2EE-4D09-94CD-7E8053CD1C7B}" name="From"/>
     <tableColumn id="3" xr3:uid="{8ECD20EB-BEF0-47D5-8DA5-28D491EC7B0A}" name="Type"/>
-    <tableColumn id="4" xr3:uid="{87D047F3-8B64-4D30-ACC0-42FFF26FEC3E}" name="Amount" dataDxfId="15"/>
-    <tableColumn id="5" xr3:uid="{C982624C-E448-4958-A5CE-7D794FC142FA}" name="Repaid" dataDxfId="14"/>
-    <tableColumn id="6" xr3:uid="{665D5056-3744-4E56-95C7-F0943FD35707}" name="Remaining" dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{87D047F3-8B64-4D30-ACC0-42FFF26FEC3E}" name="Amount" dataDxfId="16"/>
+    <tableColumn id="5" xr3:uid="{C982624C-E448-4958-A5CE-7D794FC142FA}" name="Repaid" dataDxfId="15"/>
+    <tableColumn id="6" xr3:uid="{665D5056-3744-4E56-95C7-F0943FD35707}" name="Remaining" dataDxfId="14"/>
     <tableColumn id="7" xr3:uid="{FFDA91C5-2668-4023-9FEE-465A59D85270}" name="Due Date"/>
     <tableColumn id="8" xr3:uid="{748EB09B-78B0-49AB-AC7E-88A7F4C42C89}" name="Status"/>
     <tableColumn id="9" xr3:uid="{9F5FA8E8-540D-4C48-B339-C097673FD287}" name="Notes"/>
@@ -1105,23 +1134,23 @@
 </table>
 </file>
 
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{7C5D4057-F5F1-485E-AE6E-34A855BB81C8}" name="IncomeTable" displayName="IncomeTable" ref="A1:G4" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{7C5D4057-F5F1-485E-AE6E-34A855BB81C8}" name="IncomeTable" displayName="IncomeTable" ref="A1:G4" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
   <autoFilter ref="A1:G4" xr:uid="{7C5D4057-F5F1-485E-AE6E-34A855BB81C8}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{85417279-B333-4129-826F-4B13A464B0A1}" name="Date" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{72151722-7F6E-43AF-AADF-05A0452D151E}" name="Source" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{A9F1D760-964B-4BC4-876E-FE2B218C85B6}" name="Category" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{31C0BCAE-AC93-4345-9B1C-546CE0735A6B}" name="Amount" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{C6E99480-C881-404B-8F25-E2549BD2CCCD}" name="Status" dataDxfId="6"/>
-    <tableColumn id="7" xr3:uid="{29AC2CCC-8D50-4D4F-9049-D5CBB08CDAB6}" name="Recurring" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{4D5A0A55-4298-4332-9A93-683CDAE35676}" name="Notes" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{85417279-B333-4129-826F-4B13A464B0A1}" name="Date" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{72151722-7F6E-43AF-AADF-05A0452D151E}" name="Source" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{A9F1D760-964B-4BC4-876E-FE2B218C85B6}" name="Category" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{31C0BCAE-AC93-4345-9B1C-546CE0735A6B}" name="Amount" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{C6E99480-C881-404B-8F25-E2549BD2CCCD}" name="Status" dataDxfId="7"/>
+    <tableColumn id="7" xr3:uid="{29AC2CCC-8D50-4D4F-9049-D5CBB08CDAB6}" name="Recurring" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{4D5A0A55-4298-4332-9A93-683CDAE35676}" name="Notes" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2E0C23CD-1E80-4D43-9A03-38675147AE03}" name="Table2" displayName="Table2" ref="A1:J50" totalsRowShown="0">
   <autoFilter ref="A1:J50" xr:uid="{2E0C23CD-1E80-4D43-9A03-38675147AE03}"/>
   <tableColumns count="10">
@@ -1650,10 +1679,10 @@
     <mergeCell ref="A1:D1"/>
   </mergeCells>
   <conditionalFormatting sqref="B17:B20">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="4" priority="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="3" priority="2" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1663,22 +1692,158 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{062E0065-A33A-40A3-8681-B93160D6FE12}">
+  <dimension ref="A1:Q5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="10.77734375" customWidth="1"/>
+    <col min="4" max="4" width="13.6640625" customWidth="1"/>
+    <col min="5" max="5" width="14.77734375" customWidth="1"/>
+    <col min="7" max="7" width="11.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C1" t="s">
+        <v>127</v>
+      </c>
+      <c r="D1" t="s">
+        <v>128</v>
+      </c>
+      <c r="E1" t="s">
+        <v>129</v>
+      </c>
+      <c r="F1" t="s">
+        <v>130</v>
+      </c>
+      <c r="G1" t="s">
+        <v>178</v>
+      </c>
+      <c r="H1" t="s">
+        <v>131</v>
+      </c>
+      <c r="I1" t="s">
+        <v>179</v>
+      </c>
+      <c r="J1" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" t="s">
+        <v>142</v>
+      </c>
+      <c r="C2">
+        <v>22000</v>
+      </c>
+      <c r="F2" t="s">
+        <v>132</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" t="s">
+        <v>143</v>
+      </c>
+      <c r="C3">
+        <v>23000</v>
+      </c>
+      <c r="F3" t="s">
+        <v>132</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s">
+        <v>144</v>
+      </c>
+      <c r="C4">
+        <v>28000</v>
+      </c>
+      <c r="F4" t="s">
+        <v>132</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>145</v>
+      </c>
+      <c r="B5" t="s">
+        <v>146</v>
+      </c>
+      <c r="C5">
+        <v>20000</v>
+      </c>
+      <c r="F5" t="s">
+        <v>132</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>150</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="4">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F50" xr:uid="{B7B46CB3-D4D6-4415-A547-30F33809F18A}">
+      <formula1>AppliedStatus</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H50" xr:uid="{A0AB4D2E-03DC-499E-A809-B6BDCD0E9591}">
+      <formula1>InterviewResult</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G1:G1048576" xr:uid="{DAD8A552-FAB1-4D16-90F0-ACE3B457489B}">
+      <formula1>InterviewRound</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I1:I1048576" xr:uid="{F32AF372-FB7D-40CA-8785-F217A85AC485}">
+      <formula1>NextAction</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52E36AC4-05BC-4C7B-BA73-388CE26BAB52}">
   <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>57</v>
@@ -1686,52 +1851,52 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
   </sheetData>
@@ -1739,7 +1904,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{729B4158-2DD5-48A6-9BEC-2F739409F312}">
   <dimension ref="A1:Q19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1761,16 +1926,16 @@
         <v>75</v>
       </c>
       <c r="K1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="M1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="O1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="Q1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.3">
@@ -1790,16 +1955,16 @@
         <v>76</v>
       </c>
       <c r="K2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="M2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="O2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="Q2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.3">
@@ -1813,16 +1978,16 @@
         <v>69</v>
       </c>
       <c r="K3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="M3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="O3" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="Q3" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.3">
@@ -1836,16 +2001,16 @@
         <v>70</v>
       </c>
       <c r="I4" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="K4" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="O4" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q4" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.3">
@@ -1853,16 +2018,16 @@
         <v>29</v>
       </c>
       <c r="I5" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="K5" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="O5" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="Q5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.3">
@@ -1870,10 +2035,10 @@
         <v>30</v>
       </c>
       <c r="K6" t="s">
+        <v>183</v>
+      </c>
+      <c r="Q6" t="s">
         <v>182</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.3">
@@ -1881,16 +2046,16 @@
         <v>31</v>
       </c>
       <c r="C7" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I7" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="K7" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="Q7" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.3">
@@ -1898,13 +2063,13 @@
         <v>32</v>
       </c>
       <c r="C8" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I8" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="K8" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.3">
@@ -1912,10 +2077,10 @@
         <v>33</v>
       </c>
       <c r="C9" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="K9" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.3">
@@ -1923,10 +2088,10 @@
         <v>71</v>
       </c>
       <c r="C10" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="K10" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.3">
@@ -1934,7 +2099,7 @@
         <v>72</v>
       </c>
       <c r="C11" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.3">
@@ -1942,7 +2107,7 @@
         <v>73</v>
       </c>
       <c r="C12" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.3">
@@ -1950,7 +2115,7 @@
         <v>69</v>
       </c>
       <c r="C13" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.3">
@@ -1958,7 +2123,7 @@
         <v>74</v>
       </c>
       <c r="C14" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.3">
@@ -1966,7 +2131,7 @@
         <v>34</v>
       </c>
       <c r="C15" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.3">
@@ -1976,17 +2141,17 @@
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
   </sheetData>
@@ -2046,7 +2211,7 @@
         <v>28</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E2" s="24">
         <v>260</v>
@@ -2072,7 +2237,7 @@
         <v>9</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E3" s="25">
         <v>40</v>
@@ -2098,7 +2263,7 @@
         <v>9</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E4" s="24">
         <v>200</v>
@@ -2124,7 +2289,7 @@
         <v>28</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E5" s="25">
         <v>60</v>
@@ -3118,342 +3283,46 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25FB69CB-2FB6-48CF-B292-D5EA7E2EAA09}">
-  <dimension ref="A1:B31"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B82E164A-0D11-4427-AF36-BC223AAE005B}">
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.21875" style="31" customWidth="1"/>
+    <col min="3" max="3" width="15.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="B5" s="5">
-        <v>22000</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="B6" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="B7" s="6">
-        <f>B5+B6</f>
-        <v>22000</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B8" s="7"/>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B9" s="7"/>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="B10" s="7"/>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B11" s="7"/>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B12" s="6">
-        <f>SUM(Transactions!$E$2:$E$100)</f>
-        <v>560</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B13" s="6">
-        <f>SUMIF(Transactions!$F$2:$F$100,"Need",Transactions!$E$2:$E$100)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B14" s="6">
-        <f>SUMIF(Transactions!$F$2:$F$100,"Want",Transactions!$E$2:$E$100)</f>
-        <v>260</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B15" s="6">
-        <f>SUMIF(Transactions!$C$2:$C$100,"Food",Transactions!$E$2:$E$100)</f>
-        <v>320</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B16" s="6">
-        <f>SUMIF(Transactions!$C$2:$C$100,"Travel",Transactions!$E$2:$E$100)</f>
-        <v>240</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B17" s="7"/>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B18" s="7"/>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A19" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="B19" s="7"/>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B20" s="7"/>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A21" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B21" s="6">
-        <f>B7-B12</f>
-        <v>21440</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A22" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B22" s="1">
-        <f>B21/B7%</f>
-        <v>97.454545454545453</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A23" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="B23" s="1" t="str">
-        <f>IF(B21&gt;=5000,"🟢 Excellent",IF(B21&gt;=0,"🟡 Stable","🔴 Risk"))</f>
-        <v>🟢 Excellent</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A24" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="B24" s="1" t="str">
-        <f>IF(B21&gt;=0,"✅ On Track","⚠️ Overspending")</f>
-        <v>✅ On Track</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>205</v>
-      </c>
-      <c r="B27" s="17">
-        <f>SUM(FinancialCommitments[Remaining])</f>
-        <v>11000</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>206</v>
-      </c>
-      <c r="B29" s="18">
-        <f>1-(SUM(FinancialCommitments[Remaining])/SUM(FinancialCommitments[Amount]))</f>
-        <v>0.15384615384615385</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>207</v>
-      </c>
-      <c r="B31" s="7">
-        <f>B21-B27</f>
-        <v>10440</v>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="31" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C1" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="31">
+        <v>7</v>
+      </c>
+      <c r="B2">
+        <v>2026</v>
+      </c>
+      <c r="C2">
+        <v>8000</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F24486AA-4411-496D-83B5-A5D6BB792B45}">
-  <dimension ref="A1:B24"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B1" s="8">
-        <v>46174</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>60</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{783F04F9-B9B3-40A0-AFB4-B858E144E097}">
-  <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>163</v>
-      </c>
-      <c r="B1" t="s">
-        <v>164</v>
-      </c>
-      <c r="C1" t="s">
-        <v>165</v>
-      </c>
-      <c r="D1" t="s">
-        <v>166</v>
-      </c>
-      <c r="E1" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>176</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED4B5016-8080-45D9-A027-E465FB36B2D6}">
   <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3467,10 +3336,10 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="30" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C1" t="s">
         <v>66</v>
@@ -3479,16 +3348,16 @@
         <v>2</v>
       </c>
       <c r="E1" s="22" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F1" s="22" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="G1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="H1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I1" t="s">
         <v>57</v>
@@ -3499,10 +3368,10 @@
         <v>46204</v>
       </c>
       <c r="B2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D2" s="22">
         <v>10000</v>
@@ -3514,13 +3383,13 @@
         <v>10000</v>
       </c>
       <c r="G2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="H2" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="I2" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
@@ -3528,10 +3397,10 @@
         <v>46206</v>
       </c>
       <c r="B3" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C3" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D3" s="22">
         <v>2000</v>
@@ -3546,10 +3415,10 @@
         <v>46249</v>
       </c>
       <c r="H3" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="I3" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -3557,10 +3426,10 @@
         <v>46208</v>
       </c>
       <c r="B4" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C4" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D4" s="22">
         <v>1000</v>
@@ -3575,10 +3444,10 @@
         <v>46209</v>
       </c>
       <c r="H4" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="I4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
   </sheetData>
@@ -3597,7 +3466,343 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25FB69CB-2FB6-48CF-B292-D5EA7E2EAA09}">
+  <dimension ref="A1:B31"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="11.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B5" s="5">
+        <v>22000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B6" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" s="6">
+        <f>B5+B6</f>
+        <v>22000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B8" s="7"/>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B9" s="7"/>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B10" s="7"/>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B11" s="7"/>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="6">
+        <f>SUM(Transactions!$E$2:$E$100)</f>
+        <v>560</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B13" s="6">
+        <f>SUMIF(Transactions!$F$2:$F$100,"Need",Transactions!$E$2:$E$100)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" s="6">
+        <f>SUMIF(Transactions!$F$2:$F$100,"Want",Transactions!$E$2:$E$100)</f>
+        <v>260</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B15" s="6">
+        <f>SUMIF(Transactions!$C$2:$C$100,"Food",Transactions!$E$2:$E$100)</f>
+        <v>320</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B16" s="6">
+        <f>SUMIF(Transactions!$C$2:$C$100,"Travel",Transactions!$E$2:$E$100)</f>
+        <v>240</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B17" s="7"/>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B18" s="7"/>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B19" s="7"/>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B20" s="7"/>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B21" s="6">
+        <f>B7-B12</f>
+        <v>21440</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B22" s="1">
+        <f>B21/B7%</f>
+        <v>97.454545454545453</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B23" s="1" t="str">
+        <f>IF(B21&gt;=5000,"🟢 Excellent",IF(B21&gt;=0,"🟡 Stable","🔴 Risk"))</f>
+        <v>🟢 Excellent</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B24" s="1" t="str">
+        <f>IF(B21&gt;=0,"✅ On Track","⚠️ Overspending")</f>
+        <v>✅ On Track</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>206</v>
+      </c>
+      <c r="B27" s="17">
+        <f>SUM(FinancialCommitments[Remaining])</f>
+        <v>11000</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>207</v>
+      </c>
+      <c r="B29" s="18">
+        <f>1-(SUM(FinancialCommitments[Remaining])/SUM(FinancialCommitments[Amount]))</f>
+        <v>0.15384615384615385</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>208</v>
+      </c>
+      <c r="B31" s="7">
+        <f>B21-B27</f>
+        <v>10440</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F24486AA-4411-496D-83B5-A5D6BB792B45}">
+  <dimension ref="A1:B24"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" s="8">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>60</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{783F04F9-B9B3-40A0-AFB4-B858E144E097}">
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>164</v>
+      </c>
+      <c r="B1" t="s">
+        <v>165</v>
+      </c>
+      <c r="C1" t="s">
+        <v>166</v>
+      </c>
+      <c r="D1" t="s">
+        <v>167</v>
+      </c>
+      <c r="E1" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>177</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8C2D160-B4CC-4D85-A856-F7EE7CF0468E}">
   <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3611,7 +3816,7 @@
         <v>27</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>24</v>
@@ -3620,7 +3825,7 @@
         <v>2</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F1" s="4" t="s">
         <v>77</v>
@@ -3634,22 +3839,22 @@
         <v>46204</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D2" s="20">
         <v>22000</v>
       </c>
       <c r="E2" s="19" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F2" s="19" t="s">
         <v>75</v>
       </c>
       <c r="G2" s="19" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3657,22 +3862,22 @@
         <v>46218</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C3" s="19" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D3" s="20">
         <v>5000</v>
       </c>
       <c r="E3" s="19" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F3" s="19" t="s">
         <v>76</v>
       </c>
       <c r="G3" s="19" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -3680,22 +3885,22 @@
         <v>46223</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D4" s="20">
         <v>2000</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F4" s="19" t="s">
         <v>76</v>
       </c>
       <c r="G4" s="19" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
   </sheetData>
@@ -3717,28 +3922,28 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C985A9ED-FFB7-41B9-BD81-D99D84E9A097}">
   <dimension ref="A1:J35"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
@@ -3747,40 +3952,40 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B5" s="1">
         <v>24</v>
       </c>
       <c r="J5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J7" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
@@ -3791,12 +3996,12 @@
         <v>8600</v>
       </c>
       <c r="J9" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B10" s="15">
         <v>0</v>
@@ -3804,35 +4009,35 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="J11" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J13" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J15" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
@@ -3840,16 +4045,16 @@
         <v>13</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D16" s="1">
         <v>22000</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
@@ -3857,19 +4062,19 @@
         <v>14</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D17" s="1">
         <v>23000</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="J17" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
@@ -3877,232 +4082,96 @@
         <v>15</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D18" s="1">
         <v>28000</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="J19" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="J21" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="J23" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="J25" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="J27" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="J29" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="J31" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="33" spans="10:10" x14ac:dyDescent="0.3">
       <c r="J33" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="35" spans="10:10" x14ac:dyDescent="0.3">
       <c r="J35" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{062E0065-A33A-40A3-8681-B93160D6FE12}">
-  <dimension ref="A1:Q5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="10.77734375" customWidth="1"/>
-    <col min="4" max="4" width="13.6640625" customWidth="1"/>
-    <col min="5" max="5" width="14.77734375" customWidth="1"/>
-    <col min="7" max="7" width="11.33203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>124</v>
-      </c>
-      <c r="B1" t="s">
-        <v>125</v>
-      </c>
-      <c r="C1" t="s">
-        <v>126</v>
-      </c>
-      <c r="D1" t="s">
-        <v>127</v>
-      </c>
-      <c r="E1" t="s">
-        <v>128</v>
-      </c>
-      <c r="F1" t="s">
-        <v>129</v>
-      </c>
-      <c r="G1" t="s">
-        <v>177</v>
-      </c>
-      <c r="H1" t="s">
-        <v>130</v>
-      </c>
-      <c r="I1" t="s">
-        <v>178</v>
-      </c>
-      <c r="J1" t="s">
-        <v>57</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" t="s">
-        <v>141</v>
-      </c>
-      <c r="C2">
-        <v>22000</v>
-      </c>
-      <c r="F2" t="s">
-        <v>131</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" t="s">
-        <v>142</v>
-      </c>
-      <c r="C3">
-        <v>23000</v>
-      </c>
-      <c r="F3" t="s">
-        <v>131</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" t="s">
-        <v>143</v>
-      </c>
-      <c r="C4">
-        <v>28000</v>
-      </c>
-      <c r="F4" t="s">
-        <v>131</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>144</v>
-      </c>
-      <c r="B5" t="s">
-        <v>145</v>
-      </c>
-      <c r="C5">
-        <v>20000</v>
-      </c>
-      <c r="F5" t="s">
-        <v>131</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>149</v>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F50" xr:uid="{B7B46CB3-D4D6-4415-A547-30F33809F18A}">
-      <formula1>AppliedStatus</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H50" xr:uid="{A0AB4D2E-03DC-499E-A809-B6BDCD0E9591}">
-      <formula1>InterviewResult</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G1:G1048576" xr:uid="{DAD8A552-FAB1-4D16-90F0-ACE3B457489B}">
-      <formula1>InterviewRound</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I1:I1048576" xr:uid="{F32AF372-FB7D-40CA-8785-F217A85AC485}">
-      <formula1>NextAction</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
v0.9.1 add Savings Engine with financial savings metrics
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pratham OS\Development\Finance-AI\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0E21683-B879-4BDB-8E6F-21B29DB494F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C91D089-7722-4E67-AA6A-80600EC69375}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="2" xr2:uid="{D6DE1A26-0963-4585-A363-547897EAF3B2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="3" xr2:uid="{D6DE1A26-0963-4585-A363-547897EAF3B2}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan" sheetId="1" r:id="rId1"/>
@@ -911,7 +911,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -945,28 +945,18 @@
     <xf numFmtId="164" fontId="0" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="2" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="2" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="20">
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1041,7 +1031,13 @@
       <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
     </dxf>
     <dxf>
       <border outline="0">
@@ -1074,6 +1070,9 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1088,14 +1087,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{42D67FA3-A40A-4607-BCB9-468A9ECB0007}" name="Table1" displayName="Table1" ref="A1:H1048576" totalsRowShown="0" headerRowDxfId="19" tableBorderDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{42D67FA3-A40A-4607-BCB9-468A9ECB0007}" name="Table1" displayName="Table1" ref="A1:H1048576" totalsRowShown="0" headerRowDxfId="18" tableBorderDxfId="17">
   <autoFilter ref="A1:H1048576" xr:uid="{42D67FA3-A40A-4607-BCB9-468A9ECB0007}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{1D37F906-33D7-46E6-8270-56D5EEA80EC7}" name="Date" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{1D37F906-33D7-46E6-8270-56D5EEA80EC7}" name="Date" dataDxfId="16"/>
     <tableColumn id="4" xr3:uid="{E805A8A8-660D-4099-912A-BE1B697553ED}" name="Type"/>
     <tableColumn id="5" xr3:uid="{ABF1E4D7-7922-479D-94F4-994DCBA1062D}" name="Category"/>
     <tableColumn id="6" xr3:uid="{E21EA904-BC60-4EB5-B4BD-249E5A12FC76}" name="Description "/>
-    <tableColumn id="7" xr3:uid="{EFA172CE-B81A-4A83-BB09-0C52BED62422}" name="Amount" dataDxfId="17"/>
+    <tableColumn id="7" xr3:uid="{EFA172CE-B81A-4A83-BB09-0C52BED62422}" name="Amount" dataDxfId="15"/>
     <tableColumn id="8" xr3:uid="{E811D3EB-DAD5-46D9-B70D-01072B332F5C}" name="Need/Want"/>
     <tableColumn id="9" xr3:uid="{1E8766C9-2C6F-4CE3-9C7E-C6C8545D3945}" name="Payment Mode"/>
     <tableColumn id="10" xr3:uid="{BA26CD78-BAFB-4644-808D-0A18546F6CAF}" name="Recurring"/>
@@ -1108,7 +1107,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{204CD917-42D7-44E9-889E-B87F7E170616}" name="Table5" displayName="Table5" ref="A1:C100" totalsRowShown="0">
   <autoFilter ref="A1:C100" xr:uid="{204CD917-42D7-44E9-889E-B87F7E170616}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{CCD99EA9-9CA0-4F69-8282-1EE2E5FE7967}" name="Month" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{CCD99EA9-9CA0-4F69-8282-1EE2E5FE7967}" name="Month" dataDxfId="19"/>
     <tableColumn id="2" xr3:uid="{5C307EC1-8BAE-4B8C-AF42-D468202B7A5E}" name="Year"/>
     <tableColumn id="3" xr3:uid="{2B3569FD-9348-4E00-BFEA-53DF4F58E82C}" name="Monthly_Budget"/>
   </tableColumns>
@@ -1120,12 +1119,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{1AFBBFA5-5EA2-4DA5-91C7-5EE90985F084}" name="FinancialCommitments" displayName="FinancialCommitments" ref="A1:I50" totalsRowShown="0">
   <autoFilter ref="A1:I50" xr:uid="{1AFBBFA5-5EA2-4DA5-91C7-5EE90985F084}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{C10697DD-F282-4D7F-A12A-9BFC6193DC4E}" name="Date " dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{C10697DD-F282-4D7F-A12A-9BFC6193DC4E}" name="Date " dataDxfId="14"/>
     <tableColumn id="2" xr3:uid="{D6130D6E-B2EE-4D09-94CD-7E8053CD1C7B}" name="From"/>
     <tableColumn id="3" xr3:uid="{8ECD20EB-BEF0-47D5-8DA5-28D491EC7B0A}" name="Type"/>
-    <tableColumn id="4" xr3:uid="{87D047F3-8B64-4D30-ACC0-42FFF26FEC3E}" name="Amount" dataDxfId="16"/>
-    <tableColumn id="5" xr3:uid="{C982624C-E448-4958-A5CE-7D794FC142FA}" name="Repaid" dataDxfId="15"/>
-    <tableColumn id="6" xr3:uid="{665D5056-3744-4E56-95C7-F0943FD35707}" name="Remaining" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{87D047F3-8B64-4D30-ACC0-42FFF26FEC3E}" name="Amount" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{C982624C-E448-4958-A5CE-7D794FC142FA}" name="Repaid" dataDxfId="12"/>
+    <tableColumn id="6" xr3:uid="{665D5056-3744-4E56-95C7-F0943FD35707}" name="Remaining" dataDxfId="11"/>
     <tableColumn id="7" xr3:uid="{FFDA91C5-2668-4023-9FEE-465A59D85270}" name="Due Date"/>
     <tableColumn id="8" xr3:uid="{748EB09B-78B0-49AB-AC7E-88A7F4C42C89}" name="Status"/>
     <tableColumn id="9" xr3:uid="{9F5FA8E8-540D-4C48-B339-C097673FD287}" name="Notes"/>
@@ -1135,16 +1134,16 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{7C5D4057-F5F1-485E-AE6E-34A855BB81C8}" name="IncomeTable" displayName="IncomeTable" ref="A1:G4" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{7C5D4057-F5F1-485E-AE6E-34A855BB81C8}" name="IncomeTable" displayName="IncomeTable" ref="A1:G4" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
   <autoFilter ref="A1:G4" xr:uid="{7C5D4057-F5F1-485E-AE6E-34A855BB81C8}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{85417279-B333-4129-826F-4B13A464B0A1}" name="Date" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{72151722-7F6E-43AF-AADF-05A0452D151E}" name="Source" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{A9F1D760-964B-4BC4-876E-FE2B218C85B6}" name="Category" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{31C0BCAE-AC93-4345-9B1C-546CE0735A6B}" name="Amount" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{C6E99480-C881-404B-8F25-E2549BD2CCCD}" name="Status" dataDxfId="7"/>
-    <tableColumn id="7" xr3:uid="{29AC2CCC-8D50-4D4F-9049-D5CBB08CDAB6}" name="Recurring" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{4D5A0A55-4298-4332-9A93-683CDAE35676}" name="Notes" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{85417279-B333-4129-826F-4B13A464B0A1}" name="Date" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{72151722-7F6E-43AF-AADF-05A0452D151E}" name="Source" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{A9F1D760-964B-4BC4-876E-FE2B218C85B6}" name="Category" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{31C0BCAE-AC93-4345-9B1C-546CE0735A6B}" name="Amount" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{C6E99480-C881-404B-8F25-E2549BD2CCCD}" name="Status" dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{29AC2CCC-8D50-4D4F-9049-D5CBB08CDAB6}" name="Recurring" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{4D5A0A55-4298-4332-9A93-683CDAE35676}" name="Notes" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1490,12 +1489,12 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -1679,10 +1678,10 @@
     <mergeCell ref="A1:D1"/>
   </mergeCells>
   <conditionalFormatting sqref="B17:B20">
-    <cfRule type="cellIs" dxfId="4" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2164,7 +2163,7 @@
   <dimension ref="A1:H100"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.6640625" style="30" customWidth="1"/>
+    <col min="1" max="1" width="19.6640625" style="29" customWidth="1"/>
     <col min="2" max="2" width="9.5546875" customWidth="1"/>
     <col min="3" max="3" width="10.21875" customWidth="1"/>
     <col min="4" max="4" width="12.88671875" customWidth="1"/>
@@ -2175,7 +2174,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="27" t="s">
         <v>27</v>
       </c>
       <c r="B1" s="14" t="s">
@@ -3245,7 +3244,7 @@
       <c r="H99" s="13"/>
     </row>
     <row r="100" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A100" s="29"/>
+      <c r="A100" s="28"/>
       <c r="B100" s="9"/>
       <c r="C100" s="9"/>
       <c r="D100" s="9"/>
@@ -3287,12 +3286,12 @@
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.21875" style="31" customWidth="1"/>
+    <col min="1" max="1" width="15.21875" customWidth="1"/>
     <col min="3" max="3" width="15.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="31" t="s">
+      <c r="A1" t="s">
         <v>52</v>
       </c>
       <c r="B1" t="s">
@@ -3303,7 +3302,7 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="31">
+      <c r="A2">
         <v>7</v>
       </c>
       <c r="B2">
@@ -3327,7 +3326,7 @@
   <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.44140625" style="30" customWidth="1"/>
+    <col min="1" max="1" width="12.44140625" style="29" customWidth="1"/>
     <col min="4" max="4" width="13" style="22" customWidth="1"/>
     <col min="5" max="5" width="9.44140625" style="22" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.6640625" style="22" customWidth="1"/>
@@ -3335,7 +3334,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="29" t="s">
         <v>192</v>
       </c>
       <c r="B1" t="s">
@@ -3364,7 +3363,7 @@
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="30">
+      <c r="A2" s="29">
         <v>46204</v>
       </c>
       <c r="B2" t="s">
@@ -3393,7 +3392,7 @@
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="30">
+      <c r="A3" s="29">
         <v>46206</v>
       </c>
       <c r="B3" t="s">
@@ -3422,7 +3421,7 @@
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="30">
+      <c r="A4" s="29">
         <v>46208</v>
       </c>
       <c r="B4" t="s">

</xml_diff>

<commit_message>
v0.9.2 add Emergency Fund Engine and monthly commitment tracking
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pratham OS\Development\Finance-AI\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C91D089-7722-4E67-AA6A-80600EC69375}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{730C3D7B-58C4-4F50-8D32-14C92560ECA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="3" xr2:uid="{D6DE1A26-0963-4585-A363-547897EAF3B2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="855" firstSheet="3" activeTab="3" xr2:uid="{D6DE1A26-0963-4585-A363-547897EAF3B2}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
     <definedName name="IncomeStatus">Lists!$I$4:$I$5</definedName>
     <definedName name="InterviewResult">Lists!$M$1:$M$3</definedName>
     <definedName name="InterviewRound">Lists!$O$1:$O$5</definedName>
-    <definedName name="LoanType">Lists!$A$17:$A$19</definedName>
+    <definedName name="LoanType">Lists!$A$18:$A$23</definedName>
     <definedName name="NeedWant">Lists!$C$1:$C$2</definedName>
     <definedName name="NextAction">Lists!$Q$1:$Q$7</definedName>
     <definedName name="PaymentMode">Lists!$E$1:$E$4</definedName>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="231">
   <si>
     <t>August Financial Plan</t>
   </si>
@@ -643,9 +643,6 @@
     <t>Joined</t>
   </si>
   <si>
-    <t xml:space="preserve">Date </t>
-  </si>
-  <si>
     <t>From</t>
   </si>
   <si>
@@ -658,30 +655,18 @@
     <t>Due Date</t>
   </si>
   <si>
-    <t>Mummy</t>
-  </si>
-  <si>
     <t>Family Loan</t>
   </si>
   <si>
-    <t xml:space="preserve">Flexible </t>
-  </si>
-  <si>
     <t>Active</t>
   </si>
   <si>
-    <t>Survival</t>
-  </si>
-  <si>
     <t>Vivek</t>
   </si>
   <si>
     <t>Friend Loan</t>
   </si>
   <si>
-    <t>Job Search</t>
-  </si>
-  <si>
     <t>Credit Card</t>
   </si>
   <si>
@@ -739,9 +724,6 @@
     <t>Paid</t>
   </si>
   <si>
-    <t>Raj</t>
-  </si>
-  <si>
     <t>rapido</t>
   </si>
   <si>
@@ -749,6 +731,33 @@
   </si>
   <si>
     <t>Monthly_Budget</t>
+  </si>
+  <si>
+    <t>commitment</t>
+  </si>
+  <si>
+    <t>Fixed Expense</t>
+  </si>
+  <si>
+    <t>Loan</t>
+  </si>
+  <si>
+    <t>Total Amount</t>
+  </si>
+  <si>
+    <t>Monthly Payment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Start Date </t>
+  </si>
+  <si>
+    <t>End Date</t>
+  </si>
+  <si>
+    <t>Bajaj (Chacha Ji)</t>
+  </si>
+  <si>
+    <t>Laptop EMI</t>
   </si>
 </sst>
 </file>
@@ -911,7 +920,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -928,7 +937,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="6" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -956,7 +964,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="20">
+  <dxfs count="22">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -976,6 +984,24 @@
           <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1022,16 +1048,7 @@
       </font>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
@@ -1070,9 +1087,6 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1087,14 +1101,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{42D67FA3-A40A-4607-BCB9-468A9ECB0007}" name="Table1" displayName="Table1" ref="A1:H1048576" totalsRowShown="0" headerRowDxfId="18" tableBorderDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{42D67FA3-A40A-4607-BCB9-468A9ECB0007}" name="Table1" displayName="Table1" ref="A1:H1048576" totalsRowShown="0" headerRowDxfId="21" tableBorderDxfId="20">
   <autoFilter ref="A1:H1048576" xr:uid="{42D67FA3-A40A-4607-BCB9-468A9ECB0007}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{1D37F906-33D7-46E6-8270-56D5EEA80EC7}" name="Date" dataDxfId="16"/>
+    <tableColumn id="1" xr3:uid="{1D37F906-33D7-46E6-8270-56D5EEA80EC7}" name="Date" dataDxfId="19"/>
     <tableColumn id="4" xr3:uid="{E805A8A8-660D-4099-912A-BE1B697553ED}" name="Type"/>
     <tableColumn id="5" xr3:uid="{ABF1E4D7-7922-479D-94F4-994DCBA1062D}" name="Category"/>
     <tableColumn id="6" xr3:uid="{E21EA904-BC60-4EB5-B4BD-249E5A12FC76}" name="Description "/>
-    <tableColumn id="7" xr3:uid="{EFA172CE-B81A-4A83-BB09-0C52BED62422}" name="Amount" dataDxfId="15"/>
+    <tableColumn id="7" xr3:uid="{EFA172CE-B81A-4A83-BB09-0C52BED62422}" name="Amount" dataDxfId="18"/>
     <tableColumn id="8" xr3:uid="{E811D3EB-DAD5-46D9-B70D-01072B332F5C}" name="Need/Want"/>
     <tableColumn id="9" xr3:uid="{1E8766C9-2C6F-4CE3-9C7E-C6C8545D3945}" name="Payment Mode"/>
     <tableColumn id="10" xr3:uid="{BA26CD78-BAFB-4644-808D-0A18546F6CAF}" name="Recurring"/>
@@ -1107,7 +1121,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{204CD917-42D7-44E9-889E-B87F7E170616}" name="Table5" displayName="Table5" ref="A1:C100" totalsRowShown="0">
   <autoFilter ref="A1:C100" xr:uid="{204CD917-42D7-44E9-889E-B87F7E170616}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{CCD99EA9-9CA0-4F69-8282-1EE2E5FE7967}" name="Month" dataDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{CCD99EA9-9CA0-4F69-8282-1EE2E5FE7967}" name="Month" dataDxfId="17"/>
     <tableColumn id="2" xr3:uid="{5C307EC1-8BAE-4B8C-AF42-D468202B7A5E}" name="Year"/>
     <tableColumn id="3" xr3:uid="{2B3569FD-9348-4E00-BFEA-53DF4F58E82C}" name="Monthly_Budget"/>
   </tableColumns>
@@ -1116,34 +1130,36 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{1AFBBFA5-5EA2-4DA5-91C7-5EE90985F084}" name="FinancialCommitments" displayName="FinancialCommitments" ref="A1:I50" totalsRowShown="0">
-  <autoFilter ref="A1:I50" xr:uid="{1AFBBFA5-5EA2-4DA5-91C7-5EE90985F084}"/>
-  <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{C10697DD-F282-4D7F-A12A-9BFC6193DC4E}" name="Date " dataDxfId="14"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{1AFBBFA5-5EA2-4DA5-91C7-5EE90985F084}" name="FinancialCommitments" displayName="FinancialCommitments" ref="A1:K46" totalsRowShown="0">
+  <autoFilter ref="A1:K46" xr:uid="{1AFBBFA5-5EA2-4DA5-91C7-5EE90985F084}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{C10697DD-F282-4D7F-A12A-9BFC6193DC4E}" name="Start Date " dataDxfId="7"/>
     <tableColumn id="2" xr3:uid="{D6130D6E-B2EE-4D09-94CD-7E8053CD1C7B}" name="From"/>
     <tableColumn id="3" xr3:uid="{8ECD20EB-BEF0-47D5-8DA5-28D491EC7B0A}" name="Type"/>
-    <tableColumn id="4" xr3:uid="{87D047F3-8B64-4D30-ACC0-42FFF26FEC3E}" name="Amount" dataDxfId="13"/>
-    <tableColumn id="5" xr3:uid="{C982624C-E448-4958-A5CE-7D794FC142FA}" name="Repaid" dataDxfId="12"/>
-    <tableColumn id="6" xr3:uid="{665D5056-3744-4E56-95C7-F0943FD35707}" name="Remaining" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{87D047F3-8B64-4D30-ACC0-42FFF26FEC3E}" name="Total Amount" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{C982624C-E448-4958-A5CE-7D794FC142FA}" name="Repaid" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{665D5056-3744-4E56-95C7-F0943FD35707}" name="Remaining" dataDxfId="4"/>
     <tableColumn id="7" xr3:uid="{FFDA91C5-2668-4023-9FEE-465A59D85270}" name="Due Date"/>
     <tableColumn id="8" xr3:uid="{748EB09B-78B0-49AB-AC7E-88A7F4C42C89}" name="Status"/>
-    <tableColumn id="9" xr3:uid="{9F5FA8E8-540D-4C48-B339-C097673FD287}" name="Notes"/>
+    <tableColumn id="10" xr3:uid="{39DD9F5E-EB31-47B4-A27F-BDA3AA61DA00}" name="commitment"/>
+    <tableColumn id="11" xr3:uid="{740721D4-21BC-47E8-A178-052DE413178D}" name="Monthly Payment" dataDxfId="2"/>
+    <tableColumn id="12" xr3:uid="{2EEE087F-37EF-44B3-8405-6F6CCBE4BDEB}" name="End Date" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{7C5D4057-F5F1-485E-AE6E-34A855BB81C8}" name="IncomeTable" displayName="IncomeTable" ref="A1:G4" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{7C5D4057-F5F1-485E-AE6E-34A855BB81C8}" name="IncomeTable" displayName="IncomeTable" ref="A1:G4" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
   <autoFilter ref="A1:G4" xr:uid="{7C5D4057-F5F1-485E-AE6E-34A855BB81C8}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{85417279-B333-4129-826F-4B13A464B0A1}" name="Date" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{72151722-7F6E-43AF-AADF-05A0452D151E}" name="Source" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{A9F1D760-964B-4BC4-876E-FE2B218C85B6}" name="Category" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{31C0BCAE-AC93-4345-9B1C-546CE0735A6B}" name="Amount" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{C6E99480-C881-404B-8F25-E2549BD2CCCD}" name="Status" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{29AC2CCC-8D50-4D4F-9049-D5CBB08CDAB6}" name="Recurring" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{4D5A0A55-4298-4332-9A93-683CDAE35676}" name="Notes" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{85417279-B333-4129-826F-4B13A464B0A1}" name="Date" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{72151722-7F6E-43AF-AADF-05A0452D151E}" name="Source" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{A9F1D760-964B-4BC4-876E-FE2B218C85B6}" name="Category" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{31C0BCAE-AC93-4345-9B1C-546CE0735A6B}" name="Amount" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{C6E99480-C881-404B-8F25-E2549BD2CCCD}" name="Status" dataDxfId="10"/>
+    <tableColumn id="7" xr3:uid="{29AC2CCC-8D50-4D4F-9049-D5CBB08CDAB6}" name="Recurring" dataDxfId="9"/>
+    <tableColumn id="6" xr3:uid="{4D5A0A55-4298-4332-9A93-683CDAE35676}" name="Notes" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1489,12 +1505,12 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -1905,7 +1921,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{729B4158-2DD5-48A6-9BEC-2F739409F312}">
-  <dimension ref="A1:Q19"/>
+  <dimension ref="A1:Q23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.3">
@@ -2000,7 +2016,7 @@
         <v>70</v>
       </c>
       <c r="I4" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="K4" t="s">
         <v>135</v>
@@ -2045,10 +2061,10 @@
         <v>31</v>
       </c>
       <c r="C7" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="I7" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="K7" t="s">
         <v>138</v>
@@ -2065,7 +2081,7 @@
         <v>96</v>
       </c>
       <c r="I8" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="K8" t="s">
         <v>137</v>
@@ -2076,7 +2092,7 @@
         <v>33</v>
       </c>
       <c r="C9" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="K9" t="s">
         <v>139</v>
@@ -2087,7 +2103,7 @@
         <v>71</v>
       </c>
       <c r="C10" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="K10" t="s">
         <v>140</v>
@@ -2098,7 +2114,7 @@
         <v>72</v>
       </c>
       <c r="C11" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.3">
@@ -2106,7 +2122,7 @@
         <v>73</v>
       </c>
       <c r="C12" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.3">
@@ -2114,7 +2130,7 @@
         <v>69</v>
       </c>
       <c r="C13" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.3">
@@ -2122,7 +2138,7 @@
         <v>74</v>
       </c>
       <c r="C14" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.3">
@@ -2130,7 +2146,7 @@
         <v>34</v>
       </c>
       <c r="C15" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.3">
@@ -2138,19 +2154,34 @@
         <v>34</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>198</v>
-      </c>
-    </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>205</v>
+        <v>199</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>224</v>
       </c>
     </row>
   </sheetData>
@@ -2163,18 +2194,18 @@
   <dimension ref="A1:H100"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.6640625" style="29" customWidth="1"/>
+    <col min="1" max="1" width="19.6640625" style="28" customWidth="1"/>
     <col min="2" max="2" width="9.5546875" customWidth="1"/>
     <col min="3" max="3" width="10.21875" customWidth="1"/>
     <col min="4" max="4" width="12.88671875" customWidth="1"/>
-    <col min="5" max="5" width="9.33203125" style="22" customWidth="1"/>
+    <col min="5" max="5" width="9.33203125" style="21" customWidth="1"/>
     <col min="6" max="6" width="12.33203125" customWidth="1"/>
     <col min="7" max="7" width="15.109375" customWidth="1"/>
     <col min="8" max="8" width="10.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="26" t="s">
         <v>27</v>
       </c>
       <c r="B1" s="14" t="s">
@@ -2186,7 +2217,7 @@
       <c r="D1" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="E1" s="23" t="s">
+      <c r="E1" s="22" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="14" t="s">
@@ -2210,9 +2241,9 @@
         <v>28</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>222</v>
-      </c>
-      <c r="E2" s="24">
+        <v>217</v>
+      </c>
+      <c r="E2" s="23">
         <v>260</v>
       </c>
       <c r="F2" s="11" t="s">
@@ -2236,9 +2267,9 @@
         <v>9</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>225</v>
-      </c>
-      <c r="E3" s="25">
+        <v>219</v>
+      </c>
+      <c r="E3" s="24">
         <v>40</v>
       </c>
       <c r="F3" s="13" t="s">
@@ -2262,9 +2293,9 @@
         <v>9</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>225</v>
-      </c>
-      <c r="E4" s="24">
+        <v>219</v>
+      </c>
+      <c r="E4" s="23">
         <v>200</v>
       </c>
       <c r="F4" s="11" t="s">
@@ -2288,9 +2319,9 @@
         <v>28</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>226</v>
-      </c>
-      <c r="E5" s="25">
+        <v>220</v>
+      </c>
+      <c r="E5" s="24">
         <v>60</v>
       </c>
       <c r="F5" s="13" t="s">
@@ -2308,7 +2339,7 @@
       <c r="B6" s="11"/>
       <c r="C6" s="11"/>
       <c r="D6" s="11"/>
-      <c r="E6" s="24"/>
+      <c r="E6" s="23"/>
       <c r="F6" s="11"/>
       <c r="G6" s="11"/>
       <c r="H6" s="11"/>
@@ -2318,7 +2349,7 @@
       <c r="B7" s="13"/>
       <c r="C7" s="13"/>
       <c r="D7" s="13"/>
-      <c r="E7" s="25"/>
+      <c r="E7" s="24"/>
       <c r="F7" s="13"/>
       <c r="G7" s="13"/>
       <c r="H7" s="13"/>
@@ -2328,7 +2359,7 @@
       <c r="B8" s="11"/>
       <c r="C8" s="11"/>
       <c r="D8" s="11"/>
-      <c r="E8" s="24"/>
+      <c r="E8" s="23"/>
       <c r="F8" s="11"/>
       <c r="G8" s="11"/>
       <c r="H8" s="11"/>
@@ -2338,7 +2369,7 @@
       <c r="B9" s="13"/>
       <c r="C9" s="13"/>
       <c r="D9" s="13"/>
-      <c r="E9" s="25"/>
+      <c r="E9" s="24"/>
       <c r="F9" s="13"/>
       <c r="G9" s="13"/>
       <c r="H9" s="13"/>
@@ -2348,7 +2379,7 @@
       <c r="B10" s="11"/>
       <c r="C10" s="11"/>
       <c r="D10" s="11"/>
-      <c r="E10" s="24"/>
+      <c r="E10" s="23"/>
       <c r="F10" s="11"/>
       <c r="G10" s="11"/>
       <c r="H10" s="11"/>
@@ -2358,7 +2389,7 @@
       <c r="B11" s="13"/>
       <c r="C11" s="13"/>
       <c r="D11" s="13"/>
-      <c r="E11" s="25"/>
+      <c r="E11" s="24"/>
       <c r="F11" s="13"/>
       <c r="G11" s="13"/>
       <c r="H11" s="13"/>
@@ -2368,7 +2399,7 @@
       <c r="B12" s="11"/>
       <c r="C12" s="11"/>
       <c r="D12" s="11"/>
-      <c r="E12" s="24"/>
+      <c r="E12" s="23"/>
       <c r="F12" s="11"/>
       <c r="G12" s="11"/>
       <c r="H12" s="11"/>
@@ -2378,7 +2409,7 @@
       <c r="B13" s="13"/>
       <c r="C13" s="13"/>
       <c r="D13" s="13"/>
-      <c r="E13" s="25"/>
+      <c r="E13" s="24"/>
       <c r="F13" s="13"/>
       <c r="G13" s="13"/>
       <c r="H13" s="13"/>
@@ -2388,7 +2419,7 @@
       <c r="B14" s="11"/>
       <c r="C14" s="11"/>
       <c r="D14" s="11"/>
-      <c r="E14" s="24"/>
+      <c r="E14" s="23"/>
       <c r="F14" s="11"/>
       <c r="G14" s="11"/>
       <c r="H14" s="11"/>
@@ -2398,7 +2429,7 @@
       <c r="B15" s="13"/>
       <c r="C15" s="13"/>
       <c r="D15" s="13"/>
-      <c r="E15" s="25"/>
+      <c r="E15" s="24"/>
       <c r="F15" s="13"/>
       <c r="G15" s="13"/>
       <c r="H15" s="13"/>
@@ -2408,7 +2439,7 @@
       <c r="B16" s="11"/>
       <c r="C16" s="11"/>
       <c r="D16" s="11"/>
-      <c r="E16" s="24"/>
+      <c r="E16" s="23"/>
       <c r="F16" s="11"/>
       <c r="G16" s="11"/>
       <c r="H16" s="11"/>
@@ -2418,7 +2449,7 @@
       <c r="B17" s="13"/>
       <c r="C17" s="13"/>
       <c r="D17" s="13"/>
-      <c r="E17" s="25"/>
+      <c r="E17" s="24"/>
       <c r="F17" s="13"/>
       <c r="G17" s="13"/>
       <c r="H17" s="13"/>
@@ -2428,7 +2459,7 @@
       <c r="B18" s="11"/>
       <c r="C18" s="11"/>
       <c r="D18" s="11"/>
-      <c r="E18" s="24"/>
+      <c r="E18" s="23"/>
       <c r="F18" s="11"/>
       <c r="G18" s="11"/>
       <c r="H18" s="11"/>
@@ -2438,7 +2469,7 @@
       <c r="B19" s="13"/>
       <c r="C19" s="13"/>
       <c r="D19" s="13"/>
-      <c r="E19" s="25"/>
+      <c r="E19" s="24"/>
       <c r="F19" s="13"/>
       <c r="G19" s="13"/>
       <c r="H19" s="13"/>
@@ -2448,7 +2479,7 @@
       <c r="B20" s="11"/>
       <c r="C20" s="11"/>
       <c r="D20" s="11"/>
-      <c r="E20" s="24"/>
+      <c r="E20" s="23"/>
       <c r="F20" s="11"/>
       <c r="G20" s="11"/>
       <c r="H20" s="11"/>
@@ -2458,7 +2489,7 @@
       <c r="B21" s="13"/>
       <c r="C21" s="13"/>
       <c r="D21" s="13"/>
-      <c r="E21" s="25"/>
+      <c r="E21" s="24"/>
       <c r="F21" s="13"/>
       <c r="G21" s="13"/>
       <c r="H21" s="13"/>
@@ -2468,7 +2499,7 @@
       <c r="B22" s="11"/>
       <c r="C22" s="11"/>
       <c r="D22" s="11"/>
-      <c r="E22" s="24"/>
+      <c r="E22" s="23"/>
       <c r="F22" s="11"/>
       <c r="G22" s="11"/>
       <c r="H22" s="11"/>
@@ -2478,7 +2509,7 @@
       <c r="B23" s="13"/>
       <c r="C23" s="13"/>
       <c r="D23" s="13"/>
-      <c r="E23" s="25"/>
+      <c r="E23" s="24"/>
       <c r="F23" s="13"/>
       <c r="G23" s="13"/>
       <c r="H23" s="13"/>
@@ -2488,7 +2519,7 @@
       <c r="B24" s="11"/>
       <c r="C24" s="11"/>
       <c r="D24" s="11"/>
-      <c r="E24" s="24"/>
+      <c r="E24" s="23"/>
       <c r="F24" s="11"/>
       <c r="G24" s="11"/>
       <c r="H24" s="11"/>
@@ -2498,7 +2529,7 @@
       <c r="B25" s="13"/>
       <c r="C25" s="13"/>
       <c r="D25" s="13"/>
-      <c r="E25" s="25"/>
+      <c r="E25" s="24"/>
       <c r="F25" s="13"/>
       <c r="G25" s="13"/>
       <c r="H25" s="13"/>
@@ -2508,7 +2539,7 @@
       <c r="B26" s="11"/>
       <c r="C26" s="11"/>
       <c r="D26" s="11"/>
-      <c r="E26" s="24"/>
+      <c r="E26" s="23"/>
       <c r="F26" s="11"/>
       <c r="G26" s="11"/>
       <c r="H26" s="11"/>
@@ -2518,7 +2549,7 @@
       <c r="B27" s="13"/>
       <c r="C27" s="13"/>
       <c r="D27" s="13"/>
-      <c r="E27" s="25"/>
+      <c r="E27" s="24"/>
       <c r="F27" s="13"/>
       <c r="G27" s="13"/>
       <c r="H27" s="13"/>
@@ -2528,7 +2559,7 @@
       <c r="B28" s="11"/>
       <c r="C28" s="11"/>
       <c r="D28" s="11"/>
-      <c r="E28" s="24"/>
+      <c r="E28" s="23"/>
       <c r="F28" s="11"/>
       <c r="G28" s="11"/>
       <c r="H28" s="11"/>
@@ -2538,7 +2569,7 @@
       <c r="B29" s="13"/>
       <c r="C29" s="13"/>
       <c r="D29" s="13"/>
-      <c r="E29" s="25"/>
+      <c r="E29" s="24"/>
       <c r="F29" s="13"/>
       <c r="G29" s="13"/>
       <c r="H29" s="13"/>
@@ -2548,7 +2579,7 @@
       <c r="B30" s="11"/>
       <c r="C30" s="11"/>
       <c r="D30" s="11"/>
-      <c r="E30" s="24"/>
+      <c r="E30" s="23"/>
       <c r="F30" s="11"/>
       <c r="G30" s="11"/>
       <c r="H30" s="11"/>
@@ -2558,7 +2589,7 @@
       <c r="B31" s="13"/>
       <c r="C31" s="13"/>
       <c r="D31" s="13"/>
-      <c r="E31" s="25"/>
+      <c r="E31" s="24"/>
       <c r="F31" s="13"/>
       <c r="G31" s="13"/>
       <c r="H31" s="13"/>
@@ -2568,7 +2599,7 @@
       <c r="B32" s="11"/>
       <c r="C32" s="11"/>
       <c r="D32" s="11"/>
-      <c r="E32" s="24"/>
+      <c r="E32" s="23"/>
       <c r="F32" s="11"/>
       <c r="G32" s="11"/>
       <c r="H32" s="11"/>
@@ -2578,7 +2609,7 @@
       <c r="B33" s="13"/>
       <c r="C33" s="13"/>
       <c r="D33" s="13"/>
-      <c r="E33" s="25"/>
+      <c r="E33" s="24"/>
       <c r="F33" s="13"/>
       <c r="G33" s="13"/>
       <c r="H33" s="13"/>
@@ -2588,7 +2619,7 @@
       <c r="B34" s="11"/>
       <c r="C34" s="11"/>
       <c r="D34" s="11"/>
-      <c r="E34" s="24"/>
+      <c r="E34" s="23"/>
       <c r="F34" s="11"/>
       <c r="G34" s="11"/>
       <c r="H34" s="11"/>
@@ -2598,7 +2629,7 @@
       <c r="B35" s="13"/>
       <c r="C35" s="13"/>
       <c r="D35" s="13"/>
-      <c r="E35" s="25"/>
+      <c r="E35" s="24"/>
       <c r="F35" s="13"/>
       <c r="G35" s="13"/>
       <c r="H35" s="13"/>
@@ -2608,7 +2639,7 @@
       <c r="B36" s="11"/>
       <c r="C36" s="11"/>
       <c r="D36" s="11"/>
-      <c r="E36" s="24"/>
+      <c r="E36" s="23"/>
       <c r="F36" s="11"/>
       <c r="G36" s="11"/>
       <c r="H36" s="11"/>
@@ -2618,7 +2649,7 @@
       <c r="B37" s="13"/>
       <c r="C37" s="13"/>
       <c r="D37" s="13"/>
-      <c r="E37" s="25"/>
+      <c r="E37" s="24"/>
       <c r="F37" s="13"/>
       <c r="G37" s="13"/>
       <c r="H37" s="13"/>
@@ -2628,7 +2659,7 @@
       <c r="B38" s="11"/>
       <c r="C38" s="11"/>
       <c r="D38" s="11"/>
-      <c r="E38" s="24"/>
+      <c r="E38" s="23"/>
       <c r="F38" s="11"/>
       <c r="G38" s="11"/>
       <c r="H38" s="11"/>
@@ -2638,7 +2669,7 @@
       <c r="B39" s="13"/>
       <c r="C39" s="13"/>
       <c r="D39" s="13"/>
-      <c r="E39" s="25"/>
+      <c r="E39" s="24"/>
       <c r="F39" s="13"/>
       <c r="G39" s="13"/>
       <c r="H39" s="13"/>
@@ -2648,7 +2679,7 @@
       <c r="B40" s="11"/>
       <c r="C40" s="11"/>
       <c r="D40" s="11"/>
-      <c r="E40" s="24"/>
+      <c r="E40" s="23"/>
       <c r="F40" s="11"/>
       <c r="G40" s="11"/>
       <c r="H40" s="11"/>
@@ -2658,7 +2689,7 @@
       <c r="B41" s="13"/>
       <c r="C41" s="13"/>
       <c r="D41" s="13"/>
-      <c r="E41" s="25"/>
+      <c r="E41" s="24"/>
       <c r="F41" s="13"/>
       <c r="G41" s="13"/>
       <c r="H41" s="13"/>
@@ -2668,7 +2699,7 @@
       <c r="B42" s="11"/>
       <c r="C42" s="11"/>
       <c r="D42" s="11"/>
-      <c r="E42" s="24"/>
+      <c r="E42" s="23"/>
       <c r="F42" s="11"/>
       <c r="G42" s="11"/>
       <c r="H42" s="11"/>
@@ -2678,7 +2709,7 @@
       <c r="B43" s="13"/>
       <c r="C43" s="13"/>
       <c r="D43" s="13"/>
-      <c r="E43" s="25"/>
+      <c r="E43" s="24"/>
       <c r="F43" s="13"/>
       <c r="G43" s="13"/>
       <c r="H43" s="13"/>
@@ -2688,7 +2719,7 @@
       <c r="B44" s="11"/>
       <c r="C44" s="11"/>
       <c r="D44" s="11"/>
-      <c r="E44" s="24"/>
+      <c r="E44" s="23"/>
       <c r="F44" s="11"/>
       <c r="G44" s="11"/>
       <c r="H44" s="11"/>
@@ -2698,7 +2729,7 @@
       <c r="B45" s="13"/>
       <c r="C45" s="13"/>
       <c r="D45" s="13"/>
-      <c r="E45" s="25"/>
+      <c r="E45" s="24"/>
       <c r="F45" s="13"/>
       <c r="G45" s="13"/>
       <c r="H45" s="13"/>
@@ -2708,7 +2739,7 @@
       <c r="B46" s="11"/>
       <c r="C46" s="11"/>
       <c r="D46" s="11"/>
-      <c r="E46" s="24"/>
+      <c r="E46" s="23"/>
       <c r="F46" s="11"/>
       <c r="G46" s="11"/>
       <c r="H46" s="11"/>
@@ -2718,7 +2749,7 @@
       <c r="B47" s="13"/>
       <c r="C47" s="13"/>
       <c r="D47" s="13"/>
-      <c r="E47" s="25"/>
+      <c r="E47" s="24"/>
       <c r="F47" s="13"/>
       <c r="G47" s="13"/>
       <c r="H47" s="13"/>
@@ -2728,7 +2759,7 @@
       <c r="B48" s="11"/>
       <c r="C48" s="11"/>
       <c r="D48" s="11"/>
-      <c r="E48" s="24"/>
+      <c r="E48" s="23"/>
       <c r="F48" s="11"/>
       <c r="G48" s="11"/>
       <c r="H48" s="11"/>
@@ -2738,7 +2769,7 @@
       <c r="B49" s="13"/>
       <c r="C49" s="13"/>
       <c r="D49" s="13"/>
-      <c r="E49" s="25"/>
+      <c r="E49" s="24"/>
       <c r="F49" s="13"/>
       <c r="G49" s="13"/>
       <c r="H49" s="13"/>
@@ -2748,7 +2779,7 @@
       <c r="B50" s="11"/>
       <c r="C50" s="11"/>
       <c r="D50" s="11"/>
-      <c r="E50" s="24"/>
+      <c r="E50" s="23"/>
       <c r="F50" s="11"/>
       <c r="G50" s="11"/>
       <c r="H50" s="11"/>
@@ -2758,7 +2789,7 @@
       <c r="B51" s="13"/>
       <c r="C51" s="13"/>
       <c r="D51" s="13"/>
-      <c r="E51" s="25"/>
+      <c r="E51" s="24"/>
       <c r="F51" s="13"/>
       <c r="G51" s="13"/>
       <c r="H51" s="13"/>
@@ -2768,7 +2799,7 @@
       <c r="B52" s="11"/>
       <c r="C52" s="11"/>
       <c r="D52" s="11"/>
-      <c r="E52" s="24"/>
+      <c r="E52" s="23"/>
       <c r="F52" s="11"/>
       <c r="G52" s="11"/>
       <c r="H52" s="11"/>
@@ -2778,7 +2809,7 @@
       <c r="B53" s="13"/>
       <c r="C53" s="13"/>
       <c r="D53" s="13"/>
-      <c r="E53" s="25"/>
+      <c r="E53" s="24"/>
       <c r="F53" s="13"/>
       <c r="G53" s="13"/>
       <c r="H53" s="13"/>
@@ -2788,7 +2819,7 @@
       <c r="B54" s="11"/>
       <c r="C54" s="11"/>
       <c r="D54" s="11"/>
-      <c r="E54" s="24"/>
+      <c r="E54" s="23"/>
       <c r="F54" s="11"/>
       <c r="G54" s="11"/>
       <c r="H54" s="11"/>
@@ -2798,7 +2829,7 @@
       <c r="B55" s="13"/>
       <c r="C55" s="13"/>
       <c r="D55" s="13"/>
-      <c r="E55" s="25"/>
+      <c r="E55" s="24"/>
       <c r="F55" s="13"/>
       <c r="G55" s="13"/>
       <c r="H55" s="13"/>
@@ -2808,7 +2839,7 @@
       <c r="B56" s="11"/>
       <c r="C56" s="11"/>
       <c r="D56" s="11"/>
-      <c r="E56" s="24"/>
+      <c r="E56" s="23"/>
       <c r="F56" s="11"/>
       <c r="G56" s="11"/>
       <c r="H56" s="11"/>
@@ -2818,7 +2849,7 @@
       <c r="B57" s="13"/>
       <c r="C57" s="13"/>
       <c r="D57" s="13"/>
-      <c r="E57" s="25"/>
+      <c r="E57" s="24"/>
       <c r="F57" s="13"/>
       <c r="G57" s="13"/>
       <c r="H57" s="13"/>
@@ -2828,7 +2859,7 @@
       <c r="B58" s="11"/>
       <c r="C58" s="11"/>
       <c r="D58" s="11"/>
-      <c r="E58" s="24"/>
+      <c r="E58" s="23"/>
       <c r="F58" s="11"/>
       <c r="G58" s="11"/>
       <c r="H58" s="11"/>
@@ -2838,7 +2869,7 @@
       <c r="B59" s="13"/>
       <c r="C59" s="13"/>
       <c r="D59" s="13"/>
-      <c r="E59" s="25"/>
+      <c r="E59" s="24"/>
       <c r="F59" s="13"/>
       <c r="G59" s="13"/>
       <c r="H59" s="13"/>
@@ -2848,7 +2879,7 @@
       <c r="B60" s="11"/>
       <c r="C60" s="11"/>
       <c r="D60" s="11"/>
-      <c r="E60" s="24"/>
+      <c r="E60" s="23"/>
       <c r="F60" s="11"/>
       <c r="G60" s="11"/>
       <c r="H60" s="11"/>
@@ -2858,7 +2889,7 @@
       <c r="B61" s="13"/>
       <c r="C61" s="13"/>
       <c r="D61" s="13"/>
-      <c r="E61" s="25"/>
+      <c r="E61" s="24"/>
       <c r="F61" s="13"/>
       <c r="G61" s="13"/>
       <c r="H61" s="13"/>
@@ -2868,7 +2899,7 @@
       <c r="B62" s="11"/>
       <c r="C62" s="11"/>
       <c r="D62" s="11"/>
-      <c r="E62" s="24"/>
+      <c r="E62" s="23"/>
       <c r="F62" s="11"/>
       <c r="G62" s="11"/>
       <c r="H62" s="11"/>
@@ -2878,7 +2909,7 @@
       <c r="B63" s="13"/>
       <c r="C63" s="13"/>
       <c r="D63" s="13"/>
-      <c r="E63" s="25"/>
+      <c r="E63" s="24"/>
       <c r="F63" s="13"/>
       <c r="G63" s="13"/>
       <c r="H63" s="13"/>
@@ -2888,7 +2919,7 @@
       <c r="B64" s="11"/>
       <c r="C64" s="11"/>
       <c r="D64" s="11"/>
-      <c r="E64" s="24"/>
+      <c r="E64" s="23"/>
       <c r="F64" s="11"/>
       <c r="G64" s="11"/>
       <c r="H64" s="11"/>
@@ -2898,7 +2929,7 @@
       <c r="B65" s="13"/>
       <c r="C65" s="13"/>
       <c r="D65" s="13"/>
-      <c r="E65" s="25"/>
+      <c r="E65" s="24"/>
       <c r="F65" s="13"/>
       <c r="G65" s="13"/>
       <c r="H65" s="13"/>
@@ -2908,7 +2939,7 @@
       <c r="B66" s="11"/>
       <c r="C66" s="11"/>
       <c r="D66" s="11"/>
-      <c r="E66" s="24"/>
+      <c r="E66" s="23"/>
       <c r="F66" s="11"/>
       <c r="G66" s="11"/>
       <c r="H66" s="11"/>
@@ -2918,7 +2949,7 @@
       <c r="B67" s="13"/>
       <c r="C67" s="13"/>
       <c r="D67" s="13"/>
-      <c r="E67" s="25"/>
+      <c r="E67" s="24"/>
       <c r="F67" s="13"/>
       <c r="G67" s="13"/>
       <c r="H67" s="13"/>
@@ -2928,7 +2959,7 @@
       <c r="B68" s="11"/>
       <c r="C68" s="11"/>
       <c r="D68" s="11"/>
-      <c r="E68" s="24"/>
+      <c r="E68" s="23"/>
       <c r="F68" s="11"/>
       <c r="G68" s="11"/>
       <c r="H68" s="11"/>
@@ -2938,7 +2969,7 @@
       <c r="B69" s="13"/>
       <c r="C69" s="13"/>
       <c r="D69" s="13"/>
-      <c r="E69" s="25"/>
+      <c r="E69" s="24"/>
       <c r="F69" s="13"/>
       <c r="G69" s="13"/>
       <c r="H69" s="13"/>
@@ -2948,7 +2979,7 @@
       <c r="B70" s="11"/>
       <c r="C70" s="11"/>
       <c r="D70" s="11"/>
-      <c r="E70" s="24"/>
+      <c r="E70" s="23"/>
       <c r="F70" s="11"/>
       <c r="G70" s="11"/>
       <c r="H70" s="11"/>
@@ -2958,7 +2989,7 @@
       <c r="B71" s="13"/>
       <c r="C71" s="13"/>
       <c r="D71" s="13"/>
-      <c r="E71" s="25"/>
+      <c r="E71" s="24"/>
       <c r="F71" s="13"/>
       <c r="G71" s="13"/>
       <c r="H71" s="13"/>
@@ -2968,7 +2999,7 @@
       <c r="B72" s="11"/>
       <c r="C72" s="11"/>
       <c r="D72" s="11"/>
-      <c r="E72" s="24"/>
+      <c r="E72" s="23"/>
       <c r="F72" s="11"/>
       <c r="G72" s="11"/>
       <c r="H72" s="11"/>
@@ -2978,7 +3009,7 @@
       <c r="B73" s="13"/>
       <c r="C73" s="13"/>
       <c r="D73" s="13"/>
-      <c r="E73" s="25"/>
+      <c r="E73" s="24"/>
       <c r="F73" s="13"/>
       <c r="G73" s="13"/>
       <c r="H73" s="13"/>
@@ -2988,7 +3019,7 @@
       <c r="B74" s="11"/>
       <c r="C74" s="11"/>
       <c r="D74" s="11"/>
-      <c r="E74" s="24"/>
+      <c r="E74" s="23"/>
       <c r="F74" s="11"/>
       <c r="G74" s="11"/>
       <c r="H74" s="11"/>
@@ -2998,7 +3029,7 @@
       <c r="B75" s="13"/>
       <c r="C75" s="13"/>
       <c r="D75" s="13"/>
-      <c r="E75" s="25"/>
+      <c r="E75" s="24"/>
       <c r="F75" s="13"/>
       <c r="G75" s="13"/>
       <c r="H75" s="13"/>
@@ -3008,7 +3039,7 @@
       <c r="B76" s="11"/>
       <c r="C76" s="11"/>
       <c r="D76" s="11"/>
-      <c r="E76" s="24"/>
+      <c r="E76" s="23"/>
       <c r="F76" s="11"/>
       <c r="G76" s="11"/>
       <c r="H76" s="11"/>
@@ -3018,7 +3049,7 @@
       <c r="B77" s="13"/>
       <c r="C77" s="13"/>
       <c r="D77" s="13"/>
-      <c r="E77" s="25"/>
+      <c r="E77" s="24"/>
       <c r="F77" s="13"/>
       <c r="G77" s="13"/>
       <c r="H77" s="13"/>
@@ -3028,7 +3059,7 @@
       <c r="B78" s="11"/>
       <c r="C78" s="11"/>
       <c r="D78" s="11"/>
-      <c r="E78" s="24"/>
+      <c r="E78" s="23"/>
       <c r="F78" s="11"/>
       <c r="G78" s="11"/>
       <c r="H78" s="11"/>
@@ -3038,7 +3069,7 @@
       <c r="B79" s="13"/>
       <c r="C79" s="13"/>
       <c r="D79" s="13"/>
-      <c r="E79" s="25"/>
+      <c r="E79" s="24"/>
       <c r="F79" s="13"/>
       <c r="G79" s="13"/>
       <c r="H79" s="13"/>
@@ -3048,7 +3079,7 @@
       <c r="B80" s="11"/>
       <c r="C80" s="11"/>
       <c r="D80" s="11"/>
-      <c r="E80" s="24"/>
+      <c r="E80" s="23"/>
       <c r="F80" s="11"/>
       <c r="G80" s="11"/>
       <c r="H80" s="11"/>
@@ -3058,7 +3089,7 @@
       <c r="B81" s="13"/>
       <c r="C81" s="13"/>
       <c r="D81" s="13"/>
-      <c r="E81" s="25"/>
+      <c r="E81" s="24"/>
       <c r="F81" s="13"/>
       <c r="G81" s="13"/>
       <c r="H81" s="13"/>
@@ -3068,7 +3099,7 @@
       <c r="B82" s="11"/>
       <c r="C82" s="11"/>
       <c r="D82" s="11"/>
-      <c r="E82" s="24"/>
+      <c r="E82" s="23"/>
       <c r="F82" s="11"/>
       <c r="G82" s="11"/>
       <c r="H82" s="11"/>
@@ -3078,7 +3109,7 @@
       <c r="B83" s="13"/>
       <c r="C83" s="13"/>
       <c r="D83" s="13"/>
-      <c r="E83" s="25"/>
+      <c r="E83" s="24"/>
       <c r="F83" s="13"/>
       <c r="G83" s="13"/>
       <c r="H83" s="13"/>
@@ -3088,7 +3119,7 @@
       <c r="B84" s="11"/>
       <c r="C84" s="11"/>
       <c r="D84" s="11"/>
-      <c r="E84" s="24"/>
+      <c r="E84" s="23"/>
       <c r="F84" s="11"/>
       <c r="G84" s="11"/>
       <c r="H84" s="11"/>
@@ -3098,7 +3129,7 @@
       <c r="B85" s="13"/>
       <c r="C85" s="13"/>
       <c r="D85" s="13"/>
-      <c r="E85" s="25"/>
+      <c r="E85" s="24"/>
       <c r="F85" s="13"/>
       <c r="G85" s="13"/>
       <c r="H85" s="13"/>
@@ -3108,7 +3139,7 @@
       <c r="B86" s="11"/>
       <c r="C86" s="11"/>
       <c r="D86" s="11"/>
-      <c r="E86" s="24"/>
+      <c r="E86" s="23"/>
       <c r="F86" s="11"/>
       <c r="G86" s="11"/>
       <c r="H86" s="11"/>
@@ -3118,7 +3149,7 @@
       <c r="B87" s="13"/>
       <c r="C87" s="13"/>
       <c r="D87" s="13"/>
-      <c r="E87" s="25"/>
+      <c r="E87" s="24"/>
       <c r="F87" s="13"/>
       <c r="G87" s="13"/>
       <c r="H87" s="13"/>
@@ -3128,7 +3159,7 @@
       <c r="B88" s="11"/>
       <c r="C88" s="11"/>
       <c r="D88" s="11"/>
-      <c r="E88" s="24"/>
+      <c r="E88" s="23"/>
       <c r="F88" s="11"/>
       <c r="G88" s="11"/>
       <c r="H88" s="11"/>
@@ -3138,7 +3169,7 @@
       <c r="B89" s="13"/>
       <c r="C89" s="13"/>
       <c r="D89" s="13"/>
-      <c r="E89" s="25"/>
+      <c r="E89" s="24"/>
       <c r="F89" s="13"/>
       <c r="G89" s="13"/>
       <c r="H89" s="13"/>
@@ -3148,7 +3179,7 @@
       <c r="B90" s="11"/>
       <c r="C90" s="11"/>
       <c r="D90" s="11"/>
-      <c r="E90" s="24"/>
+      <c r="E90" s="23"/>
       <c r="F90" s="11"/>
       <c r="G90" s="11"/>
       <c r="H90" s="11"/>
@@ -3158,7 +3189,7 @@
       <c r="B91" s="13"/>
       <c r="C91" s="13"/>
       <c r="D91" s="13"/>
-      <c r="E91" s="25"/>
+      <c r="E91" s="24"/>
       <c r="F91" s="13"/>
       <c r="G91" s="13"/>
       <c r="H91" s="13"/>
@@ -3168,7 +3199,7 @@
       <c r="B92" s="11"/>
       <c r="C92" s="11"/>
       <c r="D92" s="11"/>
-      <c r="E92" s="24"/>
+      <c r="E92" s="23"/>
       <c r="F92" s="11"/>
       <c r="G92" s="11"/>
       <c r="H92" s="11"/>
@@ -3178,7 +3209,7 @@
       <c r="B93" s="13"/>
       <c r="C93" s="13"/>
       <c r="D93" s="13"/>
-      <c r="E93" s="25"/>
+      <c r="E93" s="24"/>
       <c r="F93" s="13"/>
       <c r="G93" s="13"/>
       <c r="H93" s="13"/>
@@ -3188,7 +3219,7 @@
       <c r="B94" s="11"/>
       <c r="C94" s="11"/>
       <c r="D94" s="11"/>
-      <c r="E94" s="24"/>
+      <c r="E94" s="23"/>
       <c r="F94" s="11"/>
       <c r="G94" s="11"/>
       <c r="H94" s="11"/>
@@ -3198,7 +3229,7 @@
       <c r="B95" s="13"/>
       <c r="C95" s="13"/>
       <c r="D95" s="13"/>
-      <c r="E95" s="25"/>
+      <c r="E95" s="24"/>
       <c r="F95" s="13"/>
       <c r="G95" s="13"/>
       <c r="H95" s="13"/>
@@ -3208,7 +3239,7 @@
       <c r="B96" s="11"/>
       <c r="C96" s="11"/>
       <c r="D96" s="11"/>
-      <c r="E96" s="24"/>
+      <c r="E96" s="23"/>
       <c r="F96" s="11"/>
       <c r="G96" s="11"/>
       <c r="H96" s="11"/>
@@ -3218,7 +3249,7 @@
       <c r="B97" s="13"/>
       <c r="C97" s="13"/>
       <c r="D97" s="13"/>
-      <c r="E97" s="25"/>
+      <c r="E97" s="24"/>
       <c r="F97" s="13"/>
       <c r="G97" s="13"/>
       <c r="H97" s="13"/>
@@ -3228,7 +3259,7 @@
       <c r="B98" s="11"/>
       <c r="C98" s="11"/>
       <c r="D98" s="11"/>
-      <c r="E98" s="24"/>
+      <c r="E98" s="23"/>
       <c r="F98" s="11"/>
       <c r="G98" s="11"/>
       <c r="H98" s="11"/>
@@ -3238,17 +3269,17 @@
       <c r="B99" s="13"/>
       <c r="C99" s="13"/>
       <c r="D99" s="13"/>
-      <c r="E99" s="25"/>
+      <c r="E99" s="24"/>
       <c r="F99" s="13"/>
       <c r="G99" s="13"/>
       <c r="H99" s="13"/>
     </row>
     <row r="100" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A100" s="28"/>
+      <c r="A100" s="27"/>
       <c r="B100" s="9"/>
       <c r="C100" s="9"/>
       <c r="D100" s="9"/>
-      <c r="E100" s="26"/>
+      <c r="E100" s="25"/>
       <c r="F100" s="9"/>
       <c r="G100" s="9"/>
       <c r="H100" s="9"/>
@@ -3298,7 +3329,7 @@
         <v>78</v>
       </c>
       <c r="C1" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -3323,130 +3354,89 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED4B5016-8080-45D9-A027-E465FB36B2D6}">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.44140625" style="29" customWidth="1"/>
-    <col min="4" max="4" width="13" style="22" customWidth="1"/>
-    <col min="5" max="5" width="9.44140625" style="22" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.6640625" style="22" customWidth="1"/>
+    <col min="1" max="1" width="12.44140625" style="28" customWidth="1"/>
+    <col min="2" max="2" width="10.21875" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="13" style="21" customWidth="1"/>
+    <col min="5" max="5" width="10.44140625" style="21" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.6640625" style="21" customWidth="1"/>
     <col min="7" max="7" width="10.33203125" customWidth="1"/>
+    <col min="9" max="9" width="13.5546875" customWidth="1"/>
+    <col min="10" max="10" width="14.5546875" style="21" customWidth="1"/>
+    <col min="11" max="11" width="11.33203125" style="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="29" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A1" s="28" t="s">
+        <v>227</v>
+      </c>
+      <c r="B1" t="s">
         <v>192</v>
-      </c>
-      <c r="B1" t="s">
-        <v>193</v>
       </c>
       <c r="C1" t="s">
         <v>66</v>
       </c>
-      <c r="D1" s="22" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="22" t="s">
+      <c r="D1" s="21" t="s">
+        <v>225</v>
+      </c>
+      <c r="E1" s="21" t="s">
+        <v>193</v>
+      </c>
+      <c r="F1" s="21" t="s">
         <v>194</v>
       </c>
-      <c r="F1" s="22" t="s">
+      <c r="G1" t="s">
         <v>195</v>
-      </c>
-      <c r="G1" t="s">
-        <v>196</v>
       </c>
       <c r="H1" t="s">
         <v>130</v>
       </c>
       <c r="I1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="29">
-        <v>46204</v>
+        <v>222</v>
+      </c>
+      <c r="J1" s="21" t="s">
+        <v>226</v>
+      </c>
+      <c r="K1" s="28" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A2" s="28">
+        <v>46197</v>
       </c>
       <c r="B2" t="s">
+        <v>229</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="21">
+        <v>86000</v>
+      </c>
+      <c r="E2" s="21">
+        <v>0</v>
+      </c>
+      <c r="F2" s="21">
+        <v>86000</v>
+      </c>
+      <c r="G2" s="28">
+        <v>46235</v>
+      </c>
+      <c r="H2" t="s">
         <v>197</v>
       </c>
-      <c r="C2" t="s">
-        <v>198</v>
-      </c>
-      <c r="D2" s="22">
-        <v>10000</v>
-      </c>
-      <c r="E2" s="22">
-        <v>0</v>
-      </c>
-      <c r="F2" s="22">
-        <v>10000</v>
-      </c>
-      <c r="G2" t="s">
-        <v>199</v>
-      </c>
-      <c r="H2" t="s">
-        <v>200</v>
-      </c>
       <c r="I2" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="29">
-        <v>46206</v>
-      </c>
-      <c r="B3" t="s">
-        <v>202</v>
-      </c>
-      <c r="C3" t="s">
-        <v>203</v>
-      </c>
-      <c r="D3" s="22">
-        <v>2000</v>
-      </c>
-      <c r="E3" s="22">
-        <v>1000</v>
-      </c>
-      <c r="F3" s="22">
-        <v>1000</v>
-      </c>
-      <c r="G3" s="16">
-        <v>46249</v>
-      </c>
-      <c r="H3" t="s">
-        <v>200</v>
-      </c>
-      <c r="I3" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="29">
-        <v>46208</v>
-      </c>
-      <c r="B4" t="s">
-        <v>224</v>
-      </c>
-      <c r="C4" t="s">
-        <v>203</v>
-      </c>
-      <c r="D4" s="22">
-        <v>1000</v>
-      </c>
-      <c r="E4" s="22">
-        <v>1000</v>
-      </c>
-      <c r="F4" s="22">
-        <v>0</v>
-      </c>
-      <c r="G4" s="16">
-        <v>46209</v>
-      </c>
-      <c r="H4" t="s">
-        <v>223</v>
-      </c>
-      <c r="I4" t="s">
-        <v>201</v>
+        <v>230</v>
+      </c>
+      <c r="J2" s="21">
+        <v>8600</v>
+      </c>
+      <c r="K2" s="28">
+        <v>46447</v>
       </c>
     </row>
   </sheetData>
@@ -3621,29 +3611,29 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>206</v>
-      </c>
-      <c r="B27" s="17">
+        <v>201</v>
+      </c>
+      <c r="B27" s="16">
         <f>SUM(FinancialCommitments[Remaining])</f>
-        <v>11000</v>
+        <v>86000</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>207</v>
-      </c>
-      <c r="B29" s="18">
-        <f>1-(SUM(FinancialCommitments[Remaining])/SUM(FinancialCommitments[Amount]))</f>
-        <v>0.15384615384615385</v>
+        <v>202</v>
+      </c>
+      <c r="B29" s="17">
+        <f>1-(SUM(FinancialCommitments[Remaining])/SUM(FinancialCommitments[Total Amount]))</f>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="B31" s="7">
         <f>B21-B27</f>
-        <v>10440</v>
+        <v>-64560</v>
       </c>
     </row>
   </sheetData>
@@ -3834,72 +3824,72 @@
       </c>
     </row>
     <row r="2" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="21">
+      <c r="A2" s="20">
         <v>46204</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="18" t="s">
         <v>127</v>
       </c>
-      <c r="C2" s="19" t="s">
+      <c r="C2" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="D2" s="19">
+        <v>22000</v>
+      </c>
+      <c r="E2" s="18" t="s">
+        <v>205</v>
+      </c>
+      <c r="F2" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="G2" s="18" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="20">
+        <v>46218</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>96</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="D3" s="19">
+        <v>5000</v>
+      </c>
+      <c r="E3" s="18" t="s">
+        <v>141</v>
+      </c>
+      <c r="F3" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="G3" s="18" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="20">
+        <v>46223</v>
+      </c>
+      <c r="B4" s="18" t="s">
         <v>209</v>
       </c>
-      <c r="D2" s="20">
-        <v>22000</v>
-      </c>
-      <c r="E2" s="19" t="s">
+      <c r="C4" s="18" t="s">
         <v>210</v>
       </c>
-      <c r="F2" s="19" t="s">
-        <v>75</v>
-      </c>
-      <c r="G2" s="19" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="21">
-        <v>46218</v>
-      </c>
-      <c r="B3" s="19" t="s">
-        <v>96</v>
-      </c>
-      <c r="C3" s="19" t="s">
-        <v>212</v>
-      </c>
-      <c r="D3" s="20">
-        <v>5000</v>
-      </c>
-      <c r="E3" s="19" t="s">
-        <v>141</v>
-      </c>
-      <c r="F3" s="19" t="s">
+      <c r="D4" s="19">
+        <v>2000</v>
+      </c>
+      <c r="E4" s="18" t="s">
+        <v>205</v>
+      </c>
+      <c r="F4" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="G3" s="19" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="21">
-        <v>46223</v>
-      </c>
-      <c r="B4" s="19" t="s">
-        <v>214</v>
-      </c>
-      <c r="C4" s="19" t="s">
-        <v>215</v>
-      </c>
-      <c r="D4" s="20">
-        <v>2000</v>
-      </c>
-      <c r="E4" s="19" t="s">
-        <v>210</v>
-      </c>
-      <c r="F4" s="19" t="s">
-        <v>76</v>
-      </c>
-      <c r="G4" s="19" t="s">
-        <v>202</v>
+      <c r="G4" s="18" t="s">
+        <v>198</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
v0.9.3 : implement complete Goal Engine and Goal Snapshot
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pratham OS\Development\Finance-AI\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{730C3D7B-58C4-4F50-8D32-14C92560ECA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5A23B97-B064-4DB3-87AC-632EBF3E9DFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="855" firstSheet="3" activeTab="3" xr2:uid="{D6DE1A26-0963-4585-A363-547897EAF3B2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="855" firstSheet="3" activeTab="8" xr2:uid="{D6DE1A26-0963-4585-A363-547897EAF3B2}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan" sheetId="1" r:id="rId1"/>
@@ -21,10 +21,11 @@
     <sheet name="Monthly Review" sheetId="5" r:id="rId6"/>
     <sheet name="Skill Tracker" sheetId="9" r:id="rId7"/>
     <sheet name="Income" sheetId="11" r:id="rId8"/>
-    <sheet name="Income engine" sheetId="6" r:id="rId9"/>
-    <sheet name="Carrer Tracker" sheetId="7" r:id="rId10"/>
-    <sheet name="Interview Prep" sheetId="8" r:id="rId11"/>
-    <sheet name="Lists" sheetId="3" r:id="rId12"/>
+    <sheet name="Financial Goals" sheetId="16" r:id="rId9"/>
+    <sheet name="Income engine" sheetId="6" r:id="rId10"/>
+    <sheet name="Carrer Tracker" sheetId="7" r:id="rId11"/>
+    <sheet name="Interview Prep" sheetId="8" r:id="rId12"/>
+    <sheet name="Lists" sheetId="3" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="AppliedStatus">Lists!$K$1:$K$10</definedName>
@@ -32,6 +33,8 @@
     <definedName name="Categories">Lists!$A$1:$A$15</definedName>
     <definedName name="Choice">Lists!$I$1:$I$2</definedName>
     <definedName name="CommitmentStatus">Lists!$I$7:$I$8</definedName>
+    <definedName name="GoalStatus">Lists!$G$10:$G$13</definedName>
+    <definedName name="GoalType">Lists!$E$10:$E$16</definedName>
     <definedName name="IncomeCategory">Lists!$C$7:$C$16</definedName>
     <definedName name="IncomeStatus">Lists!$I$4:$I$5</definedName>
     <definedName name="InterviewResult">Lists!$M$1:$M$3</definedName>
@@ -40,6 +43,7 @@
     <definedName name="NeedWant">Lists!$C$1:$C$2</definedName>
     <definedName name="NextAction">Lists!$Q$1:$Q$7</definedName>
     <definedName name="PaymentMode">Lists!$E$1:$E$4</definedName>
+    <definedName name="Priority">Lists!$F$10:$F$12</definedName>
     <definedName name="TransactionTe">Lists!#REF!</definedName>
     <definedName name="TransactionType">Lists!$G$1:$G$4</definedName>
     <definedName name="v">Lists!#REF!</definedName>
@@ -65,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="244">
   <si>
     <t>August Financial Plan</t>
   </si>
@@ -758,6 +762,45 @@
   </si>
   <si>
     <t>Laptop EMI</t>
+  </si>
+  <si>
+    <t>Goal</t>
+  </si>
+  <si>
+    <t>Target Amount</t>
+  </si>
+  <si>
+    <t>Current Amount</t>
+  </si>
+  <si>
+    <t>Start Date</t>
+  </si>
+  <si>
+    <t>Target Date</t>
+  </si>
+  <si>
+    <t>Emergency</t>
+  </si>
+  <si>
+    <t>Business Capital</t>
+  </si>
+  <si>
+    <t>Bike</t>
+  </si>
+  <si>
+    <t>Purchase</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>Paused</t>
+  </si>
+  <si>
+    <t>Cancelled</t>
   </si>
 </sst>
 </file>
@@ -920,7 +963,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -956,6 +999,18 @@
     <xf numFmtId="14" fontId="2" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -964,7 +1019,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="22">
+  <dxfs count="31">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -984,24 +1039,6 @@
           <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1048,6 +1085,24 @@
       </font>
     </dxf>
     <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
@@ -1086,6 +1141,51 @@
           <bgColor theme="2" tint="-9.9978637043366805E-2"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1133,39 +1233,56 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{1AFBBFA5-5EA2-4DA5-91C7-5EE90985F084}" name="FinancialCommitments" displayName="FinancialCommitments" ref="A1:K46" totalsRowShown="0">
   <autoFilter ref="A1:K46" xr:uid="{1AFBBFA5-5EA2-4DA5-91C7-5EE90985F084}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{C10697DD-F282-4D7F-A12A-9BFC6193DC4E}" name="Start Date " dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{C10697DD-F282-4D7F-A12A-9BFC6193DC4E}" name="Start Date " dataDxfId="16"/>
     <tableColumn id="2" xr3:uid="{D6130D6E-B2EE-4D09-94CD-7E8053CD1C7B}" name="From"/>
     <tableColumn id="3" xr3:uid="{8ECD20EB-BEF0-47D5-8DA5-28D491EC7B0A}" name="Type"/>
-    <tableColumn id="4" xr3:uid="{87D047F3-8B64-4D30-ACC0-42FFF26FEC3E}" name="Total Amount" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{C982624C-E448-4958-A5CE-7D794FC142FA}" name="Repaid" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{665D5056-3744-4E56-95C7-F0943FD35707}" name="Remaining" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{87D047F3-8B64-4D30-ACC0-42FFF26FEC3E}" name="Total Amount" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{C982624C-E448-4958-A5CE-7D794FC142FA}" name="Repaid" dataDxfId="14"/>
+    <tableColumn id="6" xr3:uid="{665D5056-3744-4E56-95C7-F0943FD35707}" name="Remaining" dataDxfId="13"/>
     <tableColumn id="7" xr3:uid="{FFDA91C5-2668-4023-9FEE-465A59D85270}" name="Due Date"/>
     <tableColumn id="8" xr3:uid="{748EB09B-78B0-49AB-AC7E-88A7F4C42C89}" name="Status"/>
     <tableColumn id="10" xr3:uid="{39DD9F5E-EB31-47B4-A27F-BDA3AA61DA00}" name="commitment"/>
-    <tableColumn id="11" xr3:uid="{740721D4-21BC-47E8-A178-052DE413178D}" name="Monthly Payment" dataDxfId="2"/>
-    <tableColumn id="12" xr3:uid="{2EEE087F-37EF-44B3-8405-6F6CCBE4BDEB}" name="End Date" dataDxfId="3"/>
+    <tableColumn id="11" xr3:uid="{740721D4-21BC-47E8-A178-052DE413178D}" name="Monthly Payment" dataDxfId="12"/>
+    <tableColumn id="12" xr3:uid="{2EEE087F-37EF-44B3-8405-6F6CCBE4BDEB}" name="End Date" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{7C5D4057-F5F1-485E-AE6E-34A855BB81C8}" name="IncomeTable" displayName="IncomeTable" ref="A1:G4" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{7C5D4057-F5F1-485E-AE6E-34A855BB81C8}" name="IncomeTable" displayName="IncomeTable" ref="A1:G4" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
   <autoFilter ref="A1:G4" xr:uid="{7C5D4057-F5F1-485E-AE6E-34A855BB81C8}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{85417279-B333-4129-826F-4B13A464B0A1}" name="Date" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{72151722-7F6E-43AF-AADF-05A0452D151E}" name="Source" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{A9F1D760-964B-4BC4-876E-FE2B218C85B6}" name="Category" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{31C0BCAE-AC93-4345-9B1C-546CE0735A6B}" name="Amount" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{C6E99480-C881-404B-8F25-E2549BD2CCCD}" name="Status" dataDxfId="10"/>
-    <tableColumn id="7" xr3:uid="{29AC2CCC-8D50-4D4F-9049-D5CBB08CDAB6}" name="Recurring" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{4D5A0A55-4298-4332-9A93-683CDAE35676}" name="Notes" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{85417279-B333-4129-826F-4B13A464B0A1}" name="Date" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{72151722-7F6E-43AF-AADF-05A0452D151E}" name="Source" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{A9F1D760-964B-4BC4-876E-FE2B218C85B6}" name="Category" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{31C0BCAE-AC93-4345-9B1C-546CE0735A6B}" name="Amount" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{C6E99480-C881-404B-8F25-E2549BD2CCCD}" name="Status" dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{29AC2CCC-8D50-4D4F-9049-D5CBB08CDAB6}" name="Recurring" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{4D5A0A55-4298-4332-9A93-683CDAE35676}" name="Notes" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{ED3F2086-7429-4708-9751-1D0D42E41B00}" name="Table6" displayName="Table6" ref="A1:H4" totalsRowShown="0" headerRowDxfId="30">
+  <autoFilter ref="A1:H4" xr:uid="{ED3F2086-7429-4708-9751-1D0D42E41B00}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{02A819B9-5B65-4731-BA10-C393EA3AE4AE}" name="Goal" dataDxfId="29"/>
+    <tableColumn id="2" xr3:uid="{51D61835-0ABB-4183-9CDE-6E008A5BE534}" name="Type" dataDxfId="28"/>
+    <tableColumn id="3" xr3:uid="{26F4B186-E946-48D7-9DD2-DA125EFEB650}" name="Target Amount" dataDxfId="27"/>
+    <tableColumn id="4" xr3:uid="{B407A7D5-A3D5-4F1F-A0BE-CEC184447D2F}" name="Current Amount" dataDxfId="26"/>
+    <tableColumn id="5" xr3:uid="{AC787662-7B98-4750-92E3-5F644C592A83}" name="Start Date" dataDxfId="25"/>
+    <tableColumn id="6" xr3:uid="{219A44EC-76A4-456E-8296-B0D5D5DB8C37}" name="Target Date" dataDxfId="24"/>
+    <tableColumn id="7" xr3:uid="{401F98C6-DE93-4917-B06B-A1F0D02774EE}" name="Priority" dataDxfId="23"/>
+    <tableColumn id="8" xr3:uid="{AFB6C60C-D1A2-49E4-B330-36821968B1DD}" name="Status" dataDxfId="22"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2E0C23CD-1E80-4D43-9A03-38675147AE03}" name="Table2" displayName="Table2" ref="A1:J50" totalsRowShown="0">
   <autoFilter ref="A1:J50" xr:uid="{2E0C23CD-1E80-4D43-9A03-38675147AE03}"/>
   <tableColumns count="10">
@@ -1505,12 +1622,12 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -1707,6 +1824,260 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C985A9ED-FFB7-41B9-BD81-D99D84E9A097}">
+  <dimension ref="A1:J35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B5" s="1">
+        <v>24</v>
+      </c>
+      <c r="J5" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="J7" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="15">
+        <v>8600</v>
+      </c>
+      <c r="J9" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B10" s="15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J11" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A13" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="J13" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="J15" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="D16" s="1">
+        <v>22000</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D17" s="1">
+        <v>23000</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="J17" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D18" s="1">
+        <v>28000</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="J19" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J21" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J23" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J25" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J27" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J29" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J31" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="33" spans="10:10" x14ac:dyDescent="0.3">
+      <c r="J33" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="35" spans="10:10" x14ac:dyDescent="0.3">
+      <c r="J35" t="s">
+        <v>123</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{062E0065-A33A-40A3-8681-B93160D6FE12}">
   <dimension ref="A1:Q5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1842,7 +2213,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52E36AC4-05BC-4C7B-BA73-388CE26BAB52}">
   <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1919,7 +2290,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{729B4158-2DD5-48A6-9BEC-2F739409F312}">
   <dimension ref="A1:Q23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2105,6 +2476,15 @@
       <c r="C10" t="s">
         <v>212</v>
       </c>
+      <c r="E10" t="s">
+        <v>236</v>
+      </c>
+      <c r="F10" t="s">
+        <v>98</v>
+      </c>
+      <c r="G10" t="s">
+        <v>197</v>
+      </c>
       <c r="K10" t="s">
         <v>140</v>
       </c>
@@ -2116,6 +2496,15 @@
       <c r="C11" t="s">
         <v>213</v>
       </c>
+      <c r="E11" t="s">
+        <v>239</v>
+      </c>
+      <c r="F11" t="s">
+        <v>99</v>
+      </c>
+      <c r="G11" t="s">
+        <v>241</v>
+      </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
@@ -2124,6 +2513,15 @@
       <c r="C12" t="s">
         <v>214</v>
       </c>
+      <c r="E12" t="s">
+        <v>71</v>
+      </c>
+      <c r="F12" t="s">
+        <v>240</v>
+      </c>
+      <c r="G12" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
@@ -2132,6 +2530,12 @@
       <c r="C13" t="s">
         <v>215</v>
       </c>
+      <c r="E13" t="s">
+        <v>69</v>
+      </c>
+      <c r="G13" t="s">
+        <v>243</v>
+      </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
@@ -2140,6 +2544,9 @@
       <c r="C14" t="s">
         <v>210</v>
       </c>
+      <c r="E14" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
@@ -2148,9 +2555,15 @@
       <c r="C15" t="s">
         <v>216</v>
       </c>
+      <c r="E15" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.3">
       <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="E16" t="s">
         <v>34</v>
       </c>
     </row>
@@ -3912,255 +4325,141 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C985A9ED-FFB7-41B9-BD81-D99D84E9A097}">
-  <dimension ref="A1:J35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22B8A8B1-D6E9-48D7-B673-8B34D210F2B5}">
+  <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.5546875" customWidth="1"/>
+    <col min="2" max="2" width="18.5546875" customWidth="1"/>
+    <col min="3" max="3" width="16.21875" customWidth="1"/>
+    <col min="4" max="4" width="15.88671875" customWidth="1"/>
+    <col min="5" max="5" width="11.21875" customWidth="1"/>
+    <col min="6" max="6" width="12.21875" customWidth="1"/>
+    <col min="7" max="7" width="9" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="B5" s="1">
-        <v>24</v>
-      </c>
-      <c r="J5" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="J7" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" s="15">
-        <v>8600</v>
-      </c>
-      <c r="J9" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
+    <row r="1" spans="1:8" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="29" t="s">
+        <v>231</v>
+      </c>
+      <c r="B1" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="C1" s="31" t="s">
+        <v>232</v>
+      </c>
+      <c r="D1" s="31" t="s">
+        <v>233</v>
+      </c>
+      <c r="E1" s="29" t="s">
+        <v>234</v>
+      </c>
+      <c r="F1" s="29" t="s">
+        <v>235</v>
+      </c>
+      <c r="G1" s="29" t="s">
+        <v>95</v>
+      </c>
+      <c r="H1" s="29" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="B10" s="15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="J11" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="J13" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="J15" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B16" s="1" t="s">
+      <c r="B2" s="18" t="s">
+        <v>236</v>
+      </c>
+      <c r="C2" s="30">
+        <v>100000</v>
+      </c>
+      <c r="D2" s="30">
+        <v>14840</v>
+      </c>
+      <c r="E2" s="32">
+        <v>46204</v>
+      </c>
+      <c r="F2" s="32">
+        <v>46387</v>
+      </c>
+      <c r="G2" s="18" t="s">
         <v>98</v>
       </c>
-      <c r="C16" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="D16" s="1">
-        <v>22000</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B17" s="1" t="s">
+      <c r="H2" s="18" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="18" t="s">
+        <v>237</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="C3" s="30">
+        <v>300000</v>
+      </c>
+      <c r="D3" s="30">
+        <v>25000</v>
+      </c>
+      <c r="E3" s="32">
+        <v>46204</v>
+      </c>
+      <c r="F3" s="32">
+        <v>46568</v>
+      </c>
+      <c r="G3" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="H3" s="18" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="18" t="s">
+        <v>238</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>239</v>
+      </c>
+      <c r="C4" s="30">
+        <v>200000</v>
+      </c>
+      <c r="D4" s="30">
+        <v>10000</v>
+      </c>
+      <c r="E4" s="32">
+        <v>46235</v>
+      </c>
+      <c r="F4" s="32">
+        <v>46600</v>
+      </c>
+      <c r="G4" s="18" t="s">
         <v>99</v>
       </c>
-      <c r="C17" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="D17" s="1">
-        <v>23000</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="J17" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A18" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="D18" s="1">
-        <v>28000</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A19" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="J19" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A20" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="J21" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="J23" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="J25" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="J27" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="J29" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="J31" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="33" spans="10:10" x14ac:dyDescent="0.3">
-      <c r="J33" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="35" spans="10:10" x14ac:dyDescent="0.3">
-      <c r="J35" t="s">
-        <v>123</v>
+      <c r="H4" s="18" t="s">
+        <v>197</v>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="4">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B1 B181:B1048576 B101:B180" xr:uid="{303291A6-40D6-47AA-ABAF-BD2736805EF3}">
+      <formula1>"GoalType"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B100" xr:uid="{26D7973C-A735-47BC-A2D4-37BDB88E3128}">
+      <formula1>GoalType</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G100" xr:uid="{263111D5-5134-4C6A-8DD8-871BE3070266}">
+      <formula1>Priority</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H100" xr:uid="{E43D34CA-1631-4479-B887-97F5579584F3}">
+      <formula1>GoalStatus</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
(v0.9.5): add Investment & Asset Intelligence Engine
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pratham OS\Development\Finance-AI\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEF25F8C-DA8B-4053-B1B3-BF35FF25DE13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6876AE58-3161-4589-BC57-652CA4974181}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="855" firstSheet="3" activeTab="8" xr2:uid="{D6DE1A26-0963-4585-A363-547897EAF3B2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="855" firstSheet="3" activeTab="11" xr2:uid="{D6DE1A26-0963-4585-A363-547897EAF3B2}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan" sheetId="1" r:id="rId1"/>
@@ -22,10 +22,12 @@
     <sheet name="Skill Tracker" sheetId="9" r:id="rId7"/>
     <sheet name="Income" sheetId="11" r:id="rId8"/>
     <sheet name="Financial Goals" sheetId="16" r:id="rId9"/>
-    <sheet name="Income engine" sheetId="6" r:id="rId10"/>
-    <sheet name="Carrer Tracker" sheetId="7" r:id="rId11"/>
-    <sheet name="Interview Prep" sheetId="8" r:id="rId12"/>
-    <sheet name="Lists" sheetId="3" r:id="rId13"/>
+    <sheet name="Investments" sheetId="17" r:id="rId10"/>
+    <sheet name="Assets" sheetId="18" r:id="rId11"/>
+    <sheet name="Income engine" sheetId="6" r:id="rId12"/>
+    <sheet name="Carrer Tracker" sheetId="7" r:id="rId13"/>
+    <sheet name="Interview Prep" sheetId="8" r:id="rId14"/>
+    <sheet name="Lists" sheetId="3" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="AppliedStatus">Lists!$K$1:$K$10</definedName>
@@ -69,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="254">
   <si>
     <t>August Financial Plan</t>
   </si>
@@ -801,6 +803,36 @@
   </si>
   <si>
     <t>Cancelled</t>
+  </si>
+  <si>
+    <t>Purchase Date</t>
+  </si>
+  <si>
+    <t>Platform</t>
+  </si>
+  <si>
+    <t>Invested Amount</t>
+  </si>
+  <si>
+    <t>Current Value</t>
+  </si>
+  <si>
+    <t>Units</t>
+  </si>
+  <si>
+    <t>Return</t>
+  </si>
+  <si>
+    <t>Asset</t>
+  </si>
+  <si>
+    <t>Purchase Value</t>
+  </si>
+  <si>
+    <t>Electronics</t>
+  </si>
+  <si>
+    <t>Vehicle</t>
   </si>
 </sst>
 </file>
@@ -1019,7 +1051,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="31">
+  <dxfs count="32">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1039,6 +1071,51 @@
           <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1143,49 +1220,7 @@
       </fill>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1201,14 +1236,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{42D67FA3-A40A-4607-BCB9-468A9ECB0007}" name="Table1" displayName="Table1" ref="A1:H1048576" totalsRowShown="0" headerRowDxfId="21" tableBorderDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{42D67FA3-A40A-4607-BCB9-468A9ECB0007}" name="Table1" displayName="Table1" ref="A1:H1048576" totalsRowShown="0" headerRowDxfId="30" tableBorderDxfId="29">
   <autoFilter ref="A1:H1048576" xr:uid="{42D67FA3-A40A-4607-BCB9-468A9ECB0007}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{1D37F906-33D7-46E6-8270-56D5EEA80EC7}" name="Date" dataDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{1D37F906-33D7-46E6-8270-56D5EEA80EC7}" name="Date" dataDxfId="28"/>
     <tableColumn id="4" xr3:uid="{E805A8A8-660D-4099-912A-BE1B697553ED}" name="Type"/>
     <tableColumn id="5" xr3:uid="{ABF1E4D7-7922-479D-94F4-994DCBA1062D}" name="Category"/>
     <tableColumn id="6" xr3:uid="{E21EA904-BC60-4EB5-B4BD-249E5A12FC76}" name="Description "/>
-    <tableColumn id="7" xr3:uid="{EFA172CE-B81A-4A83-BB09-0C52BED62422}" name="Amount" dataDxfId="18"/>
+    <tableColumn id="7" xr3:uid="{EFA172CE-B81A-4A83-BB09-0C52BED62422}" name="Amount" dataDxfId="27"/>
     <tableColumn id="8" xr3:uid="{E811D3EB-DAD5-46D9-B70D-01072B332F5C}" name="Need/Want"/>
     <tableColumn id="9" xr3:uid="{1E8766C9-2C6F-4CE3-9C7E-C6C8545D3945}" name="Payment Mode"/>
     <tableColumn id="10" xr3:uid="{BA26CD78-BAFB-4644-808D-0A18546F6CAF}" name="Recurring"/>
@@ -1221,7 +1256,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{204CD917-42D7-44E9-889E-B87F7E170616}" name="Table5" displayName="Table5" ref="A1:C100" totalsRowShown="0">
   <autoFilter ref="A1:C100" xr:uid="{204CD917-42D7-44E9-889E-B87F7E170616}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{CCD99EA9-9CA0-4F69-8282-1EE2E5FE7967}" name="Month" dataDxfId="17"/>
+    <tableColumn id="1" xr3:uid="{CCD99EA9-9CA0-4F69-8282-1EE2E5FE7967}" name="Month" dataDxfId="26"/>
     <tableColumn id="2" xr3:uid="{5C307EC1-8BAE-4B8C-AF42-D468202B7A5E}" name="Year"/>
     <tableColumn id="3" xr3:uid="{2B3569FD-9348-4E00-BFEA-53DF4F58E82C}" name="Monthly_Budget"/>
   </tableColumns>
@@ -1233,56 +1268,91 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{1AFBBFA5-5EA2-4DA5-91C7-5EE90985F084}" name="FinancialCommitments" displayName="FinancialCommitments" ref="A1:K46" totalsRowShown="0">
   <autoFilter ref="A1:K46" xr:uid="{1AFBBFA5-5EA2-4DA5-91C7-5EE90985F084}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{C10697DD-F282-4D7F-A12A-9BFC6193DC4E}" name="Start Date " dataDxfId="16"/>
+    <tableColumn id="1" xr3:uid="{C10697DD-F282-4D7F-A12A-9BFC6193DC4E}" name="Start Date " dataDxfId="25"/>
     <tableColumn id="2" xr3:uid="{D6130D6E-B2EE-4D09-94CD-7E8053CD1C7B}" name="From"/>
     <tableColumn id="3" xr3:uid="{8ECD20EB-BEF0-47D5-8DA5-28D491EC7B0A}" name="Type"/>
-    <tableColumn id="4" xr3:uid="{87D047F3-8B64-4D30-ACC0-42FFF26FEC3E}" name="Total Amount" dataDxfId="15"/>
-    <tableColumn id="5" xr3:uid="{C982624C-E448-4958-A5CE-7D794FC142FA}" name="Repaid" dataDxfId="14"/>
-    <tableColumn id="6" xr3:uid="{665D5056-3744-4E56-95C7-F0943FD35707}" name="Remaining" dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{87D047F3-8B64-4D30-ACC0-42FFF26FEC3E}" name="Total Amount" dataDxfId="24"/>
+    <tableColumn id="5" xr3:uid="{C982624C-E448-4958-A5CE-7D794FC142FA}" name="Repaid" dataDxfId="23"/>
+    <tableColumn id="6" xr3:uid="{665D5056-3744-4E56-95C7-F0943FD35707}" name="Remaining" dataDxfId="22"/>
     <tableColumn id="7" xr3:uid="{FFDA91C5-2668-4023-9FEE-465A59D85270}" name="Due Date"/>
     <tableColumn id="8" xr3:uid="{748EB09B-78B0-49AB-AC7E-88A7F4C42C89}" name="Status"/>
     <tableColumn id="10" xr3:uid="{39DD9F5E-EB31-47B4-A27F-BDA3AA61DA00}" name="commitment"/>
-    <tableColumn id="11" xr3:uid="{740721D4-21BC-47E8-A178-052DE413178D}" name="Monthly Payment" dataDxfId="12"/>
-    <tableColumn id="12" xr3:uid="{2EEE087F-37EF-44B3-8405-6F6CCBE4BDEB}" name="End Date" dataDxfId="11"/>
+    <tableColumn id="11" xr3:uid="{740721D4-21BC-47E8-A178-052DE413178D}" name="Monthly Payment" dataDxfId="21"/>
+    <tableColumn id="12" xr3:uid="{2EEE087F-37EF-44B3-8405-6F6CCBE4BDEB}" name="End Date" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{7C5D4057-F5F1-485E-AE6E-34A855BB81C8}" name="IncomeTable" displayName="IncomeTable" ref="A1:G4" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{7C5D4057-F5F1-485E-AE6E-34A855BB81C8}" name="IncomeTable" displayName="IncomeTable" ref="A1:G4" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
   <autoFilter ref="A1:G4" xr:uid="{7C5D4057-F5F1-485E-AE6E-34A855BB81C8}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{85417279-B333-4129-826F-4B13A464B0A1}" name="Date" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{72151722-7F6E-43AF-AADF-05A0452D151E}" name="Source" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{A9F1D760-964B-4BC4-876E-FE2B218C85B6}" name="Category" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{31C0BCAE-AC93-4345-9B1C-546CE0735A6B}" name="Amount" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{C6E99480-C881-404B-8F25-E2549BD2CCCD}" name="Status" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{29AC2CCC-8D50-4D4F-9049-D5CBB08CDAB6}" name="Recurring" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{4D5A0A55-4298-4332-9A93-683CDAE35676}" name="Notes" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{85417279-B333-4129-826F-4B13A464B0A1}" name="Date" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{72151722-7F6E-43AF-AADF-05A0452D151E}" name="Source" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{A9F1D760-964B-4BC4-876E-FE2B218C85B6}" name="Category" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{31C0BCAE-AC93-4345-9B1C-546CE0735A6B}" name="Amount" dataDxfId="14"/>
+    <tableColumn id="5" xr3:uid="{C6E99480-C881-404B-8F25-E2549BD2CCCD}" name="Status" dataDxfId="13"/>
+    <tableColumn id="7" xr3:uid="{29AC2CCC-8D50-4D4F-9049-D5CBB08CDAB6}" name="Recurring" dataDxfId="12"/>
+    <tableColumn id="6" xr3:uid="{4D5A0A55-4298-4332-9A93-683CDAE35676}" name="Notes" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{ED3F2086-7429-4708-9751-1D0D42E41B00}" name="Table6" displayName="Table6" ref="A1:H4" totalsRowShown="0" headerRowDxfId="30">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{ED3F2086-7429-4708-9751-1D0D42E41B00}" name="Table6" displayName="Table6" ref="A1:H4" totalsRowShown="0" headerRowDxfId="10">
   <autoFilter ref="A1:H4" xr:uid="{ED3F2086-7429-4708-9751-1D0D42E41B00}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{02A819B9-5B65-4731-BA10-C393EA3AE4AE}" name="Goal" dataDxfId="29"/>
-    <tableColumn id="2" xr3:uid="{51D61835-0ABB-4183-9CDE-6E008A5BE534}" name="Type" dataDxfId="28"/>
-    <tableColumn id="3" xr3:uid="{26F4B186-E946-48D7-9DD2-DA125EFEB650}" name="Target Amount" dataDxfId="27"/>
-    <tableColumn id="4" xr3:uid="{B407A7D5-A3D5-4F1F-A0BE-CEC184447D2F}" name="Current Amount" dataDxfId="26"/>
-    <tableColumn id="5" xr3:uid="{AC787662-7B98-4750-92E3-5F644C592A83}" name="Start Date" dataDxfId="25"/>
-    <tableColumn id="6" xr3:uid="{219A44EC-76A4-456E-8296-B0D5D5DB8C37}" name="Target Date" dataDxfId="24"/>
-    <tableColumn id="7" xr3:uid="{401F98C6-DE93-4917-B06B-A1F0D02774EE}" name="Priority" dataDxfId="23"/>
-    <tableColumn id="8" xr3:uid="{AFB6C60C-D1A2-49E4-B330-36821968B1DD}" name="Status" dataDxfId="22"/>
+    <tableColumn id="1" xr3:uid="{02A819B9-5B65-4731-BA10-C393EA3AE4AE}" name="Goal" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{51D61835-0ABB-4183-9CDE-6E008A5BE534}" name="Type" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{26F4B186-E946-48D7-9DD2-DA125EFEB650}" name="Target Amount" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{B407A7D5-A3D5-4F1F-A0BE-CEC184447D2F}" name="Current Amount" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{AC787662-7B98-4750-92E3-5F644C592A83}" name="Start Date" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{219A44EC-76A4-456E-8296-B0D5D5DB8C37}" name="Target Date" dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{401F98C6-DE93-4917-B06B-A1F0D02774EE}" name="Priority" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{AFB6C60C-D1A2-49E4-B330-36821968B1DD}" name="Status" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{7E348894-AB6B-47ED-8D66-B030107418E7}" name="Table7" displayName="Table7" ref="A1:J200" totalsRowShown="0">
+  <autoFilter ref="A1:J200" xr:uid="{7E348894-AB6B-47ED-8D66-B030107418E7}"/>
+  <tableColumns count="10">
+    <tableColumn id="1" xr3:uid="{76E56D66-576D-4754-ADFE-436DD70011B2}" name="Date"/>
+    <tableColumn id="2" xr3:uid="{AAAC6B22-EF0E-43D9-B017-EB668B0236DD}" name="Investment"/>
+    <tableColumn id="3" xr3:uid="{CF097674-7777-4A04-A504-F67ED104098F}" name="Type"/>
+    <tableColumn id="4" xr3:uid="{1C676C24-A4B4-439F-AF8F-F0507E28FD4D}" name="Platform"/>
+    <tableColumn id="5" xr3:uid="{CA468ED8-AA61-447C-8470-4B90C0EC17EE}" name="Invested Amount"/>
+    <tableColumn id="6" xr3:uid="{36BB9FF4-2216-457F-952A-3B1DD164A26A}" name="Current Value"/>
+    <tableColumn id="7" xr3:uid="{C083E934-5CB3-41D8-9FAE-0480212E73D3}" name="Units"/>
+    <tableColumn id="8" xr3:uid="{0DB5DA9B-107E-4E46-B79E-99AFD4D44BB7}" name="Return"/>
+    <tableColumn id="9" xr3:uid="{5F434CC9-3372-48CB-B21E-E9D715DEC43F}" name="Status"/>
+    <tableColumn id="10" xr3:uid="{436FBE32-C5B6-433F-96E4-875D891423A2}" name="Notes"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{E6C8C911-DBF7-413D-A8D8-C9F208A9B6E1}" name="Table8" displayName="Table8" ref="A1:G200" totalsRowShown="0">
+  <autoFilter ref="A1:G200" xr:uid="{E6C8C911-DBF7-413D-A8D8-C9F208A9B6E1}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{E1888108-78C1-492E-82D0-DAB415C45FE0}" name="Asset"/>
+    <tableColumn id="2" xr3:uid="{AC7352C6-0DC7-4AFC-BDAD-303C389924A5}" name="Category"/>
+    <tableColumn id="3" xr3:uid="{9884F549-FF9E-426C-A41E-5854163D6493}" name="Purchase Value"/>
+    <tableColumn id="4" xr3:uid="{486852BE-C51C-4E3A-9B66-11D7D9CCEE9B}" name="Current Value"/>
+    <tableColumn id="5" xr3:uid="{2F141C2F-956F-436C-B98A-F15A4A0A762D}" name="Purchase Date" dataDxfId="31"/>
+    <tableColumn id="6" xr3:uid="{ED74E306-AFE5-436F-911F-2ED2CC19D23C}" name="Status"/>
+    <tableColumn id="7" xr3:uid="{93FAD5D9-55A0-4F40-A483-B99C6367CC93}" name="Notes"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2E0C23CD-1E80-4D43-9A03-38675147AE03}" name="Table2" displayName="Table2" ref="A1:J50" totalsRowShown="0">
   <autoFilter ref="A1:J50" xr:uid="{2E0C23CD-1E80-4D43-9A03-38675147AE03}"/>
   <tableColumns count="10">
@@ -1824,6 +1894,161 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81C8BF25-6B83-466D-AAB3-1C00FAFB6B75}">
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="8.88671875" customWidth="1"/>
+    <col min="2" max="2" width="12.21875" customWidth="1"/>
+    <col min="4" max="4" width="10.109375" customWidth="1"/>
+    <col min="5" max="5" width="16.77734375" customWidth="1"/>
+    <col min="6" max="6" width="14.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D1" t="s">
+        <v>245</v>
+      </c>
+      <c r="E1" t="s">
+        <v>246</v>
+      </c>
+      <c r="F1" t="s">
+        <v>247</v>
+      </c>
+      <c r="G1" t="s">
+        <v>248</v>
+      </c>
+      <c r="H1" t="s">
+        <v>249</v>
+      </c>
+      <c r="I1" t="s">
+        <v>130</v>
+      </c>
+      <c r="J1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4BD347A-E68F-44B6-B63F-C92671AA0A69}">
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="19" customWidth="1"/>
+    <col min="2" max="2" width="10.21875" customWidth="1"/>
+    <col min="3" max="3" width="15.5546875" customWidth="1"/>
+    <col min="4" max="4" width="14.109375" customWidth="1"/>
+    <col min="5" max="5" width="14.77734375" style="28" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>250</v>
+      </c>
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" t="s">
+        <v>251</v>
+      </c>
+      <c r="D1" t="s">
+        <v>247</v>
+      </c>
+      <c r="E1" s="28" t="s">
+        <v>244</v>
+      </c>
+      <c r="F1" t="s">
+        <v>130</v>
+      </c>
+      <c r="G1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>252</v>
+      </c>
+      <c r="C2" s="18">
+        <v>86000</v>
+      </c>
+      <c r="D2" s="18">
+        <v>80000</v>
+      </c>
+      <c r="E2" s="32">
+        <v>46197</v>
+      </c>
+      <c r="F2" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="18" t="s">
+        <v>238</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>253</v>
+      </c>
+      <c r="C3" s="18">
+        <v>90000</v>
+      </c>
+      <c r="D3" s="18">
+        <v>70000</v>
+      </c>
+      <c r="E3" s="32">
+        <v>46174</v>
+      </c>
+      <c r="F3" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="18" t="s">
+        <v>86</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="C4" s="18">
+        <v>14840</v>
+      </c>
+      <c r="D4" s="18">
+        <v>14840</v>
+      </c>
+      <c r="E4" s="32">
+        <v>46220</v>
+      </c>
+      <c r="F4" t="s">
+        <v>197</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C985A9ED-FFB7-41B9-BD81-D99D84E9A097}">
   <dimension ref="A1:J35"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2077,7 +2302,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{062E0065-A33A-40A3-8681-B93160D6FE12}">
   <dimension ref="A1:Q5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2213,7 +2438,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52E36AC4-05BC-4C7B-BA73-388CE26BAB52}">
   <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2290,7 +2515,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{729B4158-2DD5-48A6-9BEC-2F739409F312}">
   <dimension ref="A1:Q23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
(v0.9.6): complete Goal, Investment, Asset and Liability Engines
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pratham OS\Development\Finance-AI\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6876AE58-3161-4589-BC57-652CA4974181}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ED00688-9096-4D04-A468-E24B7648A096}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="855" firstSheet="3" activeTab="11" xr2:uid="{D6DE1A26-0963-4585-A363-547897EAF3B2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="855" firstSheet="5" activeTab="15" xr2:uid="{D6DE1A26-0963-4585-A363-547897EAF3B2}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan" sheetId="1" r:id="rId1"/>
@@ -23,11 +23,12 @@
     <sheet name="Income" sheetId="11" r:id="rId8"/>
     <sheet name="Financial Goals" sheetId="16" r:id="rId9"/>
     <sheet name="Investments" sheetId="17" r:id="rId10"/>
-    <sheet name="Assets" sheetId="18" r:id="rId11"/>
-    <sheet name="Income engine" sheetId="6" r:id="rId12"/>
-    <sheet name="Carrer Tracker" sheetId="7" r:id="rId13"/>
-    <sheet name="Interview Prep" sheetId="8" r:id="rId14"/>
-    <sheet name="Lists" sheetId="3" r:id="rId15"/>
+    <sheet name="Liabilities" sheetId="19" r:id="rId11"/>
+    <sheet name="Assets" sheetId="18" r:id="rId12"/>
+    <sheet name="Income engine" sheetId="6" r:id="rId13"/>
+    <sheet name="Carrer Tracker" sheetId="7" r:id="rId14"/>
+    <sheet name="Interview Prep" sheetId="8" r:id="rId15"/>
+    <sheet name="Lists" sheetId="3" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="AppliedStatus">Lists!$K$1:$K$10</definedName>
@@ -41,6 +42,8 @@
     <definedName name="IncomeStatus">Lists!$I$4:$I$5</definedName>
     <definedName name="InterviewResult">Lists!$M$1:$M$3</definedName>
     <definedName name="InterviewRound">Lists!$O$1:$O$5</definedName>
+    <definedName name="LiabilityType">Lists!$I$15:$I$25</definedName>
+    <definedName name="LoanCategory">Lists!$J$15:$J$25</definedName>
     <definedName name="LoanType">Lists!$A$18:$A$23</definedName>
     <definedName name="NeedWant">Lists!$C$1:$C$2</definedName>
     <definedName name="NextAction">Lists!$Q$1:$Q$7</definedName>
@@ -51,6 +54,7 @@
     <definedName name="v">Lists!#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -71,7 +75,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="271">
   <si>
     <t>August Financial Plan</t>
   </si>
@@ -833,6 +837,57 @@
   </si>
   <si>
     <t>Vehicle</t>
+  </si>
+  <si>
+    <t>Liability</t>
+  </si>
+  <si>
+    <t>Original Loan</t>
+  </si>
+  <si>
+    <t>Outstanding Balance</t>
+  </si>
+  <si>
+    <t>Monthly EMI</t>
+  </si>
+  <si>
+    <t>Intrest %</t>
+  </si>
+  <si>
+    <t>Consumer Loan</t>
+  </si>
+  <si>
+    <t>ICICI Credit Card</t>
+  </si>
+  <si>
+    <t>SBI Home Loan</t>
+  </si>
+  <si>
+    <t>Home Loan</t>
+  </si>
+  <si>
+    <t>Car Loan</t>
+  </si>
+  <si>
+    <t>Vehicle Loan</t>
+  </si>
+  <si>
+    <t>Education Loan</t>
+  </si>
+  <si>
+    <t>Business Loan</t>
+  </si>
+  <si>
+    <t>Personal Loan</t>
+  </si>
+  <si>
+    <t>Gold Loan</t>
+  </si>
+  <si>
+    <t>BNPL</t>
+  </si>
+  <si>
+    <t>Buy Now Pay Later</t>
   </si>
 </sst>
 </file>
@@ -995,7 +1050,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1043,6 +1098,7 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1051,7 +1107,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="32">
+  <dxfs count="38">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1071,6 +1127,9 @@
           <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1222,6 +1281,21 @@
     <dxf>
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
     </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1236,14 +1310,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{42D67FA3-A40A-4607-BCB9-468A9ECB0007}" name="Table1" displayName="Table1" ref="A1:H1048576" totalsRowShown="0" headerRowDxfId="30" tableBorderDxfId="29">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{42D67FA3-A40A-4607-BCB9-468A9ECB0007}" name="Table1" displayName="Table1" ref="A1:H1048576" totalsRowShown="0" headerRowDxfId="31" tableBorderDxfId="30">
   <autoFilter ref="A1:H1048576" xr:uid="{42D67FA3-A40A-4607-BCB9-468A9ECB0007}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{1D37F906-33D7-46E6-8270-56D5EEA80EC7}" name="Date" dataDxfId="28"/>
+    <tableColumn id="1" xr3:uid="{1D37F906-33D7-46E6-8270-56D5EEA80EC7}" name="Date" dataDxfId="29"/>
     <tableColumn id="4" xr3:uid="{E805A8A8-660D-4099-912A-BE1B697553ED}" name="Type"/>
     <tableColumn id="5" xr3:uid="{ABF1E4D7-7922-479D-94F4-994DCBA1062D}" name="Category"/>
     <tableColumn id="6" xr3:uid="{E21EA904-BC60-4EB5-B4BD-249E5A12FC76}" name="Description "/>
-    <tableColumn id="7" xr3:uid="{EFA172CE-B81A-4A83-BB09-0C52BED62422}" name="Amount" dataDxfId="27"/>
+    <tableColumn id="7" xr3:uid="{EFA172CE-B81A-4A83-BB09-0C52BED62422}" name="Amount" dataDxfId="28"/>
     <tableColumn id="8" xr3:uid="{E811D3EB-DAD5-46D9-B70D-01072B332F5C}" name="Need/Want"/>
     <tableColumn id="9" xr3:uid="{1E8766C9-2C6F-4CE3-9C7E-C6C8545D3945}" name="Payment Mode"/>
     <tableColumn id="10" xr3:uid="{BA26CD78-BAFB-4644-808D-0A18546F6CAF}" name="Recurring"/>
@@ -1256,7 +1330,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{204CD917-42D7-44E9-889E-B87F7E170616}" name="Table5" displayName="Table5" ref="A1:C100" totalsRowShown="0">
   <autoFilter ref="A1:C100" xr:uid="{204CD917-42D7-44E9-889E-B87F7E170616}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{CCD99EA9-9CA0-4F69-8282-1EE2E5FE7967}" name="Month" dataDxfId="26"/>
+    <tableColumn id="1" xr3:uid="{CCD99EA9-9CA0-4F69-8282-1EE2E5FE7967}" name="Month" dataDxfId="27"/>
     <tableColumn id="2" xr3:uid="{5C307EC1-8BAE-4B8C-AF42-D468202B7A5E}" name="Year"/>
     <tableColumn id="3" xr3:uid="{2B3569FD-9348-4E00-BFEA-53DF4F58E82C}" name="Monthly_Budget"/>
   </tableColumns>
@@ -1268,50 +1342,50 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{1AFBBFA5-5EA2-4DA5-91C7-5EE90985F084}" name="FinancialCommitments" displayName="FinancialCommitments" ref="A1:K46" totalsRowShown="0">
   <autoFilter ref="A1:K46" xr:uid="{1AFBBFA5-5EA2-4DA5-91C7-5EE90985F084}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{C10697DD-F282-4D7F-A12A-9BFC6193DC4E}" name="Start Date " dataDxfId="25"/>
+    <tableColumn id="1" xr3:uid="{C10697DD-F282-4D7F-A12A-9BFC6193DC4E}" name="Start Date " dataDxfId="26"/>
     <tableColumn id="2" xr3:uid="{D6130D6E-B2EE-4D09-94CD-7E8053CD1C7B}" name="From"/>
     <tableColumn id="3" xr3:uid="{8ECD20EB-BEF0-47D5-8DA5-28D491EC7B0A}" name="Type"/>
-    <tableColumn id="4" xr3:uid="{87D047F3-8B64-4D30-ACC0-42FFF26FEC3E}" name="Total Amount" dataDxfId="24"/>
-    <tableColumn id="5" xr3:uid="{C982624C-E448-4958-A5CE-7D794FC142FA}" name="Repaid" dataDxfId="23"/>
-    <tableColumn id="6" xr3:uid="{665D5056-3744-4E56-95C7-F0943FD35707}" name="Remaining" dataDxfId="22"/>
+    <tableColumn id="4" xr3:uid="{87D047F3-8B64-4D30-ACC0-42FFF26FEC3E}" name="Total Amount" dataDxfId="25"/>
+    <tableColumn id="5" xr3:uid="{C982624C-E448-4958-A5CE-7D794FC142FA}" name="Repaid" dataDxfId="24"/>
+    <tableColumn id="6" xr3:uid="{665D5056-3744-4E56-95C7-F0943FD35707}" name="Remaining" dataDxfId="23"/>
     <tableColumn id="7" xr3:uid="{FFDA91C5-2668-4023-9FEE-465A59D85270}" name="Due Date"/>
     <tableColumn id="8" xr3:uid="{748EB09B-78B0-49AB-AC7E-88A7F4C42C89}" name="Status"/>
     <tableColumn id="10" xr3:uid="{39DD9F5E-EB31-47B4-A27F-BDA3AA61DA00}" name="commitment"/>
-    <tableColumn id="11" xr3:uid="{740721D4-21BC-47E8-A178-052DE413178D}" name="Monthly Payment" dataDxfId="21"/>
-    <tableColumn id="12" xr3:uid="{2EEE087F-37EF-44B3-8405-6F6CCBE4BDEB}" name="End Date" dataDxfId="20"/>
+    <tableColumn id="11" xr3:uid="{740721D4-21BC-47E8-A178-052DE413178D}" name="Monthly Payment" dataDxfId="22"/>
+    <tableColumn id="12" xr3:uid="{2EEE087F-37EF-44B3-8405-6F6CCBE4BDEB}" name="End Date" dataDxfId="21"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{7C5D4057-F5F1-485E-AE6E-34A855BB81C8}" name="IncomeTable" displayName="IncomeTable" ref="A1:G4" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{7C5D4057-F5F1-485E-AE6E-34A855BB81C8}" name="IncomeTable" displayName="IncomeTable" ref="A1:G4" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
   <autoFilter ref="A1:G4" xr:uid="{7C5D4057-F5F1-485E-AE6E-34A855BB81C8}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{85417279-B333-4129-826F-4B13A464B0A1}" name="Date" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{72151722-7F6E-43AF-AADF-05A0452D151E}" name="Source" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{A9F1D760-964B-4BC4-876E-FE2B218C85B6}" name="Category" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{31C0BCAE-AC93-4345-9B1C-546CE0735A6B}" name="Amount" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{C6E99480-C881-404B-8F25-E2549BD2CCCD}" name="Status" dataDxfId="13"/>
-    <tableColumn id="7" xr3:uid="{29AC2CCC-8D50-4D4F-9049-D5CBB08CDAB6}" name="Recurring" dataDxfId="12"/>
-    <tableColumn id="6" xr3:uid="{4D5A0A55-4298-4332-9A93-683CDAE35676}" name="Notes" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{85417279-B333-4129-826F-4B13A464B0A1}" name="Date" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{72151722-7F6E-43AF-AADF-05A0452D151E}" name="Source" dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{A9F1D760-964B-4BC4-876E-FE2B218C85B6}" name="Category" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{31C0BCAE-AC93-4345-9B1C-546CE0735A6B}" name="Amount" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{C6E99480-C881-404B-8F25-E2549BD2CCCD}" name="Status" dataDxfId="14"/>
+    <tableColumn id="7" xr3:uid="{29AC2CCC-8D50-4D4F-9049-D5CBB08CDAB6}" name="Recurring" dataDxfId="13"/>
+    <tableColumn id="6" xr3:uid="{4D5A0A55-4298-4332-9A93-683CDAE35676}" name="Notes" dataDxfId="12"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{ED3F2086-7429-4708-9751-1D0D42E41B00}" name="Table6" displayName="Table6" ref="A1:H4" totalsRowShown="0" headerRowDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{ED3F2086-7429-4708-9751-1D0D42E41B00}" name="Table6" displayName="Table6" ref="A1:H4" totalsRowShown="0" headerRowDxfId="11">
   <autoFilter ref="A1:H4" xr:uid="{ED3F2086-7429-4708-9751-1D0D42E41B00}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{02A819B9-5B65-4731-BA10-C393EA3AE4AE}" name="Goal" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{51D61835-0ABB-4183-9CDE-6E008A5BE534}" name="Type" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{26F4B186-E946-48D7-9DD2-DA125EFEB650}" name="Target Amount" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{B407A7D5-A3D5-4F1F-A0BE-CEC184447D2F}" name="Current Amount" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{AC787662-7B98-4750-92E3-5F644C592A83}" name="Start Date" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{219A44EC-76A4-456E-8296-B0D5D5DB8C37}" name="Target Date" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{401F98C6-DE93-4917-B06B-A1F0D02774EE}" name="Priority" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{AFB6C60C-D1A2-49E4-B330-36821968B1DD}" name="Status" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{02A819B9-5B65-4731-BA10-C393EA3AE4AE}" name="Goal" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{51D61835-0ABB-4183-9CDE-6E008A5BE534}" name="Type" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{26F4B186-E946-48D7-9DD2-DA125EFEB650}" name="Target Amount" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{B407A7D5-A3D5-4F1F-A0BE-CEC184447D2F}" name="Current Amount" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{AC787662-7B98-4750-92E3-5F644C592A83}" name="Start Date" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{219A44EC-76A4-456E-8296-B0D5D5DB8C37}" name="Target Date" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{401F98C6-DE93-4917-B06B-A1F0D02774EE}" name="Priority" dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{AFB6C60C-D1A2-49E4-B330-36821968B1DD}" name="Status" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1337,6 +1411,24 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{4F7B6D94-D8D0-4A5C-BE0A-8099B43D186B}" name="Table10" displayName="Table10" ref="A1:I70" totalsRowShown="0">
+  <autoFilter ref="A1:I70" xr:uid="{4F7B6D94-D8D0-4A5C-BE0A-8099B43D186B}"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{1BF6EFB3-081D-479F-97D0-5D410AC21987}" name="Liability"/>
+    <tableColumn id="9" xr3:uid="{0B74D237-DA90-49D5-A8A6-285DE9F93208}" name="Category"/>
+    <tableColumn id="2" xr3:uid="{63AF3204-721F-4930-9003-E0E2451D091B}" name="Original Loan" dataDxfId="37"/>
+    <tableColumn id="3" xr3:uid="{271A520E-175A-4E77-8ACA-00A70E60B367}" name="Outstanding Balance" dataDxfId="36"/>
+    <tableColumn id="4" xr3:uid="{4AC64920-C6E6-4621-AC5A-DBB95F045FB6}" name="Monthly EMI" dataDxfId="35"/>
+    <tableColumn id="5" xr3:uid="{EA313BB7-3226-4263-8B2A-D21A5A3EC593}" name="Intrest %" dataDxfId="34"/>
+    <tableColumn id="6" xr3:uid="{E47C1A29-AD81-4EC2-9222-0D1F1C94F36D}" name="Start Date" dataDxfId="33"/>
+    <tableColumn id="7" xr3:uid="{5A74DAD1-ED79-464B-A2CB-CFDC6117FC4F}" name="End Date" dataDxfId="32"/>
+    <tableColumn id="8" xr3:uid="{6232A2AD-0FD7-4B56-A36F-A1E8D77D37A2}" name="Status"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{E6C8C911-DBF7-413D-A8D8-C9F208A9B6E1}" name="Table8" displayName="Table8" ref="A1:G200" totalsRowShown="0">
   <autoFilter ref="A1:G200" xr:uid="{E6C8C911-DBF7-413D-A8D8-C9F208A9B6E1}"/>
   <tableColumns count="7">
@@ -1344,7 +1436,7 @@
     <tableColumn id="2" xr3:uid="{AC7352C6-0DC7-4AFC-BDAD-303C389924A5}" name="Category"/>
     <tableColumn id="3" xr3:uid="{9884F549-FF9E-426C-A41E-5854163D6493}" name="Purchase Value"/>
     <tableColumn id="4" xr3:uid="{486852BE-C51C-4E3A-9B66-11D7D9CCEE9B}" name="Current Value"/>
-    <tableColumn id="5" xr3:uid="{2F141C2F-956F-436C-B98A-F15A4A0A762D}" name="Purchase Date" dataDxfId="31"/>
+    <tableColumn id="5" xr3:uid="{2F141C2F-956F-436C-B98A-F15A4A0A762D}" name="Purchase Date" dataDxfId="2"/>
     <tableColumn id="6" xr3:uid="{ED74E306-AFE5-436F-911F-2ED2CC19D23C}" name="Status"/>
     <tableColumn id="7" xr3:uid="{93FAD5D9-55A0-4F40-A483-B99C6367CC93}" name="Notes"/>
   </tableColumns>
@@ -1352,7 +1444,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2E0C23CD-1E80-4D43-9A03-38675147AE03}" name="Table2" displayName="Table2" ref="A1:J50" totalsRowShown="0">
   <autoFilter ref="A1:J50" xr:uid="{2E0C23CD-1E80-4D43-9A03-38675147AE03}"/>
   <tableColumns count="10">
@@ -1692,12 +1784,12 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -1946,6 +2038,94 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{176CEA01-1253-4E00-BFB7-DF8A0096DD60}">
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="2" width="9.6640625" customWidth="1"/>
+    <col min="3" max="3" width="13.6640625" style="21" customWidth="1"/>
+    <col min="4" max="4" width="20" style="21" customWidth="1"/>
+    <col min="5" max="5" width="16.109375" style="21" customWidth="1"/>
+    <col min="6" max="6" width="10.21875" style="33" customWidth="1"/>
+    <col min="7" max="7" width="11.21875" style="28" customWidth="1"/>
+    <col min="8" max="8" width="10.33203125" style="28" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>254</v>
+      </c>
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" s="21" t="s">
+        <v>255</v>
+      </c>
+      <c r="D1" s="21" t="s">
+        <v>256</v>
+      </c>
+      <c r="E1" s="21" t="s">
+        <v>257</v>
+      </c>
+      <c r="F1" s="33" t="s">
+        <v>258</v>
+      </c>
+      <c r="G1" s="28" t="s">
+        <v>234</v>
+      </c>
+      <c r="H1" s="28" t="s">
+        <v>228</v>
+      </c>
+      <c r="I1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>230</v>
+      </c>
+      <c r="B2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C2" s="21">
+        <v>86000</v>
+      </c>
+      <c r="D2" s="21">
+        <v>86000</v>
+      </c>
+      <c r="E2" s="21">
+        <v>8600</v>
+      </c>
+      <c r="F2" s="33">
+        <v>0</v>
+      </c>
+      <c r="G2" s="28">
+        <v>46235</v>
+      </c>
+      <c r="H2" s="28">
+        <v>46508</v>
+      </c>
+      <c r="I2" t="s">
+        <v>197</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B70" xr:uid="{444B1917-D7F7-4818-80C8-8F4A52ACFF72}">
+      <formula1>LoanCategory</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A70" xr:uid="{FFDD0255-25A1-4F8C-982E-98131995D194}">
+      <formula1>LiabilityType</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4BD347A-E68F-44B6-B63F-C92671AA0A69}">
   <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2048,7 +2228,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C985A9ED-FFB7-41B9-BD81-D99D84E9A097}">
   <dimension ref="A1:J35"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2302,7 +2482,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{062E0065-A33A-40A3-8681-B93160D6FE12}">
   <dimension ref="A1:Q5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2438,7 +2618,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52E36AC4-05BC-4C7B-BA73-388CE26BAB52}">
   <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2515,9 +2695,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{729B4158-2DD5-48A6-9BEC-2F739409F312}">
-  <dimension ref="A1:Q23"/>
+  <dimension ref="A1:Q25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.3">
@@ -2773,7 +2953,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>34</v>
       </c>
@@ -2783,43 +2963,115 @@
       <c r="E15" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="I15" s="18" t="s">
+        <v>230</v>
+      </c>
+      <c r="J15" s="18" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
       <c r="C16" t="s">
         <v>34</v>
       </c>
       <c r="E16" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="I16" s="18" t="s">
+        <v>260</v>
+      </c>
+      <c r="J16" s="18" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I17" s="18" t="s">
+        <v>261</v>
+      </c>
+      <c r="J17" s="18" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="I18" s="18" t="s">
+        <v>263</v>
+      </c>
+      <c r="J18" s="18" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="I19" s="18" t="s">
+        <v>265</v>
+      </c>
+      <c r="J19" s="18" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="I20" s="18" t="s">
+        <v>266</v>
+      </c>
+      <c r="J20" s="18" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="I21" s="18" t="s">
+        <v>267</v>
+      </c>
+      <c r="J21" s="18" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="I22" s="18" t="s">
+        <v>268</v>
+      </c>
+      <c r="J22" s="18" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>224</v>
+      </c>
+      <c r="I23" s="18" t="s">
+        <v>269</v>
+      </c>
+      <c r="J23" s="18" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="I24" s="18" t="s">
+        <v>196</v>
+      </c>
+      <c r="J24" s="18" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I25" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="J25" s="18" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
(v0.9.7): implement Net Worth Engine with wealth analysis
</commit_message>
<xml_diff>
--- a/data/finance.xlsx
+++ b/data/finance.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ED00688-9096-4D04-A468-E24B7648A096}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="855" firstSheet="5" activeTab="15" xr2:uid="{D6DE1A26-0963-4585-A363-547897EAF3B2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="855" firstSheet="5" activeTab="10" xr2:uid="{D6DE1A26-0963-4585-A363-547897EAF3B2}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,6 @@
     <definedName name="v">Lists!#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1132,6 +1131,24 @@
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1278,24 +1295,6 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1310,14 +1309,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{42D67FA3-A40A-4607-BCB9-468A9ECB0007}" name="Table1" displayName="Table1" ref="A1:H1048576" totalsRowShown="0" headerRowDxfId="31" tableBorderDxfId="30">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{42D67FA3-A40A-4607-BCB9-468A9ECB0007}" name="Table1" displayName="Table1" ref="A1:H1048576" totalsRowShown="0" headerRowDxfId="37" tableBorderDxfId="36">
   <autoFilter ref="A1:H1048576" xr:uid="{42D67FA3-A40A-4607-BCB9-468A9ECB0007}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{1D37F906-33D7-46E6-8270-56D5EEA80EC7}" name="Date" dataDxfId="29"/>
+    <tableColumn id="1" xr3:uid="{1D37F906-33D7-46E6-8270-56D5EEA80EC7}" name="Date" dataDxfId="35"/>
     <tableColumn id="4" xr3:uid="{E805A8A8-660D-4099-912A-BE1B697553ED}" name="Type"/>
     <tableColumn id="5" xr3:uid="{ABF1E4D7-7922-479D-94F4-994DCBA1062D}" name="Category"/>
     <tableColumn id="6" xr3:uid="{E21EA904-BC60-4EB5-B4BD-249E5A12FC76}" name="Description "/>
-    <tableColumn id="7" xr3:uid="{EFA172CE-B81A-4A83-BB09-0C52BED62422}" name="Amount" dataDxfId="28"/>
+    <tableColumn id="7" xr3:uid="{EFA172CE-B81A-4A83-BB09-0C52BED62422}" name="Amount" dataDxfId="34"/>
     <tableColumn id="8" xr3:uid="{E811D3EB-DAD5-46D9-B70D-01072B332F5C}" name="Need/Want"/>
     <tableColumn id="9" xr3:uid="{1E8766C9-2C6F-4CE3-9C7E-C6C8545D3945}" name="Payment Mode"/>
     <tableColumn id="10" xr3:uid="{BA26CD78-BAFB-4644-808D-0A18546F6CAF}" name="Recurring"/>
@@ -1330,7 +1329,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{204CD917-42D7-44E9-889E-B87F7E170616}" name="Table5" displayName="Table5" ref="A1:C100" totalsRowShown="0">
   <autoFilter ref="A1:C100" xr:uid="{204CD917-42D7-44E9-889E-B87F7E170616}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{CCD99EA9-9CA0-4F69-8282-1EE2E5FE7967}" name="Month" dataDxfId="27"/>
+    <tableColumn id="1" xr3:uid="{CCD99EA9-9CA0-4F69-8282-1EE2E5FE7967}" name="Month" dataDxfId="33"/>
     <tableColumn id="2" xr3:uid="{5C307EC1-8BAE-4B8C-AF42-D468202B7A5E}" name="Year"/>
     <tableColumn id="3" xr3:uid="{2B3569FD-9348-4E00-BFEA-53DF4F58E82C}" name="Monthly_Budget"/>
   </tableColumns>
@@ -1342,50 +1341,50 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{1AFBBFA5-5EA2-4DA5-91C7-5EE90985F084}" name="FinancialCommitments" displayName="FinancialCommitments" ref="A1:K46" totalsRowShown="0">
   <autoFilter ref="A1:K46" xr:uid="{1AFBBFA5-5EA2-4DA5-91C7-5EE90985F084}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{C10697DD-F282-4D7F-A12A-9BFC6193DC4E}" name="Start Date " dataDxfId="26"/>
+    <tableColumn id="1" xr3:uid="{C10697DD-F282-4D7F-A12A-9BFC6193DC4E}" name="Start Date " dataDxfId="32"/>
     <tableColumn id="2" xr3:uid="{D6130D6E-B2EE-4D09-94CD-7E8053CD1C7B}" name="From"/>
     <tableColumn id="3" xr3:uid="{8ECD20EB-BEF0-47D5-8DA5-28D491EC7B0A}" name="Type"/>
-    <tableColumn id="4" xr3:uid="{87D047F3-8B64-4D30-ACC0-42FFF26FEC3E}" name="Total Amount" dataDxfId="25"/>
-    <tableColumn id="5" xr3:uid="{C982624C-E448-4958-A5CE-7D794FC142FA}" name="Repaid" dataDxfId="24"/>
-    <tableColumn id="6" xr3:uid="{665D5056-3744-4E56-95C7-F0943FD35707}" name="Remaining" dataDxfId="23"/>
+    <tableColumn id="4" xr3:uid="{87D047F3-8B64-4D30-ACC0-42FFF26FEC3E}" name="Total Amount" dataDxfId="31"/>
+    <tableColumn id="5" xr3:uid="{C982624C-E448-4958-A5CE-7D794FC142FA}" name="Repaid" dataDxfId="30"/>
+    <tableColumn id="6" xr3:uid="{665D5056-3744-4E56-95C7-F0943FD35707}" name="Remaining" dataDxfId="29"/>
     <tableColumn id="7" xr3:uid="{FFDA91C5-2668-4023-9FEE-465A59D85270}" name="Due Date"/>
     <tableColumn id="8" xr3:uid="{748EB09B-78B0-49AB-AC7E-88A7F4C42C89}" name="Status"/>
     <tableColumn id="10" xr3:uid="{39DD9F5E-EB31-47B4-A27F-BDA3AA61DA00}" name="commitment"/>
-    <tableColumn id="11" xr3:uid="{740721D4-21BC-47E8-A178-052DE413178D}" name="Monthly Payment" dataDxfId="22"/>
-    <tableColumn id="12" xr3:uid="{2EEE087F-37EF-44B3-8405-6F6CCBE4BDEB}" name="End Date" dataDxfId="21"/>
+    <tableColumn id="11" xr3:uid="{740721D4-21BC-47E8-A178-052DE413178D}" name="Monthly Payment" dataDxfId="28"/>
+    <tableColumn id="12" xr3:uid="{2EEE087F-37EF-44B3-8405-6F6CCBE4BDEB}" name="End Date" dataDxfId="27"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{7C5D4057-F5F1-485E-AE6E-34A855BB81C8}" name="IncomeTable" displayName="IncomeTable" ref="A1:G4" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{7C5D4057-F5F1-485E-AE6E-34A855BB81C8}" name="IncomeTable" displayName="IncomeTable" ref="A1:G4" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25">
   <autoFilter ref="A1:G4" xr:uid="{7C5D4057-F5F1-485E-AE6E-34A855BB81C8}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{85417279-B333-4129-826F-4B13A464B0A1}" name="Date" dataDxfId="18"/>
-    <tableColumn id="2" xr3:uid="{72151722-7F6E-43AF-AADF-05A0452D151E}" name="Source" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{A9F1D760-964B-4BC4-876E-FE2B218C85B6}" name="Category" dataDxfId="16"/>
-    <tableColumn id="4" xr3:uid="{31C0BCAE-AC93-4345-9B1C-546CE0735A6B}" name="Amount" dataDxfId="15"/>
-    <tableColumn id="5" xr3:uid="{C6E99480-C881-404B-8F25-E2549BD2CCCD}" name="Status" dataDxfId="14"/>
-    <tableColumn id="7" xr3:uid="{29AC2CCC-8D50-4D4F-9049-D5CBB08CDAB6}" name="Recurring" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{4D5A0A55-4298-4332-9A93-683CDAE35676}" name="Notes" dataDxfId="12"/>
+    <tableColumn id="1" xr3:uid="{85417279-B333-4129-826F-4B13A464B0A1}" name="Date" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{72151722-7F6E-43AF-AADF-05A0452D151E}" name="Source" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{A9F1D760-964B-4BC4-876E-FE2B218C85B6}" name="Category" dataDxfId="22"/>
+    <tableColumn id="4" xr3:uid="{31C0BCAE-AC93-4345-9B1C-546CE0735A6B}" name="Amount" dataDxfId="21"/>
+    <tableColumn id="5" xr3:uid="{C6E99480-C881-404B-8F25-E2549BD2CCCD}" name="Status" dataDxfId="20"/>
+    <tableColumn id="7" xr3:uid="{29AC2CCC-8D50-4D4F-9049-D5CBB08CDAB6}" name="Recurring" dataDxfId="19"/>
+    <tableColumn id="6" xr3:uid="{4D5A0A55-4298-4332-9A93-683CDAE35676}" name="Notes" dataDxfId="18"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{ED3F2086-7429-4708-9751-1D0D42E41B00}" name="Table6" displayName="Table6" ref="A1:H4" totalsRowShown="0" headerRowDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{ED3F2086-7429-4708-9751-1D0D42E41B00}" name="Table6" displayName="Table6" ref="A1:H4" totalsRowShown="0" headerRowDxfId="17">
   <autoFilter ref="A1:H4" xr:uid="{ED3F2086-7429-4708-9751-1D0D42E41B00}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{02A819B9-5B65-4731-BA10-C393EA3AE4AE}" name="Goal" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{51D61835-0ABB-4183-9CDE-6E008A5BE534}" name="Type" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{26F4B186-E946-48D7-9DD2-DA125EFEB650}" name="Target Amount" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{B407A7D5-A3D5-4F1F-A0BE-CEC184447D2F}" name="Current Amount" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{AC787662-7B98-4750-92E3-5F644C592A83}" name="Start Date" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{219A44EC-76A4-456E-8296-B0D5D5DB8C37}" name="Target Date" dataDxfId="5"/>
-    <tableColumn id="7" xr3:uid="{401F98C6-DE93-4917-B06B-A1F0D02774EE}" name="Priority" dataDxfId="4"/>
-    <tableColumn id="8" xr3:uid="{AFB6C60C-D1A2-49E4-B330-36821968B1DD}" name="Status" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{02A819B9-5B65-4731-BA10-C393EA3AE4AE}" name="Goal" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{51D61835-0ABB-4183-9CDE-6E008A5BE534}" name="Type" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{26F4B186-E946-48D7-9DD2-DA125EFEB650}" name="Target Amount" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{B407A7D5-A3D5-4F1F-A0BE-CEC184447D2F}" name="Current Amount" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{AC787662-7B98-4750-92E3-5F644C592A83}" name="Start Date" dataDxfId="12"/>
+    <tableColumn id="6" xr3:uid="{219A44EC-76A4-456E-8296-B0D5D5DB8C37}" name="Target Date" dataDxfId="11"/>
+    <tableColumn id="7" xr3:uid="{401F98C6-DE93-4917-B06B-A1F0D02774EE}" name="Priority" dataDxfId="10"/>
+    <tableColumn id="8" xr3:uid="{AFB6C60C-D1A2-49E4-B330-36821968B1DD}" name="Status" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1416,12 +1415,12 @@
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{1BF6EFB3-081D-479F-97D0-5D410AC21987}" name="Liability"/>
     <tableColumn id="9" xr3:uid="{0B74D237-DA90-49D5-A8A6-285DE9F93208}" name="Category"/>
-    <tableColumn id="2" xr3:uid="{63AF3204-721F-4930-9003-E0E2451D091B}" name="Original Loan" dataDxfId="37"/>
-    <tableColumn id="3" xr3:uid="{271A520E-175A-4E77-8ACA-00A70E60B367}" name="Outstanding Balance" dataDxfId="36"/>
-    <tableColumn id="4" xr3:uid="{4AC64920-C6E6-4621-AC5A-DBB95F045FB6}" name="Monthly EMI" dataDxfId="35"/>
-    <tableColumn id="5" xr3:uid="{EA313BB7-3226-4263-8B2A-D21A5A3EC593}" name="Intrest %" dataDxfId="34"/>
-    <tableColumn id="6" xr3:uid="{E47C1A29-AD81-4EC2-9222-0D1F1C94F36D}" name="Start Date" dataDxfId="33"/>
-    <tableColumn id="7" xr3:uid="{5A74DAD1-ED79-464B-A2CB-CFDC6117FC4F}" name="End Date" dataDxfId="32"/>
+    <tableColumn id="2" xr3:uid="{63AF3204-721F-4930-9003-E0E2451D091B}" name="Original Loan" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{271A520E-175A-4E77-8ACA-00A70E60B367}" name="Outstanding Balance" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{4AC64920-C6E6-4621-AC5A-DBB95F045FB6}" name="Monthly EMI" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{EA313BB7-3226-4263-8B2A-D21A5A3EC593}" name="Intrest %" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{E47C1A29-AD81-4EC2-9222-0D1F1C94F36D}" name="Start Date" dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{5A74DAD1-ED79-464B-A2CB-CFDC6117FC4F}" name="End Date" dataDxfId="3"/>
     <tableColumn id="8" xr3:uid="{6232A2AD-0FD7-4B56-A36F-A1E8D77D37A2}" name="Status"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>

</xml_diff>